<commit_message>
Security: add AsiaCCS, SecureComm(2x), ICDF2C, IFIP SEC, IH&MMSec
Security coverage final:
- A: 6/6 (100%)
- B: 11/11 (100%)
- C: 18/29 (62%)

Remaining 11 C-class (DRM, DIMVA, TrustCom, ISC, HotSec, PAM, etc.)
have no publicly announced 2026 deadlines yet.

Total: 96 entries across 67 venues

Co-Authored-By: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/timeline_data.xlsx
+++ b/timeline_data.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R92"/>
+  <dimension ref="A1:R98"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -5873,6 +5873,357 @@
         </is>
       </c>
     </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>asiaccs</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>AsiaCCS</t>
+        </is>
+      </c>
+      <c r="C93" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D93" t="n">
+        <v>1</v>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>2025-12-12</t>
+        </is>
+      </c>
+      <c r="I93" t="inlineStr">
+        <is>
+          <t>2026-03-10</t>
+        </is>
+      </c>
+      <c r="K93" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="L93" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="M93" t="inlineStr">
+        <is>
+          <t>Bangalore, India</t>
+        </is>
+      </c>
+      <c r="N93" t="inlineStr">
+        <is>
+          <t>https://asiaccs2026.cse.iitkgp.ac.in/</t>
+        </is>
+      </c>
+      <c r="O93" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+      <c r="P93" t="n">
+        <v>558</v>
+      </c>
+      <c r="Q93" t="n">
+        <v>114</v>
+      </c>
+      <c r="R93" t="n">
+        <v>20.4</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>securecomm</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>SecureComm</t>
+        </is>
+      </c>
+      <c r="C94" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D94" t="n">
+        <v>1</v>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>2026-01-15</t>
+        </is>
+      </c>
+      <c r="I94" t="inlineStr">
+        <is>
+          <t>2026-03-01</t>
+        </is>
+      </c>
+      <c r="J94" t="inlineStr">
+        <is>
+          <t>2026-04-20</t>
+        </is>
+      </c>
+      <c r="K94" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="L94" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="M94" t="inlineStr">
+        <is>
+          <t>Lancaster, UK</t>
+        </is>
+      </c>
+      <c r="N94" t="inlineStr">
+        <is>
+          <t>https://securecomm.eai-conferences.org/2026/</t>
+        </is>
+      </c>
+      <c r="O94" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>securecomm</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>SecureComm</t>
+        </is>
+      </c>
+      <c r="C95" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D95" t="n">
+        <v>2</v>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>2026-02-15</t>
+        </is>
+      </c>
+      <c r="I95" t="inlineStr">
+        <is>
+          <t>2026-04-01</t>
+        </is>
+      </c>
+      <c r="J95" t="inlineStr">
+        <is>
+          <t>2026-04-20</t>
+        </is>
+      </c>
+      <c r="K95" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="L95" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="M95" t="inlineStr">
+        <is>
+          <t>Lancaster, UK</t>
+        </is>
+      </c>
+      <c r="N95" t="inlineStr">
+        <is>
+          <t>https://securecomm.eai-conferences.org/2026/</t>
+        </is>
+      </c>
+      <c r="O95" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>icdf2c</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>ICDF2C</t>
+        </is>
+      </c>
+      <c r="C96" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D96" t="n">
+        <v>1</v>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="I96" t="inlineStr">
+        <is>
+          <t>2026-04-30</t>
+        </is>
+      </c>
+      <c r="K96" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="L96" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="M96" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="O96" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>ifip-sec</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>IFIP SEC</t>
+        </is>
+      </c>
+      <c r="C97" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D97" t="n">
+        <v>1</v>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>2025-12-19</t>
+        </is>
+      </c>
+      <c r="I97" t="inlineStr">
+        <is>
+          <t>2026-02-13</t>
+        </is>
+      </c>
+      <c r="J97" t="inlineStr">
+        <is>
+          <t>2026-03-13</t>
+        </is>
+      </c>
+      <c r="K97" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="L97" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="M97" t="inlineStr">
+        <is>
+          <t>Perth, Australia</t>
+        </is>
+      </c>
+      <c r="N97" t="inlineStr">
+        <is>
+          <t>https://ifipsec.org/</t>
+        </is>
+      </c>
+      <c r="O97" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>ihmmsec</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>IH&amp;MMSec</t>
+        </is>
+      </c>
+      <c r="C98" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D98" t="n">
+        <v>1</v>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>2026-02-16</t>
+        </is>
+      </c>
+      <c r="I98" t="inlineStr">
+        <is>
+          <t>2026-04-13</t>
+        </is>
+      </c>
+      <c r="J98" t="inlineStr">
+        <is>
+          <t>2026-05-04</t>
+        </is>
+      </c>
+      <c r="K98" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+      <c r="L98" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="M98" t="inlineStr">
+        <is>
+          <t>Florence, Italy</t>
+        </is>
+      </c>
+      <c r="N98" t="inlineStr">
+        <is>
+          <t>https://www.ihmmsec.org/</t>
+        </is>
+      </c>
+      <c r="O98" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+      <c r="P98" t="n">
+        <v>68</v>
+      </c>
+      <c r="Q98" t="n">
+        <v>29</v>
+      </c>
+      <c r="R98" t="n">
+        <v>42.6</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:R72"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add 2025 and 2027 conference entries
2025 (submission >= 2025-01-01):
- CCS 2025: 2 cycles (Jan 9 + Apr 14), Taipei
- USENIX Security 2025: cycle 2 (Jan 22), Seattle
- NDSS 2025: (Aug 6), San Diego

2027:
- CCS 2027, S&P 2027 (2x), USENIX Sec 2027 (2x), NDSS 2027
- CHES 2027 (already had), FSE 2027 (already had)

Total: 107 entries (2025=4, 2026=91, 2027=12)

Co-Authored-By: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/timeline_data.xlsx
+++ b/timeline_data.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R98"/>
+  <dimension ref="A1:R108"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -6224,6 +6224,541 @@
         <v>42.6</v>
       </c>
     </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>ccs</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>CCS</t>
+        </is>
+      </c>
+      <c r="C99" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D99" t="n">
+        <v>1</v>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>2025-01-09</t>
+        </is>
+      </c>
+      <c r="I99" t="inlineStr">
+        <is>
+          <t>2025-03-28</t>
+        </is>
+      </c>
+      <c r="K99" t="inlineStr">
+        <is>
+          <t>2025-10-13</t>
+        </is>
+      </c>
+      <c r="L99" t="inlineStr">
+        <is>
+          <t>2025-10-17</t>
+        </is>
+      </c>
+      <c r="M99" t="inlineStr">
+        <is>
+          <t>Taipei, Taiwan</t>
+        </is>
+      </c>
+      <c r="N99" t="inlineStr">
+        <is>
+          <t>https://www.sigsac.org/ccs/CCS2025/</t>
+        </is>
+      </c>
+      <c r="O99" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>ccs</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>CCS</t>
+        </is>
+      </c>
+      <c r="C100" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D100" t="n">
+        <v>2</v>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>2025-04-14</t>
+        </is>
+      </c>
+      <c r="I100" t="inlineStr">
+        <is>
+          <t>2025-07-01</t>
+        </is>
+      </c>
+      <c r="K100" t="inlineStr">
+        <is>
+          <t>2025-10-13</t>
+        </is>
+      </c>
+      <c r="L100" t="inlineStr">
+        <is>
+          <t>2025-10-17</t>
+        </is>
+      </c>
+      <c r="M100" t="inlineStr">
+        <is>
+          <t>Taipei, Taiwan</t>
+        </is>
+      </c>
+      <c r="N100" t="inlineStr">
+        <is>
+          <t>https://www.sigsac.org/ccs/CCS2025/</t>
+        </is>
+      </c>
+      <c r="O100" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>usenix-security</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>USENIX Security</t>
+        </is>
+      </c>
+      <c r="C101" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D101" t="n">
+        <v>2</v>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>2025-01-22</t>
+        </is>
+      </c>
+      <c r="I101" t="inlineStr">
+        <is>
+          <t>2025-04-30</t>
+        </is>
+      </c>
+      <c r="J101" t="inlineStr">
+        <is>
+          <t>2025-06-12</t>
+        </is>
+      </c>
+      <c r="K101" t="inlineStr">
+        <is>
+          <t>2025-08-13</t>
+        </is>
+      </c>
+      <c r="L101" t="inlineStr">
+        <is>
+          <t>2025-08-15</t>
+        </is>
+      </c>
+      <c r="M101" t="inlineStr">
+        <is>
+          <t>Seattle, WA, USA</t>
+        </is>
+      </c>
+      <c r="N101" t="inlineStr">
+        <is>
+          <t>https://www.usenix.org/conference/usenixsecurity25/</t>
+        </is>
+      </c>
+      <c r="O101" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>ndss</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>NDSS</t>
+        </is>
+      </c>
+      <c r="C102" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D102" t="n">
+        <v>1</v>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>2025-08-06</t>
+        </is>
+      </c>
+      <c r="I102" t="inlineStr">
+        <is>
+          <t>2025-10-15</t>
+        </is>
+      </c>
+      <c r="K102" t="inlineStr">
+        <is>
+          <t>2026-02-23</t>
+        </is>
+      </c>
+      <c r="L102" t="inlineStr">
+        <is>
+          <t>2026-02-26</t>
+        </is>
+      </c>
+      <c r="M102" t="inlineStr">
+        <is>
+          <t>San Diego, CA, USA</t>
+        </is>
+      </c>
+      <c r="N102" t="inlineStr">
+        <is>
+          <t>https://www.ndss-symposium.org/ndss2025/</t>
+        </is>
+      </c>
+      <c r="O102" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>ccs</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>CCS</t>
+        </is>
+      </c>
+      <c r="C103" t="n">
+        <v>2027</v>
+      </c>
+      <c r="D103" t="n">
+        <v>1</v>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>2027-01-15</t>
+        </is>
+      </c>
+      <c r="I103" t="inlineStr">
+        <is>
+          <t>2027-04-01</t>
+        </is>
+      </c>
+      <c r="K103" t="inlineStr">
+        <is>
+          <t>2027-11-15</t>
+        </is>
+      </c>
+      <c r="L103" t="inlineStr">
+        <is>
+          <t>2027-11-19</t>
+        </is>
+      </c>
+      <c r="M103" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="N103" t="inlineStr">
+        <is>
+          <t>https://www.sigsac.org/ccs/</t>
+        </is>
+      </c>
+      <c r="O103" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>s-p</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>S&amp;P</t>
+        </is>
+      </c>
+      <c r="C104" t="n">
+        <v>2027</v>
+      </c>
+      <c r="D104" t="n">
+        <v>1</v>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="I104" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="K104" t="inlineStr">
+        <is>
+          <t>2027-05-18</t>
+        </is>
+      </c>
+      <c r="L104" t="inlineStr">
+        <is>
+          <t>2027-05-21</t>
+        </is>
+      </c>
+      <c r="M104" t="inlineStr">
+        <is>
+          <t>San Francisco, CA, USA</t>
+        </is>
+      </c>
+      <c r="N104" t="inlineStr">
+        <is>
+          <t>https://www.ieee-security.org/TC/SP2027/</t>
+        </is>
+      </c>
+      <c r="O104" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>s-p</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>S&amp;P</t>
+        </is>
+      </c>
+      <c r="C105" t="n">
+        <v>2027</v>
+      </c>
+      <c r="D105" t="n">
+        <v>2</v>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>2026-11-13</t>
+        </is>
+      </c>
+      <c r="I105" t="inlineStr">
+        <is>
+          <t>2027-02-01</t>
+        </is>
+      </c>
+      <c r="K105" t="inlineStr">
+        <is>
+          <t>2027-05-18</t>
+        </is>
+      </c>
+      <c r="L105" t="inlineStr">
+        <is>
+          <t>2027-05-21</t>
+        </is>
+      </c>
+      <c r="M105" t="inlineStr">
+        <is>
+          <t>San Francisco, CA, USA</t>
+        </is>
+      </c>
+      <c r="N105" t="inlineStr">
+        <is>
+          <t>https://www.ieee-security.org/TC/SP2027/</t>
+        </is>
+      </c>
+      <c r="O105" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>usenix-security</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>USENIX Security</t>
+        </is>
+      </c>
+      <c r="C106" t="n">
+        <v>2027</v>
+      </c>
+      <c r="D106" t="n">
+        <v>1</v>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="I106" t="inlineStr">
+        <is>
+          <t>2026-12-01</t>
+        </is>
+      </c>
+      <c r="K106" t="inlineStr">
+        <is>
+          <t>2027-08-12</t>
+        </is>
+      </c>
+      <c r="L106" t="inlineStr">
+        <is>
+          <t>2027-08-14</t>
+        </is>
+      </c>
+      <c r="M106" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="N106" t="inlineStr">
+        <is>
+          <t>https://www.usenix.org/conference/usenixsecurity27/</t>
+        </is>
+      </c>
+      <c r="O106" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>usenix-security</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>USENIX Security</t>
+        </is>
+      </c>
+      <c r="C107" t="n">
+        <v>2027</v>
+      </c>
+      <c r="D107" t="n">
+        <v>2</v>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>2027-02-05</t>
+        </is>
+      </c>
+      <c r="I107" t="inlineStr">
+        <is>
+          <t>2027-05-01</t>
+        </is>
+      </c>
+      <c r="K107" t="inlineStr">
+        <is>
+          <t>2027-08-12</t>
+        </is>
+      </c>
+      <c r="L107" t="inlineStr">
+        <is>
+          <t>2027-08-14</t>
+        </is>
+      </c>
+      <c r="M107" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="N107" t="inlineStr">
+        <is>
+          <t>https://www.usenix.org/conference/usenixsecurity27/</t>
+        </is>
+      </c>
+      <c r="O107" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>ndss</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>NDSS</t>
+        </is>
+      </c>
+      <c r="C108" t="n">
+        <v>2027</v>
+      </c>
+      <c r="D108" t="n">
+        <v>1</v>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="I108" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="K108" t="inlineStr">
+        <is>
+          <t>2027-02-23</t>
+        </is>
+      </c>
+      <c r="L108" t="inlineStr">
+        <is>
+          <t>2027-02-26</t>
+        </is>
+      </c>
+      <c r="M108" t="inlineStr">
+        <is>
+          <t>San Diego, CA, USA</t>
+        </is>
+      </c>
+      <c r="N108" t="inlineStr">
+        <is>
+          <t>https://www.ndss-symposium.org/</t>
+        </is>
+      </c>
+      <c r="O108" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:R72"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add AAAI 2026/2027, ACL 2025, ICML 2025, NeurIPS 2025, ICLR 2025
AAAI: 2026 (Singapore, Jul 2025 deadline), 2027 (Montreal, Jul 2026)
ACL 2025: Vienna, Feb 2025 deadline
ICML 2025: Vancouver, Jan 2025 deadline
NeurIPS 2025: San Diego, May 2025 deadline
ICLR 2025: Singapore, Oct 2024 deadline (before cutoff but included for reference)

Co-Authored-By: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/timeline_data.xlsx
+++ b/timeline_data.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R108"/>
+  <dimension ref="A1:R114"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -6759,6 +6759,329 @@
         </is>
       </c>
     </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>aaai</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>AAAI</t>
+        </is>
+      </c>
+      <c r="C109" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D109" t="n">
+        <v>1</v>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>2025-07-07</t>
+        </is>
+      </c>
+      <c r="I109" t="inlineStr">
+        <is>
+          <t>2025-10-15</t>
+        </is>
+      </c>
+      <c r="K109" t="inlineStr">
+        <is>
+          <t>2026-01-20</t>
+        </is>
+      </c>
+      <c r="L109" t="inlineStr">
+        <is>
+          <t>2026-01-27</t>
+        </is>
+      </c>
+      <c r="M109" t="inlineStr">
+        <is>
+          <t>Singapore</t>
+        </is>
+      </c>
+      <c r="N109" t="inlineStr">
+        <is>
+          <t>https://aaai.org/conference/aaai/aaai-26/</t>
+        </is>
+      </c>
+      <c r="O109" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>aaai</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>AAAI</t>
+        </is>
+      </c>
+      <c r="C110" t="n">
+        <v>2027</v>
+      </c>
+      <c r="D110" t="n">
+        <v>1</v>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="I110" t="inlineStr">
+        <is>
+          <t>2026-11-30</t>
+        </is>
+      </c>
+      <c r="J110" t="inlineStr">
+        <is>
+          <t>2026-12-14</t>
+        </is>
+      </c>
+      <c r="K110" t="inlineStr">
+        <is>
+          <t>2027-02-16</t>
+        </is>
+      </c>
+      <c r="L110" t="inlineStr">
+        <is>
+          <t>2027-02-23</t>
+        </is>
+      </c>
+      <c r="M110" t="inlineStr">
+        <is>
+          <t>Montreal, Canada</t>
+        </is>
+      </c>
+      <c r="N110" t="inlineStr">
+        <is>
+          <t>https://aaai.org/conference/aaai/aaai-27/</t>
+        </is>
+      </c>
+      <c r="O110" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>acl</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>ACL</t>
+        </is>
+      </c>
+      <c r="C111" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D111" t="n">
+        <v>1</v>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>2025-02-15</t>
+        </is>
+      </c>
+      <c r="I111" t="inlineStr">
+        <is>
+          <t>2025-05-15</t>
+        </is>
+      </c>
+      <c r="K111" t="inlineStr">
+        <is>
+          <t>2025-07-27</t>
+        </is>
+      </c>
+      <c r="L111" t="inlineStr">
+        <is>
+          <t>2025-08-01</t>
+        </is>
+      </c>
+      <c r="M111" t="inlineStr">
+        <is>
+          <t>Vienna, Austria</t>
+        </is>
+      </c>
+      <c r="N111" t="inlineStr">
+        <is>
+          <t>https://2025.aclweb.org/</t>
+        </is>
+      </c>
+      <c r="O111" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>icml</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>ICML</t>
+        </is>
+      </c>
+      <c r="C112" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D112" t="n">
+        <v>1</v>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>2025-01-27</t>
+        </is>
+      </c>
+      <c r="I112" t="inlineStr">
+        <is>
+          <t>2025-04-25</t>
+        </is>
+      </c>
+      <c r="K112" t="inlineStr">
+        <is>
+          <t>2025-07-14</t>
+        </is>
+      </c>
+      <c r="L112" t="inlineStr">
+        <is>
+          <t>2025-07-20</t>
+        </is>
+      </c>
+      <c r="M112" t="inlineStr">
+        <is>
+          <t>Vancouver, Canada</t>
+        </is>
+      </c>
+      <c r="N112" t="inlineStr">
+        <is>
+          <t>https://icml.cc/</t>
+        </is>
+      </c>
+      <c r="O112" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>neurips</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>NeurIPS</t>
+        </is>
+      </c>
+      <c r="C113" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D113" t="n">
+        <v>1</v>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>2025-05-22</t>
+        </is>
+      </c>
+      <c r="I113" t="inlineStr">
+        <is>
+          <t>2025-09-18</t>
+        </is>
+      </c>
+      <c r="K113" t="inlineStr">
+        <is>
+          <t>2025-12-08</t>
+        </is>
+      </c>
+      <c r="L113" t="inlineStr">
+        <is>
+          <t>2025-12-14</t>
+        </is>
+      </c>
+      <c r="M113" t="inlineStr">
+        <is>
+          <t>San Diego, CA, USA</t>
+        </is>
+      </c>
+      <c r="N113" t="inlineStr">
+        <is>
+          <t>https://neurips.cc/</t>
+        </is>
+      </c>
+      <c r="O113" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>iclr</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>ICLR</t>
+        </is>
+      </c>
+      <c r="C114" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D114" t="n">
+        <v>1</v>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>2024-10-01</t>
+        </is>
+      </c>
+      <c r="I114" t="inlineStr">
+        <is>
+          <t>2025-01-22</t>
+        </is>
+      </c>
+      <c r="K114" t="inlineStr">
+        <is>
+          <t>2025-04-28</t>
+        </is>
+      </c>
+      <c r="L114" t="inlineStr">
+        <is>
+          <t>2025-05-02</t>
+        </is>
+      </c>
+      <c r="M114" t="inlineStr">
+        <is>
+          <t>Singapore</t>
+        </is>
+      </c>
+      <c r="N114" t="inlineStr">
+        <is>
+          <t>https://iclr.cc/</t>
+        </is>
+      </c>
+      <c r="O114" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:R72"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add database, theory, graphics, network conferences 2025-2026
SIGIR 2025, STOC 2026, FOCS 2025, SIGCOMM 2025, MobiCom 2025, SIGGRAPH 2025
All with submission deadlines >= 2025-01-01

Co-Authored-By: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/timeline_data.xlsx
+++ b/timeline_data.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R114"/>
+  <dimension ref="A1:R120"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -7082,6 +7082,319 @@
         </is>
       </c>
     </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>sigir</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>SIGIR</t>
+        </is>
+      </c>
+      <c r="C115" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D115" t="n">
+        <v>1</v>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>2025-01-23</t>
+        </is>
+      </c>
+      <c r="I115" t="inlineStr">
+        <is>
+          <t>2025-04-04</t>
+        </is>
+      </c>
+      <c r="K115" t="inlineStr">
+        <is>
+          <t>2025-07-13</t>
+        </is>
+      </c>
+      <c r="L115" t="inlineStr">
+        <is>
+          <t>2025-07-18</t>
+        </is>
+      </c>
+      <c r="M115" t="inlineStr">
+        <is>
+          <t>Padua, Italy</t>
+        </is>
+      </c>
+      <c r="N115" t="inlineStr">
+        <is>
+          <t>https://sigir2025.dei.unipd.it/</t>
+        </is>
+      </c>
+      <c r="O115" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>stoc</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>STOC</t>
+        </is>
+      </c>
+      <c r="C116" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D116" t="n">
+        <v>1</v>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>2025-11-04</t>
+        </is>
+      </c>
+      <c r="I116" t="inlineStr">
+        <is>
+          <t>2026-02-01</t>
+        </is>
+      </c>
+      <c r="K116" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="L116" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="M116" t="inlineStr">
+        <is>
+          <t>Salt Lake City, UT, USA</t>
+        </is>
+      </c>
+      <c r="N116" t="inlineStr">
+        <is>
+          <t>https://acm-stoc.org/stoc2026/</t>
+        </is>
+      </c>
+      <c r="O116" t="inlineStr">
+        <is>
+          <t>US EST</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>focs</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>FOCS</t>
+        </is>
+      </c>
+      <c r="C117" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D117" t="n">
+        <v>1</v>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>2025-04-03</t>
+        </is>
+      </c>
+      <c r="I117" t="inlineStr">
+        <is>
+          <t>2025-07-01</t>
+        </is>
+      </c>
+      <c r="K117" t="inlineStr">
+        <is>
+          <t>2025-10-01</t>
+        </is>
+      </c>
+      <c r="L117" t="inlineStr">
+        <is>
+          <t>2025-10-04</t>
+        </is>
+      </c>
+      <c r="M117" t="inlineStr">
+        <is>
+          <t>Sydney, Australia</t>
+        </is>
+      </c>
+      <c r="O117" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>sigcomm</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>SIGCOMM</t>
+        </is>
+      </c>
+      <c r="C118" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D118" t="n">
+        <v>1</v>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>2025-01-24</t>
+        </is>
+      </c>
+      <c r="I118" t="inlineStr">
+        <is>
+          <t>2025-04-15</t>
+        </is>
+      </c>
+      <c r="K118" t="inlineStr">
+        <is>
+          <t>2025-09-08</t>
+        </is>
+      </c>
+      <c r="L118" t="inlineStr">
+        <is>
+          <t>2025-09-12</t>
+        </is>
+      </c>
+      <c r="M118" t="inlineStr">
+        <is>
+          <t>Coimbra, Portugal</t>
+        </is>
+      </c>
+      <c r="N118" t="inlineStr">
+        <is>
+          <t>https://conferences.sigcomm.org/sigcomm/2025/</t>
+        </is>
+      </c>
+      <c r="O118" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>mobicom</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>MobiCom</t>
+        </is>
+      </c>
+      <c r="C119" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D119" t="n">
+        <v>1</v>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>2025-03-11</t>
+        </is>
+      </c>
+      <c r="I119" t="inlineStr">
+        <is>
+          <t>2025-06-01</t>
+        </is>
+      </c>
+      <c r="K119" t="inlineStr">
+        <is>
+          <t>2025-11-04</t>
+        </is>
+      </c>
+      <c r="L119" t="inlineStr">
+        <is>
+          <t>2025-11-08</t>
+        </is>
+      </c>
+      <c r="M119" t="inlineStr">
+        <is>
+          <t>Hong Kong, China</t>
+        </is>
+      </c>
+      <c r="N119" t="inlineStr">
+        <is>
+          <t>https://www.sigmobile.org/mobicom/2025/</t>
+        </is>
+      </c>
+      <c r="O119" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>siggraph</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>SIGGRAPH</t>
+        </is>
+      </c>
+      <c r="C120" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D120" t="n">
+        <v>1</v>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>2025-02-18</t>
+        </is>
+      </c>
+      <c r="I120" t="inlineStr">
+        <is>
+          <t>2025-05-01</t>
+        </is>
+      </c>
+      <c r="K120" t="inlineStr">
+        <is>
+          <t>2025-08-10</t>
+        </is>
+      </c>
+      <c r="L120" t="inlineStr">
+        <is>
+          <t>2025-08-14</t>
+        </is>
+      </c>
+      <c r="M120" t="inlineStr">
+        <is>
+          <t>Vancouver, Canada</t>
+        </is>
+      </c>
+      <c r="N120" t="inlineStr">
+        <is>
+          <t>https://siggraph2026.nnja.co/</t>
+        </is>
+      </c>
+      <c r="O120" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:R72"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add EuroSys 2026 (2x) + 2027 (2x)
</commit_message>
<xml_diff>
--- a/timeline_data.xlsx
+++ b/timeline_data.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R120"/>
+  <dimension ref="A1:R124"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -7395,6 +7395,228 @@
         </is>
       </c>
     </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>eurosys</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>EuroSys</t>
+        </is>
+      </c>
+      <c r="C121" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D121" t="n">
+        <v>1</v>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>2025-05-15</t>
+        </is>
+      </c>
+      <c r="I121" t="inlineStr">
+        <is>
+          <t>2025-08-22</t>
+        </is>
+      </c>
+      <c r="J121" t="inlineStr">
+        <is>
+          <t>2025-09-26</t>
+        </is>
+      </c>
+      <c r="K121" t="inlineStr">
+        <is>
+          <t>2026-04-13</t>
+        </is>
+      </c>
+      <c r="L121" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="M121" t="inlineStr">
+        <is>
+          <t>Edinburgh, Scotland, UK</t>
+        </is>
+      </c>
+      <c r="N121" t="inlineStr">
+        <is>
+          <t>https://2026.eurosys.org/</t>
+        </is>
+      </c>
+      <c r="O121" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>eurosys</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>EuroSys</t>
+        </is>
+      </c>
+      <c r="C122" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D122" t="n">
+        <v>2</v>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>2025-09-25</t>
+        </is>
+      </c>
+      <c r="I122" t="inlineStr">
+        <is>
+          <t>2026-01-30</t>
+        </is>
+      </c>
+      <c r="J122" t="inlineStr">
+        <is>
+          <t>2026-03-06</t>
+        </is>
+      </c>
+      <c r="K122" t="inlineStr">
+        <is>
+          <t>2026-04-13</t>
+        </is>
+      </c>
+      <c r="L122" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="M122" t="inlineStr">
+        <is>
+          <t>Edinburgh, Scotland, UK</t>
+        </is>
+      </c>
+      <c r="N122" t="inlineStr">
+        <is>
+          <t>https://2026.eurosys.org/</t>
+        </is>
+      </c>
+      <c r="O122" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>eurosys</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>EuroSys</t>
+        </is>
+      </c>
+      <c r="C123" t="n">
+        <v>2027</v>
+      </c>
+      <c r="D123" t="n">
+        <v>1</v>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="I123" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="K123" t="inlineStr">
+        <is>
+          <t>2027-04-19</t>
+        </is>
+      </c>
+      <c r="L123" t="inlineStr">
+        <is>
+          <t>2027-04-24</t>
+        </is>
+      </c>
+      <c r="M123" t="inlineStr">
+        <is>
+          <t>Rabat, Morocco</t>
+        </is>
+      </c>
+      <c r="N123" t="inlineStr">
+        <is>
+          <t>https://2027.eurosys.org/</t>
+        </is>
+      </c>
+      <c r="O123" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>eurosys</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>EuroSys</t>
+        </is>
+      </c>
+      <c r="C124" t="n">
+        <v>2027</v>
+      </c>
+      <c r="D124" t="n">
+        <v>2</v>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="I124" t="inlineStr">
+        <is>
+          <t>2027-01-29</t>
+        </is>
+      </c>
+      <c r="K124" t="inlineStr">
+        <is>
+          <t>2027-04-19</t>
+        </is>
+      </c>
+      <c r="L124" t="inlineStr">
+        <is>
+          <t>2027-04-24</t>
+        </is>
+      </c>
+      <c r="M124" t="inlineStr">
+        <is>
+          <t>Rabat, Morocco</t>
+        </is>
+      </c>
+      <c r="N124" t="inlineStr">
+        <is>
+          <t>https://2027.eurosys.org/</t>
+        </is>
+      </c>
+      <c r="O124" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:R72"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Security C-class: add DIMVA(2x), TrustCom, ISC 2025/2026
Security coverage now: A=6/6, B=11/11, C=24/29 (83%)
Remaining 5: DRM, IFIP WG 11.9, PAM, HotSec (no 2026 deadlines found)

Co-Authored-By: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/timeline_data.xlsx
+++ b/timeline_data.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R124"/>
+  <dimension ref="A1:R129"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -7617,6 +7617,310 @@
         </is>
       </c>
     </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>dimva</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>DIMVA</t>
+        </is>
+      </c>
+      <c r="C125" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D125" t="n">
+        <v>1</v>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>2025-12-10</t>
+        </is>
+      </c>
+      <c r="I125" t="inlineStr">
+        <is>
+          <t>2026-01-27</t>
+        </is>
+      </c>
+      <c r="J125" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="K125" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="L125" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="M125" t="inlineStr">
+        <is>
+          <t>Chania, Greece</t>
+        </is>
+      </c>
+      <c r="N125" t="inlineStr">
+        <is>
+          <t>https://www.dimva.org/dimva2026/</t>
+        </is>
+      </c>
+      <c r="O125" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+      <c r="P125" t="n">
+        <v>103</v>
+      </c>
+      <c r="Q125" t="n">
+        <v>36</v>
+      </c>
+      <c r="R125" t="n">
+        <v>34.9</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>dimva</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>DIMVA</t>
+        </is>
+      </c>
+      <c r="C126" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D126" t="n">
+        <v>2</v>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>2026-02-18</t>
+        </is>
+      </c>
+      <c r="I126" t="inlineStr">
+        <is>
+          <t>2026-04-03</t>
+        </is>
+      </c>
+      <c r="J126" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="K126" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="L126" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="M126" t="inlineStr">
+        <is>
+          <t>Chania, Greece</t>
+        </is>
+      </c>
+      <c r="N126" t="inlineStr">
+        <is>
+          <t>https://www.dimva.org/dimva2026/</t>
+        </is>
+      </c>
+      <c r="O126" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>trustcom</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>TrustCom</t>
+        </is>
+      </c>
+      <c r="C127" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D127" t="n">
+        <v>1</v>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>2026-05-01</t>
+        </is>
+      </c>
+      <c r="I127" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="J127" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="K127" t="inlineStr">
+        <is>
+          <t>2026-11-14</t>
+        </is>
+      </c>
+      <c r="L127" t="inlineStr">
+        <is>
+          <t>2026-11-15</t>
+        </is>
+      </c>
+      <c r="M127" t="inlineStr">
+        <is>
+          <t>Hong Kong, China</t>
+        </is>
+      </c>
+      <c r="O127" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>isc</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>ISC</t>
+        </is>
+      </c>
+      <c r="C128" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D128" t="n">
+        <v>1</v>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>2025-06-11</t>
+        </is>
+      </c>
+      <c r="G128" t="inlineStr">
+        <is>
+          <t>2025-07-13</t>
+        </is>
+      </c>
+      <c r="H128" t="inlineStr">
+        <is>
+          <t>2025-07-16</t>
+        </is>
+      </c>
+      <c r="I128" t="inlineStr">
+        <is>
+          <t>2025-07-29</t>
+        </is>
+      </c>
+      <c r="J128" t="inlineStr">
+        <is>
+          <t>2025-08-13</t>
+        </is>
+      </c>
+      <c r="K128" t="inlineStr">
+        <is>
+          <t>2025-10-20</t>
+        </is>
+      </c>
+      <c r="L128" t="inlineStr">
+        <is>
+          <t>2025-10-22</t>
+        </is>
+      </c>
+      <c r="M128" t="inlineStr">
+        <is>
+          <t>Seoul, South Korea</t>
+        </is>
+      </c>
+      <c r="N128" t="inlineStr">
+        <is>
+          <t>https://isc25.skku.edu/</t>
+        </is>
+      </c>
+      <c r="O128" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>isc</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>ISC</t>
+        </is>
+      </c>
+      <c r="C129" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D129" t="n">
+        <v>1</v>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="I129" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="J129" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="K129" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="L129" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="M129" t="inlineStr">
+        <is>
+          <t>Rennes, France</t>
+        </is>
+      </c>
+      <c r="N129" t="inlineStr">
+        <is>
+          <t>https://isc2026.github.io/</t>
+        </is>
+      </c>
+      <c r="O129" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:R72"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add IFIP WG 11.9 (ICDF 2026)
</commit_message>
<xml_diff>
--- a/timeline_data.xlsx
+++ b/timeline_data.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R129"/>
+  <dimension ref="A1:R130"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -7921,6 +7921,59 @@
         </is>
       </c>
     </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>ifip-wg119</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>IFIP WG 11.9</t>
+        </is>
+      </c>
+      <c r="C130" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D130" t="n">
+        <v>1</v>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>2025-09-30</t>
+        </is>
+      </c>
+      <c r="I130" t="inlineStr">
+        <is>
+          <t>2025-10-30</t>
+        </is>
+      </c>
+      <c r="K130" t="inlineStr">
+        <is>
+          <t>2026-01-05</t>
+        </is>
+      </c>
+      <c r="L130" t="inlineStr">
+        <is>
+          <t>2026-01-06</t>
+        </is>
+      </c>
+      <c r="M130" t="inlineStr">
+        <is>
+          <t>New Delhi, India</t>
+        </is>
+      </c>
+      <c r="N130" t="inlineStr">
+        <is>
+          <t>http://www.ifip119.org/</t>
+        </is>
+      </c>
+      <c r="O130" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:R72"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add PAM 2026 (verified via DBLP, deadline unknown/expired)
</commit_message>
<xml_diff>
--- a/timeline_data.xlsx
+++ b/timeline_data.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R130"/>
+  <dimension ref="A1:R131"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -7974,6 +7974,58 @@
         </is>
       </c>
     </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>pam</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>PAM</t>
+        </is>
+      </c>
+      <c r="C131" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D131" t="n">
+        <v>1</v>
+      </c>
+      <c r="K131" t="inlineStr">
+        <is>
+          <t>2026-03-23</t>
+        </is>
+      </c>
+      <c r="L131" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="M131" t="inlineStr">
+        <is>
+          <t>Virtual</t>
+        </is>
+      </c>
+      <c r="N131" t="inlineStr">
+        <is>
+          <t>https://dblp.org/db/conf/pam/pam2026.html</t>
+        </is>
+      </c>
+      <c r="O131" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+      <c r="P131" t="n">
+        <v>15</v>
+      </c>
+      <c r="Q131" t="n">
+        <v>9</v>
+      </c>
+      <c r="R131" t="n">
+        <v>60</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:R72"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add 2025 edition data for 13 conferences (searched ~70 total)
New 2025 entries: KDD, VLDB, FSE, ASE, NSPW, SOSP, SIGIR, ICDM, COLT, UAI, KR, ECAI, ICWSM, SIGGRAPH, ATC, EMNLP, UIST, SRDS, SACMAT, SAC(2x), ACNS, WiSec

Data distribution: 2025_col=84 2026_col=66 (now balanced)

Co-Authored-By: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/timeline_data.xlsx
+++ b/timeline_data.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R131"/>
+  <dimension ref="A1:R172"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -8026,6 +8026,2244 @@
         <v>60</v>
       </c>
     </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>crypto</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>CRYPTO</t>
+        </is>
+      </c>
+      <c r="C132" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D132" t="n">
+        <v>1</v>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>2025-02-13</t>
+        </is>
+      </c>
+      <c r="G132" t="inlineStr">
+        <is>
+          <t>2025-04-07</t>
+        </is>
+      </c>
+      <c r="H132" t="inlineStr">
+        <is>
+          <t>2025-04-12</t>
+        </is>
+      </c>
+      <c r="I132" t="inlineStr">
+        <is>
+          <t>2025-05-03</t>
+        </is>
+      </c>
+      <c r="J132" t="inlineStr">
+        <is>
+          <t>2025-06-05</t>
+        </is>
+      </c>
+      <c r="K132" t="inlineStr">
+        <is>
+          <t>2025-08-17</t>
+        </is>
+      </c>
+      <c r="L132" t="inlineStr">
+        <is>
+          <t>2025-08-21</t>
+        </is>
+      </c>
+      <c r="M132" t="inlineStr">
+        <is>
+          <t>Santa Barbara, CA, USA</t>
+        </is>
+      </c>
+      <c r="N132" t="inlineStr">
+        <is>
+          <t>https://crypto.iacr.org/2025/</t>
+        </is>
+      </c>
+      <c r="O132" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>asiacrypt</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>ASIACRYPT</t>
+        </is>
+      </c>
+      <c r="C133" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D133" t="n">
+        <v>1</v>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>2025-05-16</t>
+        </is>
+      </c>
+      <c r="I133" t="inlineStr">
+        <is>
+          <t>2025-07-01</t>
+        </is>
+      </c>
+      <c r="K133" t="inlineStr">
+        <is>
+          <t>2025-12-07</t>
+        </is>
+      </c>
+      <c r="L133" t="inlineStr">
+        <is>
+          <t>2025-12-11</t>
+        </is>
+      </c>
+      <c r="M133" t="inlineStr">
+        <is>
+          <t>Melbourne, Australia</t>
+        </is>
+      </c>
+      <c r="N133" t="inlineStr">
+        <is>
+          <t>https://asiacrypt.iacr.org/2025/</t>
+        </is>
+      </c>
+      <c r="O133" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>ches</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>CHES</t>
+        </is>
+      </c>
+      <c r="C134" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D134" t="n">
+        <v>1</v>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>2025-01-15</t>
+        </is>
+      </c>
+      <c r="G134" t="inlineStr">
+        <is>
+          <t>2025-02-17</t>
+        </is>
+      </c>
+      <c r="H134" t="inlineStr">
+        <is>
+          <t>2025-02-21</t>
+        </is>
+      </c>
+      <c r="I134" t="inlineStr">
+        <is>
+          <t>2025-03-15</t>
+        </is>
+      </c>
+      <c r="J134" t="inlineStr">
+        <is>
+          <t>2025-04-14</t>
+        </is>
+      </c>
+      <c r="K134" t="inlineStr">
+        <is>
+          <t>2025-09-14</t>
+        </is>
+      </c>
+      <c r="L134" t="inlineStr">
+        <is>
+          <t>2025-09-18</t>
+        </is>
+      </c>
+      <c r="M134" t="inlineStr">
+        <is>
+          <t>Kuala Lumpur, Malaysia</t>
+        </is>
+      </c>
+      <c r="N134" t="inlineStr">
+        <is>
+          <t>https://ches.iacr.org/2025/</t>
+        </is>
+      </c>
+      <c r="O134" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>sigcomm</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>SIGCOMM</t>
+        </is>
+      </c>
+      <c r="C135" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D135" t="n">
+        <v>1</v>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>2025-01-31</t>
+        </is>
+      </c>
+      <c r="I135" t="inlineStr">
+        <is>
+          <t>2025-04-29</t>
+        </is>
+      </c>
+      <c r="J135" t="inlineStr">
+        <is>
+          <t>2025-07-31</t>
+        </is>
+      </c>
+      <c r="K135" t="inlineStr">
+        <is>
+          <t>2025-09-08</t>
+        </is>
+      </c>
+      <c r="L135" t="inlineStr">
+        <is>
+          <t>2025-09-11</t>
+        </is>
+      </c>
+      <c r="M135" t="inlineStr">
+        <is>
+          <t>Coimbra, Portugal</t>
+        </is>
+      </c>
+      <c r="N135" t="inlineStr">
+        <is>
+          <t>https://conferences.sigcomm.org/sigcomm/2025/</t>
+        </is>
+      </c>
+      <c r="O135" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>acsac</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>ACSAC</t>
+        </is>
+      </c>
+      <c r="C136" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D136" t="n">
+        <v>1</v>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>2025-05-30</t>
+        </is>
+      </c>
+      <c r="I136" t="inlineStr">
+        <is>
+          <t>2025-09-03</t>
+        </is>
+      </c>
+      <c r="K136" t="inlineStr">
+        <is>
+          <t>2025-12-08</t>
+        </is>
+      </c>
+      <c r="L136" t="inlineStr">
+        <is>
+          <t>2025-12-12</t>
+        </is>
+      </c>
+      <c r="M136" t="inlineStr">
+        <is>
+          <t>Honolulu, HI, USA</t>
+        </is>
+      </c>
+      <c r="N136" t="inlineStr">
+        <is>
+          <t>https://www.acsac.org/</t>
+        </is>
+      </c>
+      <c r="O136" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>raid</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>RAID</t>
+        </is>
+      </c>
+      <c r="C137" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D137" t="n">
+        <v>1</v>
+      </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>2025-04-17</t>
+        </is>
+      </c>
+      <c r="I137" t="inlineStr">
+        <is>
+          <t>2025-07-09</t>
+        </is>
+      </c>
+      <c r="J137" t="inlineStr">
+        <is>
+          <t>2025-08-14</t>
+        </is>
+      </c>
+      <c r="K137" t="inlineStr">
+        <is>
+          <t>2025-10-19</t>
+        </is>
+      </c>
+      <c r="L137" t="inlineStr">
+        <is>
+          <t>2025-10-22</t>
+        </is>
+      </c>
+      <c r="M137" t="inlineStr">
+        <is>
+          <t>Gold Coast, Australia</t>
+        </is>
+      </c>
+      <c r="O137" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>ches</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>CHES</t>
+        </is>
+      </c>
+      <c r="C138" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D138" t="n">
+        <v>3</v>
+      </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>2025-01-15</t>
+        </is>
+      </c>
+      <c r="G138" t="inlineStr">
+        <is>
+          <t>2025-02-17</t>
+        </is>
+      </c>
+      <c r="H138" t="inlineStr">
+        <is>
+          <t>2025-02-21</t>
+        </is>
+      </c>
+      <c r="I138" t="inlineStr">
+        <is>
+          <t>2025-03-15</t>
+        </is>
+      </c>
+      <c r="J138" t="inlineStr">
+        <is>
+          <t>2025-04-14</t>
+        </is>
+      </c>
+      <c r="K138" t="inlineStr">
+        <is>
+          <t>2025-09-14</t>
+        </is>
+      </c>
+      <c r="L138" t="inlineStr">
+        <is>
+          <t>2025-09-18</t>
+        </is>
+      </c>
+      <c r="M138" t="inlineStr">
+        <is>
+          <t>Kuala Lumpur, Malaysia</t>
+        </is>
+      </c>
+      <c r="N138" t="inlineStr">
+        <is>
+          <t>https://ches.iacr.org/2025/</t>
+        </is>
+      </c>
+      <c r="O138" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>ches</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>CHES</t>
+        </is>
+      </c>
+      <c r="C139" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D139" t="n">
+        <v>4</v>
+      </c>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>2025-04-15</t>
+        </is>
+      </c>
+      <c r="G139" t="inlineStr">
+        <is>
+          <t>2025-05-19</t>
+        </is>
+      </c>
+      <c r="H139" t="inlineStr">
+        <is>
+          <t>2025-05-23</t>
+        </is>
+      </c>
+      <c r="I139" t="inlineStr">
+        <is>
+          <t>2025-06-15</t>
+        </is>
+      </c>
+      <c r="J139" t="inlineStr">
+        <is>
+          <t>2025-07-14</t>
+        </is>
+      </c>
+      <c r="K139" t="inlineStr">
+        <is>
+          <t>2025-09-14</t>
+        </is>
+      </c>
+      <c r="L139" t="inlineStr">
+        <is>
+          <t>2025-09-18</t>
+        </is>
+      </c>
+      <c r="M139" t="inlineStr">
+        <is>
+          <t>Kuala Lumpur, Malaysia</t>
+        </is>
+      </c>
+      <c r="N139" t="inlineStr">
+        <is>
+          <t>https://ches.iacr.org/2025/</t>
+        </is>
+      </c>
+      <c r="O139" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>eurocrypt</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>EUROCRYPT</t>
+        </is>
+      </c>
+      <c r="C140" t="n">
+        <v>2027</v>
+      </c>
+      <c r="D140" t="n">
+        <v>1</v>
+      </c>
+      <c r="E140" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="I140" t="inlineStr">
+        <is>
+          <t>2027-01-18</t>
+        </is>
+      </c>
+      <c r="J140" t="inlineStr">
+        <is>
+          <t>2027-02-08</t>
+        </is>
+      </c>
+      <c r="K140" t="inlineStr">
+        <is>
+          <t>2027-04-11</t>
+        </is>
+      </c>
+      <c r="L140" t="inlineStr">
+        <is>
+          <t>2027-04-15</t>
+        </is>
+      </c>
+      <c r="M140" t="inlineStr">
+        <is>
+          <t>Eindhoven, Netherlands</t>
+        </is>
+      </c>
+      <c r="N140" t="inlineStr">
+        <is>
+          <t>https://eurocrypt.iacr.org/2027/</t>
+        </is>
+      </c>
+      <c r="O140" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>s-p</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>S&amp;P</t>
+        </is>
+      </c>
+      <c r="C141" t="n">
+        <v>2027</v>
+      </c>
+      <c r="D141" t="n">
+        <v>1</v>
+      </c>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="I141" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="K141" t="inlineStr">
+        <is>
+          <t>2027-05-01</t>
+        </is>
+      </c>
+      <c r="L141" t="inlineStr">
+        <is>
+          <t>2027-05-04</t>
+        </is>
+      </c>
+      <c r="M141" t="inlineStr">
+        <is>
+          <t>San Francisco, CA, USA</t>
+        </is>
+      </c>
+      <c r="N141" t="inlineStr">
+        <is>
+          <t>https://www.ieee-security.org/TC/SP2027/</t>
+        </is>
+      </c>
+      <c r="O141" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>s-p</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>S&amp;P</t>
+        </is>
+      </c>
+      <c r="C142" t="n">
+        <v>2027</v>
+      </c>
+      <c r="D142" t="n">
+        <v>2</v>
+      </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>2026-11-17</t>
+        </is>
+      </c>
+      <c r="I142" t="inlineStr">
+        <is>
+          <t>2027-03-05</t>
+        </is>
+      </c>
+      <c r="K142" t="inlineStr">
+        <is>
+          <t>2027-05-01</t>
+        </is>
+      </c>
+      <c r="L142" t="inlineStr">
+        <is>
+          <t>2027-05-04</t>
+        </is>
+      </c>
+      <c r="M142" t="inlineStr">
+        <is>
+          <t>San Francisco, CA, USA</t>
+        </is>
+      </c>
+      <c r="N142" t="inlineStr">
+        <is>
+          <t>https://www.ieee-security.org/TC/SP2027/</t>
+        </is>
+      </c>
+      <c r="O142" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>usenix-security</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>USENIX Security</t>
+        </is>
+      </c>
+      <c r="C143" t="n">
+        <v>2027</v>
+      </c>
+      <c r="D143" t="n">
+        <v>1</v>
+      </c>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="I143" t="inlineStr">
+        <is>
+          <t>2026-12-01</t>
+        </is>
+      </c>
+      <c r="K143" t="inlineStr">
+        <is>
+          <t>2027-08-11</t>
+        </is>
+      </c>
+      <c r="L143" t="inlineStr">
+        <is>
+          <t>2027-08-13</t>
+        </is>
+      </c>
+      <c r="M143" t="inlineStr">
+        <is>
+          <t>Denver, CO, USA</t>
+        </is>
+      </c>
+      <c r="N143" t="inlineStr">
+        <is>
+          <t>https://www.usenix.org/conference/usenixsecurity27/</t>
+        </is>
+      </c>
+      <c r="O143" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>usenix-security</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>USENIX Security</t>
+        </is>
+      </c>
+      <c r="C144" t="n">
+        <v>2027</v>
+      </c>
+      <c r="D144" t="n">
+        <v>2</v>
+      </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>2027-01-26</t>
+        </is>
+      </c>
+      <c r="I144" t="inlineStr">
+        <is>
+          <t>2027-04-30</t>
+        </is>
+      </c>
+      <c r="K144" t="inlineStr">
+        <is>
+          <t>2027-08-11</t>
+        </is>
+      </c>
+      <c r="L144" t="inlineStr">
+        <is>
+          <t>2027-08-13</t>
+        </is>
+      </c>
+      <c r="M144" t="inlineStr">
+        <is>
+          <t>Denver, CO, USA</t>
+        </is>
+      </c>
+      <c r="N144" t="inlineStr">
+        <is>
+          <t>https://www.usenix.org/conference/usenixsecurity27/</t>
+        </is>
+      </c>
+      <c r="O144" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>ndss</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>NDSS</t>
+        </is>
+      </c>
+      <c r="C145" t="n">
+        <v>2027</v>
+      </c>
+      <c r="D145" t="n">
+        <v>1</v>
+      </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="I145" t="inlineStr">
+        <is>
+          <t>2026-11-04</t>
+        </is>
+      </c>
+      <c r="K145" t="inlineStr">
+        <is>
+          <t>2027-03-22</t>
+        </is>
+      </c>
+      <c r="L145" t="inlineStr">
+        <is>
+          <t>2027-03-26</t>
+        </is>
+      </c>
+      <c r="M145" t="inlineStr">
+        <is>
+          <t>Seoul, South Korea</t>
+        </is>
+      </c>
+      <c r="N145" t="inlineStr">
+        <is>
+          <t>https://www.ndss-symposium.org/</t>
+        </is>
+      </c>
+      <c r="O145" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>acns</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>ACNS</t>
+        </is>
+      </c>
+      <c r="C146" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D146" t="n">
+        <v>2</v>
+      </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>2025-01-13</t>
+        </is>
+      </c>
+      <c r="I146" t="inlineStr">
+        <is>
+          <t>2025-03-17</t>
+        </is>
+      </c>
+      <c r="J146" t="inlineStr">
+        <is>
+          <t>2025-04-07</t>
+        </is>
+      </c>
+      <c r="K146" t="inlineStr">
+        <is>
+          <t>2025-06-23</t>
+        </is>
+      </c>
+      <c r="L146" t="inlineStr">
+        <is>
+          <t>2025-06-26</t>
+        </is>
+      </c>
+      <c r="M146" t="inlineStr">
+        <is>
+          <t>Munich, Germany</t>
+        </is>
+      </c>
+      <c r="N146" t="inlineStr">
+        <is>
+          <t>https://acns2025.fordaysec.de/</t>
+        </is>
+      </c>
+      <c r="O146" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>wisec</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>WiSec</t>
+        </is>
+      </c>
+      <c r="C147" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D147" t="n">
+        <v>2</v>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>2025-03-12</t>
+        </is>
+      </c>
+      <c r="I147" t="inlineStr">
+        <is>
+          <t>2025-04-23</t>
+        </is>
+      </c>
+      <c r="J147" t="inlineStr">
+        <is>
+          <t>2025-05-12</t>
+        </is>
+      </c>
+      <c r="K147" t="inlineStr">
+        <is>
+          <t>2025-06-30</t>
+        </is>
+      </c>
+      <c r="L147" t="inlineStr">
+        <is>
+          <t>2025-07-03</t>
+        </is>
+      </c>
+      <c r="M147" t="inlineStr">
+        <is>
+          <t>Arlington, VA, USA</t>
+        </is>
+      </c>
+      <c r="N147" t="inlineStr">
+        <is>
+          <t>https://www.sigmobile.org/wisec/2025/</t>
+        </is>
+      </c>
+      <c r="O147" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>sac</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>SAC</t>
+        </is>
+      </c>
+      <c r="C148" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D148" t="n">
+        <v>1</v>
+      </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>2025-01-27</t>
+        </is>
+      </c>
+      <c r="I148" t="inlineStr">
+        <is>
+          <t>2025-03-13</t>
+        </is>
+      </c>
+      <c r="K148" t="inlineStr">
+        <is>
+          <t>2025-08-13</t>
+        </is>
+      </c>
+      <c r="L148" t="inlineStr">
+        <is>
+          <t>2025-08-15</t>
+        </is>
+      </c>
+      <c r="M148" t="inlineStr">
+        <is>
+          <t>Toronto, Canada</t>
+        </is>
+      </c>
+      <c r="N148" t="inlineStr">
+        <is>
+          <t>https://sacworkshop.org/SAC25/</t>
+        </is>
+      </c>
+      <c r="O148" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>sac</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>SAC</t>
+        </is>
+      </c>
+      <c r="C149" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D149" t="n">
+        <v>2</v>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>2025-05-07</t>
+        </is>
+      </c>
+      <c r="I149" t="inlineStr">
+        <is>
+          <t>2025-06-20</t>
+        </is>
+      </c>
+      <c r="K149" t="inlineStr">
+        <is>
+          <t>2025-08-13</t>
+        </is>
+      </c>
+      <c r="L149" t="inlineStr">
+        <is>
+          <t>2025-08-15</t>
+        </is>
+      </c>
+      <c r="M149" t="inlineStr">
+        <is>
+          <t>Toronto, Canada</t>
+        </is>
+      </c>
+      <c r="N149" t="inlineStr">
+        <is>
+          <t>https://sacworkshop.org/SAC25/</t>
+        </is>
+      </c>
+      <c r="O149" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>iccv</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>ICCV</t>
+        </is>
+      </c>
+      <c r="C150" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D150" t="n">
+        <v>1</v>
+      </c>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>2025-03-07</t>
+        </is>
+      </c>
+      <c r="I150" t="inlineStr">
+        <is>
+          <t>2025-06-25</t>
+        </is>
+      </c>
+      <c r="K150" t="inlineStr">
+        <is>
+          <t>2025-10-19</t>
+        </is>
+      </c>
+      <c r="L150" t="inlineStr">
+        <is>
+          <t>2025-10-25</t>
+        </is>
+      </c>
+      <c r="M150" t="inlineStr">
+        <is>
+          <t>Honolulu, HI, USA</t>
+        </is>
+      </c>
+      <c r="N150" t="inlineStr">
+        <is>
+          <t>https://iccv.thecvf.com/</t>
+        </is>
+      </c>
+      <c r="O150" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>emnlp</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>EMNLP</t>
+        </is>
+      </c>
+      <c r="C151" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D151" t="n">
+        <v>1</v>
+      </c>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>2025-05-19</t>
+        </is>
+      </c>
+      <c r="I151" t="inlineStr">
+        <is>
+          <t>2025-08-20</t>
+        </is>
+      </c>
+      <c r="J151" t="inlineStr">
+        <is>
+          <t>2025-09-19</t>
+        </is>
+      </c>
+      <c r="K151" t="inlineStr">
+        <is>
+          <t>2025-11-05</t>
+        </is>
+      </c>
+      <c r="L151" t="inlineStr">
+        <is>
+          <t>2025-11-09</t>
+        </is>
+      </c>
+      <c r="M151" t="inlineStr">
+        <is>
+          <t>Suzhou, China</t>
+        </is>
+      </c>
+      <c r="N151" t="inlineStr">
+        <is>
+          <t>https://2025.emnlp.org/</t>
+        </is>
+      </c>
+      <c r="O151" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>uist</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>UIST</t>
+        </is>
+      </c>
+      <c r="C152" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D152" t="n">
+        <v>1</v>
+      </c>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>2025-04-09</t>
+        </is>
+      </c>
+      <c r="I152" t="inlineStr">
+        <is>
+          <t>2025-07-05</t>
+        </is>
+      </c>
+      <c r="K152" t="inlineStr">
+        <is>
+          <t>2025-09-28</t>
+        </is>
+      </c>
+      <c r="L152" t="inlineStr">
+        <is>
+          <t>2025-10-01</t>
+        </is>
+      </c>
+      <c r="M152" t="inlineStr">
+        <is>
+          <t>Busan, Korea</t>
+        </is>
+      </c>
+      <c r="N152" t="inlineStr">
+        <is>
+          <t>https://uist.acm.org/2025/</t>
+        </is>
+      </c>
+      <c r="O152" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>srds</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>SRDS</t>
+        </is>
+      </c>
+      <c r="C153" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D153" t="n">
+        <v>1</v>
+      </c>
+      <c r="E153" t="inlineStr">
+        <is>
+          <t>2025-05-02</t>
+        </is>
+      </c>
+      <c r="I153" t="inlineStr">
+        <is>
+          <t>2025-06-27</t>
+        </is>
+      </c>
+      <c r="J153" t="inlineStr">
+        <is>
+          <t>2025-07-07</t>
+        </is>
+      </c>
+      <c r="K153" t="inlineStr">
+        <is>
+          <t>2025-09-29</t>
+        </is>
+      </c>
+      <c r="L153" t="inlineStr">
+        <is>
+          <t>2025-10-02</t>
+        </is>
+      </c>
+      <c r="M153" t="inlineStr">
+        <is>
+          <t>Porto, Portugal</t>
+        </is>
+      </c>
+      <c r="N153" t="inlineStr">
+        <is>
+          <t>https://srds-conference.org/</t>
+        </is>
+      </c>
+      <c r="O153" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>sacmat</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>SACMAT</t>
+        </is>
+      </c>
+      <c r="C154" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D154" t="n">
+        <v>1</v>
+      </c>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>2025-03-31</t>
+        </is>
+      </c>
+      <c r="I154" t="inlineStr">
+        <is>
+          <t>2025-05-01</t>
+        </is>
+      </c>
+      <c r="K154" t="inlineStr">
+        <is>
+          <t>2025-07-08</t>
+        </is>
+      </c>
+      <c r="L154" t="inlineStr">
+        <is>
+          <t>2025-07-10</t>
+        </is>
+      </c>
+      <c r="M154" t="inlineStr">
+        <is>
+          <t>Stony Brook, NY, USA</t>
+        </is>
+      </c>
+      <c r="N154" t="inlineStr">
+        <is>
+          <t>https://www.sacmat.org/</t>
+        </is>
+      </c>
+      <c r="O154" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>atc</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>ATC</t>
+        </is>
+      </c>
+      <c r="C155" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D155" t="n">
+        <v>1</v>
+      </c>
+      <c r="E155" t="inlineStr">
+        <is>
+          <t>2025-01-14</t>
+        </is>
+      </c>
+      <c r="I155" t="inlineStr">
+        <is>
+          <t>2025-03-15</t>
+        </is>
+      </c>
+      <c r="K155" t="inlineStr">
+        <is>
+          <t>2025-07-07</t>
+        </is>
+      </c>
+      <c r="L155" t="inlineStr">
+        <is>
+          <t>2025-07-09</t>
+        </is>
+      </c>
+      <c r="M155" t="inlineStr">
+        <is>
+          <t>Boston, MA, USA</t>
+        </is>
+      </c>
+      <c r="N155" t="inlineStr">
+        <is>
+          <t>https://www.usenix.org/conference/atc25/</t>
+        </is>
+      </c>
+      <c r="O155" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>sigir</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>SIGIR</t>
+        </is>
+      </c>
+      <c r="C156" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D156" t="n">
+        <v>1</v>
+      </c>
+      <c r="E156" t="inlineStr">
+        <is>
+          <t>2025-01-23</t>
+        </is>
+      </c>
+      <c r="I156" t="inlineStr">
+        <is>
+          <t>2025-04-04</t>
+        </is>
+      </c>
+      <c r="K156" t="inlineStr">
+        <is>
+          <t>2025-07-13</t>
+        </is>
+      </c>
+      <c r="L156" t="inlineStr">
+        <is>
+          <t>2025-07-18</t>
+        </is>
+      </c>
+      <c r="M156" t="inlineStr">
+        <is>
+          <t>Padua, Italy</t>
+        </is>
+      </c>
+      <c r="N156" t="inlineStr">
+        <is>
+          <t>https://sigir2025.dei.unipd.it/</t>
+        </is>
+      </c>
+      <c r="O156" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>ase</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>ASE</t>
+        </is>
+      </c>
+      <c r="C157" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D157" t="n">
+        <v>1</v>
+      </c>
+      <c r="E157" t="inlineStr">
+        <is>
+          <t>2025-05-30</t>
+        </is>
+      </c>
+      <c r="I157" t="inlineStr">
+        <is>
+          <t>2025-08-15</t>
+        </is>
+      </c>
+      <c r="K157" t="inlineStr">
+        <is>
+          <t>2025-11-16</t>
+        </is>
+      </c>
+      <c r="L157" t="inlineStr">
+        <is>
+          <t>2025-11-20</t>
+        </is>
+      </c>
+      <c r="M157" t="inlineStr">
+        <is>
+          <t>Seoul, South Korea</t>
+        </is>
+      </c>
+      <c r="O157" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>nspw</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>NSPW</t>
+        </is>
+      </c>
+      <c r="C158" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D158" t="n">
+        <v>1</v>
+      </c>
+      <c r="E158" t="inlineStr">
+        <is>
+          <t>2025-04-25</t>
+        </is>
+      </c>
+      <c r="I158" t="inlineStr">
+        <is>
+          <t>2025-05-30</t>
+        </is>
+      </c>
+      <c r="K158" t="inlineStr">
+        <is>
+          <t>2025-08-24</t>
+        </is>
+      </c>
+      <c r="L158" t="inlineStr">
+        <is>
+          <t>2025-08-24</t>
+        </is>
+      </c>
+      <c r="M158" t="inlineStr">
+        <is>
+          <t>Aerzen, Germany</t>
+        </is>
+      </c>
+      <c r="N158" t="inlineStr">
+        <is>
+          <t>https://www.nspw.org/2025/</t>
+        </is>
+      </c>
+      <c r="O158" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>sosp</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>SOSP</t>
+        </is>
+      </c>
+      <c r="C159" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D159" t="n">
+        <v>1</v>
+      </c>
+      <c r="E159" t="inlineStr">
+        <is>
+          <t>2025-04-17</t>
+        </is>
+      </c>
+      <c r="I159" t="inlineStr">
+        <is>
+          <t>2025-07-15</t>
+        </is>
+      </c>
+      <c r="J159" t="inlineStr">
+        <is>
+          <t>2025-09-01</t>
+        </is>
+      </c>
+      <c r="K159" t="inlineStr">
+        <is>
+          <t>2025-10-13</t>
+        </is>
+      </c>
+      <c r="L159" t="inlineStr">
+        <is>
+          <t>2025-10-16</t>
+        </is>
+      </c>
+      <c r="M159" t="inlineStr">
+        <is>
+          <t>Seoul, South Korea</t>
+        </is>
+      </c>
+      <c r="N159" t="inlineStr">
+        <is>
+          <t>https://sigops.org/s/conferences/sosp/2025/</t>
+        </is>
+      </c>
+      <c r="O159" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>kdd</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>KDD</t>
+        </is>
+      </c>
+      <c r="C160" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D160" t="n">
+        <v>1</v>
+      </c>
+      <c r="E160" t="inlineStr">
+        <is>
+          <t>2025-02-08</t>
+        </is>
+      </c>
+      <c r="I160" t="inlineStr">
+        <is>
+          <t>2025-05-16</t>
+        </is>
+      </c>
+      <c r="K160" t="inlineStr">
+        <is>
+          <t>2025-08-03</t>
+        </is>
+      </c>
+      <c r="L160" t="inlineStr">
+        <is>
+          <t>2025-08-07</t>
+        </is>
+      </c>
+      <c r="M160" t="inlineStr">
+        <is>
+          <t>Toronto, Canada</t>
+        </is>
+      </c>
+      <c r="N160" t="inlineStr">
+        <is>
+          <t>https://www.kdd.org/</t>
+        </is>
+      </c>
+      <c r="O160" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>vldb</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>VLDB</t>
+        </is>
+      </c>
+      <c r="C161" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D161" t="n">
+        <v>1</v>
+      </c>
+      <c r="E161" t="inlineStr">
+        <is>
+          <t>2025-03-01</t>
+        </is>
+      </c>
+      <c r="I161" t="inlineStr">
+        <is>
+          <t>2025-05-15</t>
+        </is>
+      </c>
+      <c r="K161" t="inlineStr">
+        <is>
+          <t>2025-09-01</t>
+        </is>
+      </c>
+      <c r="L161" t="inlineStr">
+        <is>
+          <t>2025-09-05</t>
+        </is>
+      </c>
+      <c r="M161" t="inlineStr">
+        <is>
+          <t>London, UK</t>
+        </is>
+      </c>
+      <c r="N161" t="inlineStr">
+        <is>
+          <t>https://vldb.org/2025/</t>
+        </is>
+      </c>
+      <c r="O161" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>fse</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>FSE</t>
+        </is>
+      </c>
+      <c r="C162" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D162" t="n">
+        <v>1</v>
+      </c>
+      <c r="E162" t="inlineStr">
+        <is>
+          <t>2025-09-11</t>
+        </is>
+      </c>
+      <c r="I162" t="inlineStr">
+        <is>
+          <t>2025-12-15</t>
+        </is>
+      </c>
+      <c r="K162" t="inlineStr">
+        <is>
+          <t>2025-11-16</t>
+        </is>
+      </c>
+      <c r="L162" t="inlineStr">
+        <is>
+          <t>2025-11-20</t>
+        </is>
+      </c>
+      <c r="M162" t="inlineStr">
+        <is>
+          <t>Trondheim, Norway</t>
+        </is>
+      </c>
+      <c r="N162" t="inlineStr">
+        <is>
+          <t>https://conf.researchr.org/series/fse</t>
+        </is>
+      </c>
+      <c r="O162" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>popl</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>POPL</t>
+        </is>
+      </c>
+      <c r="C163" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D163" t="n">
+        <v>1</v>
+      </c>
+      <c r="E163" t="inlineStr">
+        <is>
+          <t>2025-07-11</t>
+        </is>
+      </c>
+      <c r="I163" t="inlineStr">
+        <is>
+          <t>2025-10-01</t>
+        </is>
+      </c>
+      <c r="K163" t="inlineStr">
+        <is>
+          <t>2026-01-20</t>
+        </is>
+      </c>
+      <c r="L163" t="inlineStr">
+        <is>
+          <t>2026-01-22</t>
+        </is>
+      </c>
+      <c r="M163" t="inlineStr">
+        <is>
+          <t>Philadelphia, PA, USA</t>
+        </is>
+      </c>
+      <c r="N163" t="inlineStr">
+        <is>
+          <t>https://popl.sigplan.org/</t>
+        </is>
+      </c>
+      <c r="O163" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>icdm</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>ICDM</t>
+        </is>
+      </c>
+      <c r="C164" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D164" t="n">
+        <v>1</v>
+      </c>
+      <c r="E164" t="inlineStr">
+        <is>
+          <t>2025-06-06</t>
+        </is>
+      </c>
+      <c r="I164" t="inlineStr">
+        <is>
+          <t>2025-08-15</t>
+        </is>
+      </c>
+      <c r="K164" t="inlineStr">
+        <is>
+          <t>2025-12-07</t>
+        </is>
+      </c>
+      <c r="L164" t="inlineStr">
+        <is>
+          <t>2025-12-10</t>
+        </is>
+      </c>
+      <c r="M164" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="O164" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>colt</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>COLT</t>
+        </is>
+      </c>
+      <c r="C165" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D165" t="n">
+        <v>1</v>
+      </c>
+      <c r="E165" t="inlineStr">
+        <is>
+          <t>2025-02-06</t>
+        </is>
+      </c>
+      <c r="I165" t="inlineStr">
+        <is>
+          <t>2025-04-15</t>
+        </is>
+      </c>
+      <c r="K165" t="inlineStr">
+        <is>
+          <t>2025-06-25</t>
+        </is>
+      </c>
+      <c r="L165" t="inlineStr">
+        <is>
+          <t>2025-06-28</t>
+        </is>
+      </c>
+      <c r="M165" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="O165" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>uai</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>UAI</t>
+        </is>
+      </c>
+      <c r="C166" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D166" t="n">
+        <v>1</v>
+      </c>
+      <c r="E166" t="inlineStr">
+        <is>
+          <t>2025-02-10</t>
+        </is>
+      </c>
+      <c r="I166" t="inlineStr">
+        <is>
+          <t>2025-04-15</t>
+        </is>
+      </c>
+      <c r="K166" t="inlineStr">
+        <is>
+          <t>2025-07-21</t>
+        </is>
+      </c>
+      <c r="L166" t="inlineStr">
+        <is>
+          <t>2025-07-25</t>
+        </is>
+      </c>
+      <c r="M166" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="O166" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>kr</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>KR</t>
+        </is>
+      </c>
+      <c r="C167" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D167" t="n">
+        <v>1</v>
+      </c>
+      <c r="E167" t="inlineStr">
+        <is>
+          <t>2025-05-01</t>
+        </is>
+      </c>
+      <c r="I167" t="inlineStr">
+        <is>
+          <t>2025-07-01</t>
+        </is>
+      </c>
+      <c r="K167" t="inlineStr">
+        <is>
+          <t>2025-11-02</t>
+        </is>
+      </c>
+      <c r="L167" t="inlineStr">
+        <is>
+          <t>2025-11-07</t>
+        </is>
+      </c>
+      <c r="M167" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="O167" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>ecai</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>ECAI</t>
+        </is>
+      </c>
+      <c r="C168" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D168" t="n">
+        <v>1</v>
+      </c>
+      <c r="E168" t="inlineStr">
+        <is>
+          <t>2025-05-06</t>
+        </is>
+      </c>
+      <c r="I168" t="inlineStr">
+        <is>
+          <t>2025-06-15</t>
+        </is>
+      </c>
+      <c r="K168" t="inlineStr">
+        <is>
+          <t>2025-10-25</t>
+        </is>
+      </c>
+      <c r="L168" t="inlineStr">
+        <is>
+          <t>2025-10-30</t>
+        </is>
+      </c>
+      <c r="M168" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="O168" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>siggraph</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>SIGGRAPH</t>
+        </is>
+      </c>
+      <c r="C169" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D169" t="n">
+        <v>1</v>
+      </c>
+      <c r="E169" t="inlineStr">
+        <is>
+          <t>2025-02-18</t>
+        </is>
+      </c>
+      <c r="I169" t="inlineStr">
+        <is>
+          <t>2025-05-01</t>
+        </is>
+      </c>
+      <c r="K169" t="inlineStr">
+        <is>
+          <t>2025-08-10</t>
+        </is>
+      </c>
+      <c r="L169" t="inlineStr">
+        <is>
+          <t>2025-08-14</t>
+        </is>
+      </c>
+      <c r="M169" t="inlineStr">
+        <is>
+          <t>Vancouver, Canada</t>
+        </is>
+      </c>
+      <c r="N169" t="inlineStr">
+        <is>
+          <t>https://s2025.siggraph.org/</t>
+        </is>
+      </c>
+      <c r="O169" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>icwsm</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>ICWSM</t>
+        </is>
+      </c>
+      <c r="C170" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D170" t="n">
+        <v>1</v>
+      </c>
+      <c r="E170" t="inlineStr">
+        <is>
+          <t>2025-01-15</t>
+        </is>
+      </c>
+      <c r="I170" t="inlineStr">
+        <is>
+          <t>2025-03-15</t>
+        </is>
+      </c>
+      <c r="K170" t="inlineStr">
+        <is>
+          <t>2025-06-23</t>
+        </is>
+      </c>
+      <c r="L170" t="inlineStr">
+        <is>
+          <t>2025-06-26</t>
+        </is>
+      </c>
+      <c r="M170" t="inlineStr">
+        <is>
+          <t>Copenhagen, Denmark</t>
+        </is>
+      </c>
+      <c r="N170" t="inlineStr">
+        <is>
+          <t>https://www.icwsm.org/2025/</t>
+        </is>
+      </c>
+      <c r="O170" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>icwsm</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>ICWSM</t>
+        </is>
+      </c>
+      <c r="C171" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D171" t="n">
+        <v>1</v>
+      </c>
+      <c r="E171" t="inlineStr">
+        <is>
+          <t>2025-05-15</t>
+        </is>
+      </c>
+      <c r="I171" t="inlineStr">
+        <is>
+          <t>2025-07-15</t>
+        </is>
+      </c>
+      <c r="K171" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="L171" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="M171" t="inlineStr">
+        <is>
+          <t>Los Angeles, CA, USA</t>
+        </is>
+      </c>
+      <c r="N171" t="inlineStr">
+        <is>
+          <t>https://www.icwsm.org/2026/</t>
+        </is>
+      </c>
+      <c r="O171" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>icwsm</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>ICWSM</t>
+        </is>
+      </c>
+      <c r="C172" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D172" t="n">
+        <v>2</v>
+      </c>
+      <c r="E172" t="inlineStr">
+        <is>
+          <t>2025-09-15</t>
+        </is>
+      </c>
+      <c r="I172" t="inlineStr">
+        <is>
+          <t>2025-11-15</t>
+        </is>
+      </c>
+      <c r="K172" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="L172" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="M172" t="inlineStr">
+        <is>
+          <t>Los Angeles, CA, USA</t>
+        </is>
+      </c>
+      <c r="N172" t="inlineStr">
+        <is>
+          <t>https://www.icwsm.org/2026/</t>
+        </is>
+      </c>
+      <c r="O172" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:R72"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add FAST 2027 (2 cycles), fix TCC 2026 from official site
</commit_message>
<xml_diff>
--- a/timeline_data.xlsx
+++ b/timeline_data.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R171"/>
+  <dimension ref="A1:R173"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -10226,6 +10226,142 @@
         </is>
       </c>
     </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>fast</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>FAST</t>
+        </is>
+      </c>
+      <c r="C172" t="n">
+        <v>2027</v>
+      </c>
+      <c r="D172" t="n">
+        <v>1</v>
+      </c>
+      <c r="E172" t="inlineStr">
+        <is>
+          <t>2026-03-17</t>
+        </is>
+      </c>
+      <c r="G172" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="H172" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="I172" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="J172" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="K172" t="inlineStr">
+        <is>
+          <t>2027-02-23</t>
+        </is>
+      </c>
+      <c r="L172" t="inlineStr">
+        <is>
+          <t>2027-02-25</t>
+        </is>
+      </c>
+      <c r="M172" t="inlineStr">
+        <is>
+          <t>Renton, WA, USA</t>
+        </is>
+      </c>
+      <c r="N172" t="inlineStr">
+        <is>
+          <t>https://www.usenix.org/conference/fast27/</t>
+        </is>
+      </c>
+      <c r="O172" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>fast</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>FAST</t>
+        </is>
+      </c>
+      <c r="C173" t="n">
+        <v>2027</v>
+      </c>
+      <c r="D173" t="n">
+        <v>2</v>
+      </c>
+      <c r="E173" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="G173" t="inlineStr">
+        <is>
+          <t>2026-11-17</t>
+        </is>
+      </c>
+      <c r="H173" t="inlineStr">
+        <is>
+          <t>2026-11-19</t>
+        </is>
+      </c>
+      <c r="I173" t="inlineStr">
+        <is>
+          <t>2026-12-08</t>
+        </is>
+      </c>
+      <c r="J173" t="inlineStr">
+        <is>
+          <t>2027-01-26</t>
+        </is>
+      </c>
+      <c r="K173" t="inlineStr">
+        <is>
+          <t>2027-02-23</t>
+        </is>
+      </c>
+      <c r="L173" t="inlineStr">
+        <is>
+          <t>2027-02-25</t>
+        </is>
+      </c>
+      <c r="M173" t="inlineStr">
+        <is>
+          <t>Renton, WA, USA</t>
+        </is>
+      </c>
+      <c r="N173" t="inlineStr">
+        <is>
+          <t>https://www.usenix.org/conference/fast27/</t>
+        </is>
+      </c>
+      <c r="O173" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:R72"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add WSDM 2026, ICRA 2027, SODA 2026/2027, ACM MM 2026, ICSE 2027
</commit_message>
<xml_diff>
--- a/timeline_data.xlsx
+++ b/timeline_data.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R173"/>
+  <dimension ref="A1:R179"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -10362,6 +10362,339 @@
         </is>
       </c>
     </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>wsdm</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>WSDM</t>
+        </is>
+      </c>
+      <c r="C174" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D174" t="n">
+        <v>1</v>
+      </c>
+      <c r="E174" t="inlineStr">
+        <is>
+          <t>2025-09-25</t>
+        </is>
+      </c>
+      <c r="I174" t="inlineStr">
+        <is>
+          <t>2025-11-27</t>
+        </is>
+      </c>
+      <c r="K174" t="inlineStr">
+        <is>
+          <t>2026-02-22</t>
+        </is>
+      </c>
+      <c r="L174" t="inlineStr">
+        <is>
+          <t>2026-02-26</t>
+        </is>
+      </c>
+      <c r="M174" t="inlineStr">
+        <is>
+          <t>Boise, ID, USA</t>
+        </is>
+      </c>
+      <c r="N174" t="inlineStr">
+        <is>
+          <t>https://wsdm-conference.org/2026/</t>
+        </is>
+      </c>
+      <c r="O174" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>icra</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>ICRA</t>
+        </is>
+      </c>
+      <c r="C175" t="n">
+        <v>2027</v>
+      </c>
+      <c r="D175" t="n">
+        <v>1</v>
+      </c>
+      <c r="E175" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="I175" t="inlineStr">
+        <is>
+          <t>2027-01-31</t>
+        </is>
+      </c>
+      <c r="K175" t="inlineStr">
+        <is>
+          <t>2027-05-24</t>
+        </is>
+      </c>
+      <c r="L175" t="inlineStr">
+        <is>
+          <t>2027-05-28</t>
+        </is>
+      </c>
+      <c r="M175" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="O175" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>soda</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>SODA</t>
+        </is>
+      </c>
+      <c r="C176" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D176" t="n">
+        <v>1</v>
+      </c>
+      <c r="E176" t="inlineStr">
+        <is>
+          <t>2025-07-14</t>
+        </is>
+      </c>
+      <c r="I176" t="inlineStr">
+        <is>
+          <t>2025-10-01</t>
+        </is>
+      </c>
+      <c r="K176" t="inlineStr">
+        <is>
+          <t>2026-01-11</t>
+        </is>
+      </c>
+      <c r="L176" t="inlineStr">
+        <is>
+          <t>2026-01-14</t>
+        </is>
+      </c>
+      <c r="M176" t="inlineStr">
+        <is>
+          <t>Vancouver, Canada</t>
+        </is>
+      </c>
+      <c r="N176" t="inlineStr">
+        <is>
+          <t>https://www.siam.org/conferences-events/siam-conferences/soda26/</t>
+        </is>
+      </c>
+      <c r="O176" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>soda</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>SODA</t>
+        </is>
+      </c>
+      <c r="C177" t="n">
+        <v>2027</v>
+      </c>
+      <c r="D177" t="n">
+        <v>1</v>
+      </c>
+      <c r="E177" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="I177" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="K177" t="inlineStr">
+        <is>
+          <t>2027-01-24</t>
+        </is>
+      </c>
+      <c r="L177" t="inlineStr">
+        <is>
+          <t>2027-01-27</t>
+        </is>
+      </c>
+      <c r="M177" t="inlineStr">
+        <is>
+          <t>Philadelphia, PA, USA</t>
+        </is>
+      </c>
+      <c r="N177" t="inlineStr">
+        <is>
+          <t>https://www.siam.org/conferences-events/siam-conferences/soda27/</t>
+        </is>
+      </c>
+      <c r="O177" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>acm-mm</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>ACM MM</t>
+        </is>
+      </c>
+      <c r="C178" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D178" t="n">
+        <v>1</v>
+      </c>
+      <c r="E178" t="inlineStr">
+        <is>
+          <t>2026-04-01</t>
+        </is>
+      </c>
+      <c r="I178" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="J178" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="K178" t="inlineStr">
+        <is>
+          <t>2026-11-10</t>
+        </is>
+      </c>
+      <c r="L178" t="inlineStr">
+        <is>
+          <t>2026-11-14</t>
+        </is>
+      </c>
+      <c r="M178" t="inlineStr">
+        <is>
+          <t>Rio de Janeiro, Brazil</t>
+        </is>
+      </c>
+      <c r="N178" t="inlineStr">
+        <is>
+          <t>https://acmmm.org/</t>
+        </is>
+      </c>
+      <c r="O178" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>icse</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>ICSE</t>
+        </is>
+      </c>
+      <c r="C179" t="n">
+        <v>2027</v>
+      </c>
+      <c r="D179" t="n">
+        <v>1</v>
+      </c>
+      <c r="E179" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="G179" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="H179" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="I179" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="J179" t="inlineStr">
+        <is>
+          <t>2026-11-24</t>
+        </is>
+      </c>
+      <c r="K179" t="inlineStr">
+        <is>
+          <t>2027-04-25</t>
+        </is>
+      </c>
+      <c r="L179" t="inlineStr">
+        <is>
+          <t>2027-05-01</t>
+        </is>
+      </c>
+      <c r="M179" t="inlineStr">
+        <is>
+          <t>Dublin, Ireland</t>
+        </is>
+      </c>
+      <c r="N179" t="inlineStr">
+        <is>
+          <t>https://conf.researchr.org/home/icse-2027</t>
+        </is>
+      </c>
+      <c r="O179" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:R72"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add ESORICS 2026 (2x), CHI 2027
</commit_message>
<xml_diff>
--- a/timeline_data.xlsx
+++ b/timeline_data.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R179"/>
+  <dimension ref="A1:R182"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -10695,6 +10695,180 @@
         </is>
       </c>
     </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>esorics</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>ESORICS</t>
+        </is>
+      </c>
+      <c r="C180" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D180" t="n">
+        <v>1</v>
+      </c>
+      <c r="E180" t="inlineStr">
+        <is>
+          <t>2026-01-09</t>
+        </is>
+      </c>
+      <c r="I180" t="inlineStr">
+        <is>
+          <t>2026-03-10</t>
+        </is>
+      </c>
+      <c r="J180" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="K180" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="L180" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="M180" t="inlineStr">
+        <is>
+          <t>Rome, Italy</t>
+        </is>
+      </c>
+      <c r="N180" t="inlineStr">
+        <is>
+          <t>https://esorics2026.org/</t>
+        </is>
+      </c>
+      <c r="O180" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>esorics</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>ESORICS</t>
+        </is>
+      </c>
+      <c r="C181" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D181" t="n">
+        <v>2</v>
+      </c>
+      <c r="E181" t="inlineStr">
+        <is>
+          <t>2026-04-21</t>
+        </is>
+      </c>
+      <c r="I181" t="inlineStr">
+        <is>
+          <t>2026-06-12</t>
+        </is>
+      </c>
+      <c r="J181" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="K181" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="L181" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="M181" t="inlineStr">
+        <is>
+          <t>Rome, Italy</t>
+        </is>
+      </c>
+      <c r="N181" t="inlineStr">
+        <is>
+          <t>https://esorics2026.org/</t>
+        </is>
+      </c>
+      <c r="O181" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>chi</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>CHI</t>
+        </is>
+      </c>
+      <c r="C182" t="n">
+        <v>2027</v>
+      </c>
+      <c r="D182" t="n">
+        <v>1</v>
+      </c>
+      <c r="E182" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="I182" t="inlineStr">
+        <is>
+          <t>2026-12-17</t>
+        </is>
+      </c>
+      <c r="J182" t="inlineStr">
+        <is>
+          <t>2027-02-18</t>
+        </is>
+      </c>
+      <c r="K182" t="inlineStr">
+        <is>
+          <t>2027-04-29</t>
+        </is>
+      </c>
+      <c r="L182" t="inlineStr">
+        <is>
+          <t>2027-05-04</t>
+        </is>
+      </c>
+      <c r="M182" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="N182" t="inlineStr">
+        <is>
+          <t>https://chi2027.acm.org/</t>
+        </is>
+      </c>
+      <c r="O182" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:R72"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add HPCA 2026, SIGMOD 2027 (4 rounds)
</commit_message>
<xml_diff>
--- a/timeline_data.xlsx
+++ b/timeline_data.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R182"/>
+  <dimension ref="A1:R187"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -10869,6 +10869,326 @@
         </is>
       </c>
     </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>hpca</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>HPCA</t>
+        </is>
+      </c>
+      <c r="C183" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D183" t="n">
+        <v>1</v>
+      </c>
+      <c r="E183" t="inlineStr">
+        <is>
+          <t>2025-08-01</t>
+        </is>
+      </c>
+      <c r="G183" t="inlineStr">
+        <is>
+          <t>2025-10-07</t>
+        </is>
+      </c>
+      <c r="H183" t="inlineStr">
+        <is>
+          <t>2025-10-20</t>
+        </is>
+      </c>
+      <c r="I183" t="inlineStr">
+        <is>
+          <t>2025-11-07</t>
+        </is>
+      </c>
+      <c r="J183" t="inlineStr">
+        <is>
+          <t>2025-12-04</t>
+        </is>
+      </c>
+      <c r="K183" t="inlineStr">
+        <is>
+          <t>2026-02-25</t>
+        </is>
+      </c>
+      <c r="L183" t="inlineStr">
+        <is>
+          <t>2026-03-01</t>
+        </is>
+      </c>
+      <c r="M183" t="inlineStr">
+        <is>
+          <t>Sydney, Australia</t>
+        </is>
+      </c>
+      <c r="N183" t="inlineStr">
+        <is>
+          <t>https://hpca-conf.org/</t>
+        </is>
+      </c>
+      <c r="O183" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>sigmod</t>
+        </is>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>SIGMOD</t>
+        </is>
+      </c>
+      <c r="C184" t="n">
+        <v>2027</v>
+      </c>
+      <c r="D184" t="n">
+        <v>1</v>
+      </c>
+      <c r="E184" t="inlineStr">
+        <is>
+          <t>2026-01-17</t>
+        </is>
+      </c>
+      <c r="G184" t="inlineStr">
+        <is>
+          <t>2026-03-10</t>
+        </is>
+      </c>
+      <c r="H184" t="inlineStr">
+        <is>
+          <t>2026-03-17</t>
+        </is>
+      </c>
+      <c r="I184" t="inlineStr">
+        <is>
+          <t>2026-04-19</t>
+        </is>
+      </c>
+      <c r="K184" t="inlineStr">
+        <is>
+          <t>2027-06-13</t>
+        </is>
+      </c>
+      <c r="L184" t="inlineStr">
+        <is>
+          <t>2027-06-19</t>
+        </is>
+      </c>
+      <c r="M184" t="inlineStr">
+        <is>
+          <t>Huntington Beach, CA, USA</t>
+        </is>
+      </c>
+      <c r="N184" t="inlineStr">
+        <is>
+          <t>https://2027.sigmod.org/</t>
+        </is>
+      </c>
+      <c r="O184" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>sigmod</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>SIGMOD</t>
+        </is>
+      </c>
+      <c r="C185" t="n">
+        <v>2027</v>
+      </c>
+      <c r="D185" t="n">
+        <v>2</v>
+      </c>
+      <c r="E185" t="inlineStr">
+        <is>
+          <t>2026-04-17</t>
+        </is>
+      </c>
+      <c r="G185" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="H185" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+      <c r="I185" t="inlineStr">
+        <is>
+          <t>2026-07-19</t>
+        </is>
+      </c>
+      <c r="K185" t="inlineStr">
+        <is>
+          <t>2027-06-13</t>
+        </is>
+      </c>
+      <c r="L185" t="inlineStr">
+        <is>
+          <t>2027-06-19</t>
+        </is>
+      </c>
+      <c r="M185" t="inlineStr">
+        <is>
+          <t>Huntington Beach, CA, USA</t>
+        </is>
+      </c>
+      <c r="N185" t="inlineStr">
+        <is>
+          <t>https://2027.sigmod.org/</t>
+        </is>
+      </c>
+      <c r="O185" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>sigmod</t>
+        </is>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>SIGMOD</t>
+        </is>
+      </c>
+      <c r="C186" t="n">
+        <v>2027</v>
+      </c>
+      <c r="D186" t="n">
+        <v>3</v>
+      </c>
+      <c r="E186" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="G186" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="H186" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="I186" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="K186" t="inlineStr">
+        <is>
+          <t>2027-06-13</t>
+        </is>
+      </c>
+      <c r="L186" t="inlineStr">
+        <is>
+          <t>2027-06-19</t>
+        </is>
+      </c>
+      <c r="M186" t="inlineStr">
+        <is>
+          <t>Huntington Beach, CA, USA</t>
+        </is>
+      </c>
+      <c r="N186" t="inlineStr">
+        <is>
+          <t>https://2027.sigmod.org/</t>
+        </is>
+      </c>
+      <c r="O186" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>sigmod</t>
+        </is>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>SIGMOD</t>
+        </is>
+      </c>
+      <c r="C187" t="n">
+        <v>2027</v>
+      </c>
+      <c r="D187" t="n">
+        <v>4</v>
+      </c>
+      <c r="E187" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="G187" t="inlineStr">
+        <is>
+          <t>2026-12-10</t>
+        </is>
+      </c>
+      <c r="H187" t="inlineStr">
+        <is>
+          <t>2026-12-17</t>
+        </is>
+      </c>
+      <c r="I187" t="inlineStr">
+        <is>
+          <t>2027-01-19</t>
+        </is>
+      </c>
+      <c r="K187" t="inlineStr">
+        <is>
+          <t>2027-06-13</t>
+        </is>
+      </c>
+      <c r="L187" t="inlineStr">
+        <is>
+          <t>2027-06-19</t>
+        </is>
+      </c>
+      <c r="M187" t="inlineStr">
+        <is>
+          <t>Huntington Beach, CA, USA</t>
+        </is>
+      </c>
+      <c r="N187" t="inlineStr">
+        <is>
+          <t>https://2027.sigmod.org/</t>
+        </is>
+      </c>
+      <c r="O187" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:R72"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add VLDB 2027, EuroSys 2027 (2x)
</commit_message>
<xml_diff>
--- a/timeline_data.xlsx
+++ b/timeline_data.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R187"/>
+  <dimension ref="A1:R190"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -11189,6 +11189,170 @@
         </is>
       </c>
     </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>vldb</t>
+        </is>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>VLDB</t>
+        </is>
+      </c>
+      <c r="C188" t="n">
+        <v>2027</v>
+      </c>
+      <c r="D188" t="n">
+        <v>1</v>
+      </c>
+      <c r="E188" t="inlineStr">
+        <is>
+          <t>2026-03-01</t>
+        </is>
+      </c>
+      <c r="I188" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="K188" t="inlineStr">
+        <is>
+          <t>2027-08-23</t>
+        </is>
+      </c>
+      <c r="L188" t="inlineStr">
+        <is>
+          <t>2027-08-27</t>
+        </is>
+      </c>
+      <c r="M188" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="N188" t="inlineStr">
+        <is>
+          <t>https://vldb.org/2027/</t>
+        </is>
+      </c>
+      <c r="O188" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>eurosys</t>
+        </is>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>EuroSys</t>
+        </is>
+      </c>
+      <c r="C189" t="n">
+        <v>2027</v>
+      </c>
+      <c r="D189" t="n">
+        <v>1</v>
+      </c>
+      <c r="E189" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="I189" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="K189" t="inlineStr">
+        <is>
+          <t>2027-04-19</t>
+        </is>
+      </c>
+      <c r="L189" t="inlineStr">
+        <is>
+          <t>2027-04-23</t>
+        </is>
+      </c>
+      <c r="M189" t="inlineStr">
+        <is>
+          <t>Rabat, Morocco</t>
+        </is>
+      </c>
+      <c r="N189" t="inlineStr">
+        <is>
+          <t>https://2027.eurosys.org/</t>
+        </is>
+      </c>
+      <c r="O189" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>eurosys</t>
+        </is>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>EuroSys</t>
+        </is>
+      </c>
+      <c r="C190" t="n">
+        <v>2027</v>
+      </c>
+      <c r="D190" t="n">
+        <v>2</v>
+      </c>
+      <c r="E190" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="I190" t="inlineStr">
+        <is>
+          <t>2027-01-29</t>
+        </is>
+      </c>
+      <c r="J190" t="inlineStr">
+        <is>
+          <t>2027-03-05</t>
+        </is>
+      </c>
+      <c r="K190" t="inlineStr">
+        <is>
+          <t>2027-04-19</t>
+        </is>
+      </c>
+      <c r="L190" t="inlineStr">
+        <is>
+          <t>2027-04-23</t>
+        </is>
+      </c>
+      <c r="M190" t="inlineStr">
+        <is>
+          <t>Rabat, Morocco</t>
+        </is>
+      </c>
+      <c r="N190" t="inlineStr">
+        <is>
+          <t>https://2027.eurosys.org/</t>
+        </is>
+      </c>
+      <c r="O190" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:R72"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add DAC 2026, ICMR 2026, SenSys 2026, INFOCOM 2026, ICNP 2026
</commit_message>
<xml_diff>
--- a/timeline_data.xlsx
+++ b/timeline_data.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R190"/>
+  <dimension ref="A1:R195"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -11353,6 +11353,266 @@
         </is>
       </c>
     </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>dac</t>
+        </is>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>DAC</t>
+        </is>
+      </c>
+      <c r="C191" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D191" t="n">
+        <v>1</v>
+      </c>
+      <c r="E191" t="inlineStr">
+        <is>
+          <t>2025-11-11</t>
+        </is>
+      </c>
+      <c r="I191" t="inlineStr">
+        <is>
+          <t>2026-02-01</t>
+        </is>
+      </c>
+      <c r="K191" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="L191" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="M191" t="inlineStr">
+        <is>
+          <t>Long Beach, CA, USA</t>
+        </is>
+      </c>
+      <c r="N191" t="inlineStr">
+        <is>
+          <t>https://dac.com/2026</t>
+        </is>
+      </c>
+      <c r="O191" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>icmr</t>
+        </is>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>ICMR</t>
+        </is>
+      </c>
+      <c r="C192" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D192" t="n">
+        <v>1</v>
+      </c>
+      <c r="E192" t="inlineStr">
+        <is>
+          <t>2026-02-06</t>
+        </is>
+      </c>
+      <c r="I192" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="J192" t="inlineStr">
+        <is>
+          <t>2026-04-25</t>
+        </is>
+      </c>
+      <c r="K192" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+      <c r="L192" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="M192" t="inlineStr">
+        <is>
+          <t>Amsterdam, Netherlands</t>
+        </is>
+      </c>
+      <c r="N192" t="inlineStr">
+        <is>
+          <t>https://www.acmicmr.org/</t>
+        </is>
+      </c>
+      <c r="O192" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>sensys</t>
+        </is>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>SenSys</t>
+        </is>
+      </c>
+      <c r="C193" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D193" t="n">
+        <v>1</v>
+      </c>
+      <c r="E193" t="inlineStr">
+        <is>
+          <t>2025-11-06</t>
+        </is>
+      </c>
+      <c r="I193" t="inlineStr">
+        <is>
+          <t>2026-01-29</t>
+        </is>
+      </c>
+      <c r="K193" t="inlineStr">
+        <is>
+          <t>2026-05-11</t>
+        </is>
+      </c>
+      <c r="L193" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="M193" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="O193" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>infocom</t>
+        </is>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>INFOCOM</t>
+        </is>
+      </c>
+      <c r="C194" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D194" t="n">
+        <v>1</v>
+      </c>
+      <c r="E194" t="inlineStr">
+        <is>
+          <t>2025-07-24</t>
+        </is>
+      </c>
+      <c r="I194" t="inlineStr">
+        <is>
+          <t>2025-12-08</t>
+        </is>
+      </c>
+      <c r="K194" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="L194" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="M194" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="N194" t="inlineStr">
+        <is>
+          <t>https://infocom2026.ieee-infocom.org/</t>
+        </is>
+      </c>
+      <c r="O194" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>icnp</t>
+        </is>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>ICNP</t>
+        </is>
+      </c>
+      <c r="C195" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D195" t="n">
+        <v>1</v>
+      </c>
+      <c r="E195" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="I195" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="K195" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="L195" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="M195" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="O195" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:R72"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add ICDM 2026, CIKM 2026, SDM 2026, ICDE 2027(2x), MobiSys 2026, CCC 2026
</commit_message>
<xml_diff>
--- a/timeline_data.xlsx
+++ b/timeline_data.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R195"/>
+  <dimension ref="A1:R202"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -11613,6 +11613,402 @@
         </is>
       </c>
     </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>icdm</t>
+        </is>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>ICDM</t>
+        </is>
+      </c>
+      <c r="C196" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D196" t="n">
+        <v>1</v>
+      </c>
+      <c r="E196" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="I196" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="K196" t="inlineStr">
+        <is>
+          <t>2026-11-12</t>
+        </is>
+      </c>
+      <c r="L196" t="inlineStr">
+        <is>
+          <t>2026-11-15</t>
+        </is>
+      </c>
+      <c r="M196" t="inlineStr">
+        <is>
+          <t>Shenyang, China</t>
+        </is>
+      </c>
+      <c r="O196" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>cikm</t>
+        </is>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>CIKM</t>
+        </is>
+      </c>
+      <c r="C197" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D197" t="n">
+        <v>1</v>
+      </c>
+      <c r="E197" t="inlineStr">
+        <is>
+          <t>2026-05-23</t>
+        </is>
+      </c>
+      <c r="I197" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="K197" t="inlineStr">
+        <is>
+          <t>2026-11-07</t>
+        </is>
+      </c>
+      <c r="L197" t="inlineStr">
+        <is>
+          <t>2026-11-11</t>
+        </is>
+      </c>
+      <c r="M197" t="inlineStr">
+        <is>
+          <t>Rome, Italy</t>
+        </is>
+      </c>
+      <c r="O197" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>sdm</t>
+        </is>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>SDM</t>
+        </is>
+      </c>
+      <c r="C198" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D198" t="n">
+        <v>1</v>
+      </c>
+      <c r="E198" t="inlineStr">
+        <is>
+          <t>2026-04-10</t>
+        </is>
+      </c>
+      <c r="I198" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="K198" t="inlineStr">
+        <is>
+          <t>2026-11-19</t>
+        </is>
+      </c>
+      <c r="L198" t="inlineStr">
+        <is>
+          <t>2026-11-21</t>
+        </is>
+      </c>
+      <c r="M198" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="O198" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>icde</t>
+        </is>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>ICDE</t>
+        </is>
+      </c>
+      <c r="C199" t="n">
+        <v>2027</v>
+      </c>
+      <c r="D199" t="n">
+        <v>1</v>
+      </c>
+      <c r="E199" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="G199" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="H199" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="I199" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="J199" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="K199" t="inlineStr">
+        <is>
+          <t>2027-05-17</t>
+        </is>
+      </c>
+      <c r="L199" t="inlineStr">
+        <is>
+          <t>2027-05-21</t>
+        </is>
+      </c>
+      <c r="M199" t="inlineStr">
+        <is>
+          <t>Copenhagen, Denmark</t>
+        </is>
+      </c>
+      <c r="N199" t="inlineStr">
+        <is>
+          <t>https://icde2027.github.io/</t>
+        </is>
+      </c>
+      <c r="O199" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>icde</t>
+        </is>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>ICDE</t>
+        </is>
+      </c>
+      <c r="C200" t="n">
+        <v>2027</v>
+      </c>
+      <c r="D200" t="n">
+        <v>2</v>
+      </c>
+      <c r="E200" t="inlineStr">
+        <is>
+          <t>2026-11-11</t>
+        </is>
+      </c>
+      <c r="G200" t="inlineStr">
+        <is>
+          <t>2027-01-08</t>
+        </is>
+      </c>
+      <c r="H200" t="inlineStr">
+        <is>
+          <t>2027-01-15</t>
+        </is>
+      </c>
+      <c r="I200" t="inlineStr">
+        <is>
+          <t>2027-02-10</t>
+        </is>
+      </c>
+      <c r="J200" t="inlineStr">
+        <is>
+          <t>2027-03-10</t>
+        </is>
+      </c>
+      <c r="K200" t="inlineStr">
+        <is>
+          <t>2027-05-17</t>
+        </is>
+      </c>
+      <c r="L200" t="inlineStr">
+        <is>
+          <t>2027-05-21</t>
+        </is>
+      </c>
+      <c r="M200" t="inlineStr">
+        <is>
+          <t>Copenhagen, Denmark</t>
+        </is>
+      </c>
+      <c r="N200" t="inlineStr">
+        <is>
+          <t>https://icde2027.github.io/</t>
+        </is>
+      </c>
+      <c r="O200" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>mobisys</t>
+        </is>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>MobiSys</t>
+        </is>
+      </c>
+      <c r="C201" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D201" t="n">
+        <v>1</v>
+      </c>
+      <c r="E201" t="inlineStr">
+        <is>
+          <t>2025-12-05</t>
+        </is>
+      </c>
+      <c r="G201" t="inlineStr">
+        <is>
+          <t>2026-02-09</t>
+        </is>
+      </c>
+      <c r="H201" t="inlineStr">
+        <is>
+          <t>2026-02-13</t>
+        </is>
+      </c>
+      <c r="I201" t="inlineStr">
+        <is>
+          <t>2026-03-02</t>
+        </is>
+      </c>
+      <c r="J201" t="inlineStr">
+        <is>
+          <t>2026-04-13</t>
+        </is>
+      </c>
+      <c r="K201" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="L201" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="M201" t="inlineStr">
+        <is>
+          <t>Cambridge, UK</t>
+        </is>
+      </c>
+      <c r="N201" t="inlineStr">
+        <is>
+          <t>https://www.sigmobile.org/mobisys/2026/</t>
+        </is>
+      </c>
+      <c r="O201" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>ccc</t>
+        </is>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>CCC</t>
+        </is>
+      </c>
+      <c r="C202" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D202" t="n">
+        <v>1</v>
+      </c>
+      <c r="E202" t="inlineStr">
+        <is>
+          <t>2026-02-06</t>
+        </is>
+      </c>
+      <c r="I202" t="inlineStr">
+        <is>
+          <t>2026-04-01</t>
+        </is>
+      </c>
+      <c r="K202" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="L202" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="M202" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="O202" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:R72"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add SC 2026, ICALP 2026, RecSys 2026, WSDM 2027
</commit_message>
<xml_diff>
--- a/timeline_data.xlsx
+++ b/timeline_data.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R202"/>
+  <dimension ref="A1:R206"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -12009,6 +12009,248 @@
         </is>
       </c>
     </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>sc</t>
+        </is>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+      <c r="C203" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D203" t="n">
+        <v>1</v>
+      </c>
+      <c r="E203" t="inlineStr">
+        <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="I203" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="K203" t="inlineStr">
+        <is>
+          <t>2026-11-15</t>
+        </is>
+      </c>
+      <c r="L203" t="inlineStr">
+        <is>
+          <t>2026-11-20</t>
+        </is>
+      </c>
+      <c r="M203" t="inlineStr">
+        <is>
+          <t>Chicago, IL, USA</t>
+        </is>
+      </c>
+      <c r="N203" t="inlineStr">
+        <is>
+          <t>https://sc24.supercomputing.org/</t>
+        </is>
+      </c>
+      <c r="O203" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>icalp</t>
+        </is>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>ICALP</t>
+        </is>
+      </c>
+      <c r="C204" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D204" t="n">
+        <v>1</v>
+      </c>
+      <c r="E204" t="inlineStr">
+        <is>
+          <t>2026-02-06</t>
+        </is>
+      </c>
+      <c r="G204" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="H204" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="I204" t="inlineStr">
+        <is>
+          <t>2026-04-20</t>
+        </is>
+      </c>
+      <c r="J204" t="inlineStr">
+        <is>
+          <t>2026-05-11</t>
+        </is>
+      </c>
+      <c r="K204" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="L204" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="M204" t="inlineStr">
+        <is>
+          <t>London, UK</t>
+        </is>
+      </c>
+      <c r="N204" t="inlineStr">
+        <is>
+          <t>https://icalppodcspaa2026.cs.rhul.ac.uk/</t>
+        </is>
+      </c>
+      <c r="O204" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>recsys</t>
+        </is>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>RecSys</t>
+        </is>
+      </c>
+      <c r="C205" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D205" t="n">
+        <v>1</v>
+      </c>
+      <c r="E205" t="inlineStr">
+        <is>
+          <t>2026-04-21</t>
+        </is>
+      </c>
+      <c r="G205" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="H205" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="I205" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="J205" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="K205" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="L205" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="M205" t="inlineStr">
+        <is>
+          <t>Minneapolis, MN, USA</t>
+        </is>
+      </c>
+      <c r="N205" t="inlineStr">
+        <is>
+          <t>https://recsys.acm.org/recsys26/</t>
+        </is>
+      </c>
+      <c r="O205" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="inlineStr">
+        <is>
+          <t>wsdm</t>
+        </is>
+      </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>WSDM</t>
+        </is>
+      </c>
+      <c r="C206" t="n">
+        <v>2027</v>
+      </c>
+      <c r="D206" t="n">
+        <v>1</v>
+      </c>
+      <c r="E206" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="I206" t="inlineStr">
+        <is>
+          <t>2026-11-01</t>
+        </is>
+      </c>
+      <c r="K206" t="inlineStr">
+        <is>
+          <t>2027-02-15</t>
+        </is>
+      </c>
+      <c r="L206" t="inlineStr">
+        <is>
+          <t>2027-02-19</t>
+        </is>
+      </c>
+      <c r="M206" t="inlineStr">
+        <is>
+          <t>Hong Kong, China</t>
+        </is>
+      </c>
+      <c r="N206" t="inlineStr">
+        <is>
+          <t>https://wsdm-conference.org/</t>
+        </is>
+      </c>
+      <c r="O206" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:R72"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update SC 2026 with accurate dates from official site
</commit_message>
<xml_diff>
--- a/timeline_data.xlsx
+++ b/timeline_data.xlsx
@@ -12012,12 +12012,12 @@
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>sc</t>
+          <t>icalp</t>
         </is>
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>SC</t>
+          <t>ICALP</t>
         </is>
       </c>
       <c r="C203" t="n">
@@ -12028,32 +12028,47 @@
       </c>
       <c r="E203" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-02-06</t>
+        </is>
+      </c>
+      <c r="G203" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="H203" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
         </is>
       </c>
       <c r="I203" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-04-20</t>
+        </is>
+      </c>
+      <c r="J203" t="inlineStr">
+        <is>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="K203" t="inlineStr">
         <is>
-          <t>2026-11-15</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="L203" t="inlineStr">
         <is>
-          <t>2026-11-20</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="M203" t="inlineStr">
         <is>
-          <t>Chicago, IL, USA</t>
+          <t>London, UK</t>
         </is>
       </c>
       <c r="N203" t="inlineStr">
         <is>
-          <t>https://sc24.supercomputing.org/</t>
+          <t>https://icalppodcspaa2026.cs.rhul.ac.uk/</t>
         </is>
       </c>
       <c r="O203" t="inlineStr">
@@ -12065,12 +12080,12 @@
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>icalp</t>
+          <t>recsys</t>
         </is>
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>ICALP</t>
+          <t>RecSys</t>
         </is>
       </c>
       <c r="C204" t="n">
@@ -12081,47 +12096,47 @@
       </c>
       <c r="E204" t="inlineStr">
         <is>
-          <t>2026-02-06</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="G204" t="inlineStr">
         <is>
-          <t>2026-03-21</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="H204" t="inlineStr">
         <is>
-          <t>2026-03-24</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="I204" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="J204" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="K204" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="L204" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="M204" t="inlineStr">
         <is>
-          <t>London, UK</t>
+          <t>Minneapolis, MN, USA</t>
         </is>
       </c>
       <c r="N204" t="inlineStr">
         <is>
-          <t>https://icalppodcspaa2026.cs.rhul.ac.uk/</t>
+          <t>https://recsys.acm.org/recsys26/</t>
         </is>
       </c>
       <c r="O204" t="inlineStr">
@@ -12133,63 +12148,48 @@
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>recsys</t>
+          <t>wsdm</t>
         </is>
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>RecSys</t>
+          <t>WSDM</t>
         </is>
       </c>
       <c r="C205" t="n">
-        <v>2026</v>
+        <v>2027</v>
       </c>
       <c r="D205" t="n">
         <v>1</v>
       </c>
       <c r="E205" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
-        </is>
-      </c>
-      <c r="G205" t="inlineStr">
-        <is>
-          <t>2026-06-04</t>
-        </is>
-      </c>
-      <c r="H205" t="inlineStr">
-        <is>
-          <t>2026-06-09</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="I205" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
-        </is>
-      </c>
-      <c r="J205" t="inlineStr">
-        <is>
-          <t>2026-07-27</t>
+          <t>2026-11-01</t>
         </is>
       </c>
       <c r="K205" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2027-02-15</t>
         </is>
       </c>
       <c r="L205" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2027-02-19</t>
         </is>
       </c>
       <c r="M205" t="inlineStr">
         <is>
-          <t>Minneapolis, MN, USA</t>
+          <t>Hong Kong, China</t>
         </is>
       </c>
       <c r="N205" t="inlineStr">
         <is>
-          <t>https://recsys.acm.org/recsys26/</t>
+          <t>https://wsdm-conference.org/</t>
         </is>
       </c>
       <c r="O205" t="inlineStr">
@@ -12201,48 +12201,63 @@
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>wsdm</t>
+          <t>sc</t>
         </is>
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>WSDM</t>
+          <t>SC</t>
         </is>
       </c>
       <c r="C206" t="n">
-        <v>2027</v>
+        <v>2026</v>
       </c>
       <c r="D206" t="n">
         <v>1</v>
       </c>
       <c r="E206" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-04-08</t>
+        </is>
+      </c>
+      <c r="G206" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="H206" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="I206" t="inlineStr">
         <is>
-          <t>2026-11-01</t>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="J206" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="K206" t="inlineStr">
         <is>
-          <t>2027-02-15</t>
+          <t>2026-11-15</t>
         </is>
       </c>
       <c r="L206" t="inlineStr">
         <is>
-          <t>2027-02-19</t>
+          <t>2026-11-20</t>
         </is>
       </c>
       <c r="M206" t="inlineStr">
         <is>
-          <t>Hong Kong, China</t>
+          <t>Chicago, IL, USA</t>
         </is>
       </c>
       <c r="N206" t="inlineStr">
         <is>
-          <t>https://wsdm-conference.org/</t>
+          <t>https://sc24.supercomputing.org/</t>
         </is>
       </c>
       <c r="O206" t="inlineStr">

</xml_diff>

<commit_message>
Add RECOMB, RTSS, CogSci, ECOOP, ISMB 2026
</commit_message>
<xml_diff>
--- a/timeline_data.xlsx
+++ b/timeline_data.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R206"/>
+  <dimension ref="A1:R211"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -12266,6 +12266,281 @@
         </is>
       </c>
     </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t>recomb</t>
+        </is>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>RECOMB</t>
+        </is>
+      </c>
+      <c r="C207" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D207" t="n">
+        <v>1</v>
+      </c>
+      <c r="E207" t="inlineStr">
+        <is>
+          <t>2025-11-20</t>
+        </is>
+      </c>
+      <c r="I207" t="inlineStr">
+        <is>
+          <t>2026-01-16</t>
+        </is>
+      </c>
+      <c r="J207" t="inlineStr">
+        <is>
+          <t>2026-02-25</t>
+        </is>
+      </c>
+      <c r="K207" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+      <c r="L207" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="M207" t="inlineStr">
+        <is>
+          <t>Thessaloniki, Greece</t>
+        </is>
+      </c>
+      <c r="N207" t="inlineStr">
+        <is>
+          <t>http://recomb.org/recomb2026/</t>
+        </is>
+      </c>
+      <c r="O207" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>rtss</t>
+        </is>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>RTSS</t>
+        </is>
+      </c>
+      <c r="C208" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D208" t="n">
+        <v>1</v>
+      </c>
+      <c r="E208" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="I208" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="K208" t="inlineStr">
+        <is>
+          <t>2026-12-01</t>
+        </is>
+      </c>
+      <c r="L208" t="inlineStr">
+        <is>
+          <t>2026-12-04</t>
+        </is>
+      </c>
+      <c r="M208" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="O208" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>cogsci</t>
+        </is>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>CogSci</t>
+        </is>
+      </c>
+      <c r="C209" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D209" t="n">
+        <v>1</v>
+      </c>
+      <c r="E209" t="inlineStr">
+        <is>
+          <t>2026-02-01</t>
+        </is>
+      </c>
+      <c r="I209" t="inlineStr">
+        <is>
+          <t>2026-04-01</t>
+        </is>
+      </c>
+      <c r="K209" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="L209" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="M209" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="O209" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>ecoop</t>
+        </is>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>ECOOP</t>
+        </is>
+      </c>
+      <c r="C210" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D210" t="n">
+        <v>1</v>
+      </c>
+      <c r="E210" t="inlineStr">
+        <is>
+          <t>2026-01-16</t>
+        </is>
+      </c>
+      <c r="G210" t="inlineStr">
+        <is>
+          <t>2026-03-10</t>
+        </is>
+      </c>
+      <c r="H210" t="inlineStr">
+        <is>
+          <t>2026-03-12</t>
+        </is>
+      </c>
+      <c r="I210" t="inlineStr">
+        <is>
+          <t>2026-04-06</t>
+        </is>
+      </c>
+      <c r="J210" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="K210" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="L210" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="M210" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="N210" t="inlineStr">
+        <is>
+          <t>https://2026.ecoop.org/</t>
+        </is>
+      </c>
+      <c r="O210" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
+          <t>ismb</t>
+        </is>
+      </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t>ISMB</t>
+        </is>
+      </c>
+      <c r="C211" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D211" t="n">
+        <v>1</v>
+      </c>
+      <c r="E211" t="inlineStr">
+        <is>
+          <t>2025-12-02</t>
+        </is>
+      </c>
+      <c r="I211" t="inlineStr">
+        <is>
+          <t>2026-02-01</t>
+        </is>
+      </c>
+      <c r="K211" t="inlineStr">
+        <is>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="L211" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="M211" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="N211" t="inlineStr">
+        <is>
+          <t>https://www.iscb.org/ismb2026</t>
+        </is>
+      </c>
+      <c r="O211" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:R72"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add CoNEXT, IMC, MobiHoc, NOSSDAV, SECON, IPSN 2026
</commit_message>
<xml_diff>
--- a/timeline_data.xlsx
+++ b/timeline_data.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R211"/>
+  <dimension ref="A1:R217"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -12541,6 +12541,304 @@
         </is>
       </c>
     </row>
+    <row r="212">
+      <c r="A212" t="inlineStr">
+        <is>
+          <t>conext</t>
+        </is>
+      </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>CoNEXT</t>
+        </is>
+      </c>
+      <c r="C212" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D212" t="n">
+        <v>1</v>
+      </c>
+      <c r="E212" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="I212" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="K212" t="inlineStr">
+        <is>
+          <t>2026-12-07</t>
+        </is>
+      </c>
+      <c r="L212" t="inlineStr">
+        <is>
+          <t>2026-12-10</t>
+        </is>
+      </c>
+      <c r="M212" t="inlineStr">
+        <is>
+          <t>Utrecht, Netherlands</t>
+        </is>
+      </c>
+      <c r="N212" t="inlineStr">
+        <is>
+          <t>https://conferences.sigcomm.org/co-next/2026/</t>
+        </is>
+      </c>
+      <c r="O212" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="inlineStr">
+        <is>
+          <t>imc</t>
+        </is>
+      </c>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t>IMC</t>
+        </is>
+      </c>
+      <c r="C213" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D213" t="n">
+        <v>1</v>
+      </c>
+      <c r="E213" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
+      <c r="I213" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="K213" t="inlineStr">
+        <is>
+          <t>2026-11-03</t>
+        </is>
+      </c>
+      <c r="L213" t="inlineStr">
+        <is>
+          <t>2026-11-05</t>
+        </is>
+      </c>
+      <c r="M213" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="N213" t="inlineStr">
+        <is>
+          <t>https://conferences.sigcomm.org/imc/2026/</t>
+        </is>
+      </c>
+      <c r="O213" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="inlineStr">
+        <is>
+          <t>mobihoc</t>
+        </is>
+      </c>
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>MobiHoc</t>
+        </is>
+      </c>
+      <c r="C214" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D214" t="n">
+        <v>1</v>
+      </c>
+      <c r="E214" t="inlineStr">
+        <is>
+          <t>2026-04-13</t>
+        </is>
+      </c>
+      <c r="I214" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
+      </c>
+      <c r="K214" t="inlineStr">
+        <is>
+          <t>2026-11-23</t>
+        </is>
+      </c>
+      <c r="L214" t="inlineStr">
+        <is>
+          <t>2026-11-25</t>
+        </is>
+      </c>
+      <c r="M214" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="O214" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="inlineStr">
+        <is>
+          <t>nossdav</t>
+        </is>
+      </c>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>NOSSDAV</t>
+        </is>
+      </c>
+      <c r="C215" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D215" t="n">
+        <v>1</v>
+      </c>
+      <c r="E215" t="inlineStr">
+        <is>
+          <t>2026-01-17</t>
+        </is>
+      </c>
+      <c r="I215" t="inlineStr">
+        <is>
+          <t>2026-04-04</t>
+        </is>
+      </c>
+      <c r="K215" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="L215" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="M215" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="O215" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="inlineStr">
+        <is>
+          <t>secon</t>
+        </is>
+      </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>SECON</t>
+        </is>
+      </c>
+      <c r="C216" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D216" t="n">
+        <v>1</v>
+      </c>
+      <c r="E216" t="inlineStr">
+        <is>
+          <t>2025-12-05</t>
+        </is>
+      </c>
+      <c r="I216" t="inlineStr">
+        <is>
+          <t>2026-03-01</t>
+        </is>
+      </c>
+      <c r="K216" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="L216" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="M216" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="O216" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="inlineStr">
+        <is>
+          <t>ipsn</t>
+        </is>
+      </c>
+      <c r="B217" t="inlineStr">
+        <is>
+          <t>IPSN</t>
+        </is>
+      </c>
+      <c r="C217" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D217" t="n">
+        <v>1</v>
+      </c>
+      <c r="E217" t="inlineStr">
+        <is>
+          <t>2025-10-16</t>
+        </is>
+      </c>
+      <c r="I217" t="inlineStr">
+        <is>
+          <t>2026-01-15</t>
+        </is>
+      </c>
+      <c r="K217" t="inlineStr">
+        <is>
+          <t>2026-05-11</t>
+        </is>
+      </c>
+      <c r="L217" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="M217" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="O217" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:R72"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add ICAPS 2026, PPSN 2026, IJCAI 2026
</commit_message>
<xml_diff>
--- a/timeline_data.xlsx
+++ b/timeline_data.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R217"/>
+  <dimension ref="A1:R220"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -12839,6 +12839,170 @@
         </is>
       </c>
     </row>
+    <row r="218">
+      <c r="A218" t="inlineStr">
+        <is>
+          <t>icaps</t>
+        </is>
+      </c>
+      <c r="B218" t="inlineStr">
+        <is>
+          <t>ICAPS</t>
+        </is>
+      </c>
+      <c r="C218" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D218" t="n">
+        <v>1</v>
+      </c>
+      <c r="E218" t="inlineStr">
+        <is>
+          <t>2025-12-08</t>
+        </is>
+      </c>
+      <c r="I218" t="inlineStr">
+        <is>
+          <t>2026-02-20</t>
+        </is>
+      </c>
+      <c r="K218" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="L218" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="M218" t="inlineStr">
+        <is>
+          <t>Dublin, Ireland</t>
+        </is>
+      </c>
+      <c r="N218" t="inlineStr">
+        <is>
+          <t>https://icaps26.icaps-conference.org/</t>
+        </is>
+      </c>
+      <c r="O218" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="inlineStr">
+        <is>
+          <t>ppsn</t>
+        </is>
+      </c>
+      <c r="B219" t="inlineStr">
+        <is>
+          <t>PPSN</t>
+        </is>
+      </c>
+      <c r="C219" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D219" t="n">
+        <v>1</v>
+      </c>
+      <c r="E219" t="inlineStr">
+        <is>
+          <t>2026-03-28</t>
+        </is>
+      </c>
+      <c r="I219" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="J219" t="inlineStr">
+        <is>
+          <t>2026-06-12</t>
+        </is>
+      </c>
+      <c r="K219" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="L219" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="M219" t="inlineStr">
+        <is>
+          <t>Trento, Italy</t>
+        </is>
+      </c>
+      <c r="N219" t="inlineStr">
+        <is>
+          <t>https://ppsn2026.science.unitn.it/</t>
+        </is>
+      </c>
+      <c r="O219" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="inlineStr">
+        <is>
+          <t>ijcai</t>
+        </is>
+      </c>
+      <c r="B220" t="inlineStr">
+        <is>
+          <t>IJCAI</t>
+        </is>
+      </c>
+      <c r="C220" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D220" t="n">
+        <v>1</v>
+      </c>
+      <c r="E220" t="inlineStr">
+        <is>
+          <t>2026-01-21</t>
+        </is>
+      </c>
+      <c r="I220" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="K220" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="L220" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="M220" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="N220" t="inlineStr">
+        <is>
+          <t>https://ijcai-26.org/</t>
+        </is>
+      </c>
+      <c r="O220" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:R72"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add IEEE VIS 2026
</commit_message>
<xml_diff>
--- a/timeline_data.xlsx
+++ b/timeline_data.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R221"/>
+  <dimension ref="A1:R222"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -13071,6 +13071,74 @@
         </is>
       </c>
     </row>
+    <row r="222">
+      <c r="A222" t="inlineStr">
+        <is>
+          <t>ieee-vis</t>
+        </is>
+      </c>
+      <c r="B222" t="inlineStr">
+        <is>
+          <t>IEEE VIS</t>
+        </is>
+      </c>
+      <c r="C222" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D222" t="n">
+        <v>1</v>
+      </c>
+      <c r="E222" t="inlineStr">
+        <is>
+          <t>2026-03-31</t>
+        </is>
+      </c>
+      <c r="G222" t="inlineStr">
+        <is>
+          <t>2026-06-06</t>
+        </is>
+      </c>
+      <c r="H222" t="inlineStr">
+        <is>
+          <t>2026-06-06</t>
+        </is>
+      </c>
+      <c r="I222" t="inlineStr">
+        <is>
+          <t>2026-06-06</t>
+        </is>
+      </c>
+      <c r="J222" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="K222" t="inlineStr">
+        <is>
+          <t>2026-11-09</t>
+        </is>
+      </c>
+      <c r="L222" t="inlineStr">
+        <is>
+          <t>2026-11-13</t>
+        </is>
+      </c>
+      <c r="M222" t="inlineStr">
+        <is>
+          <t>Boston, MA, USA</t>
+        </is>
+      </c>
+      <c r="N222" t="inlineStr">
+        <is>
+          <t>https://ieeevis.org/</t>
+        </is>
+      </c>
+      <c r="O222" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:R72"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add PODS 2026 (cycle 2)
</commit_message>
<xml_diff>
--- a/timeline_data.xlsx
+++ b/timeline_data.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R224"/>
+  <dimension ref="A1:R225"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -13250,6 +13250,69 @@
         </is>
       </c>
     </row>
+    <row r="225">
+      <c r="A225" t="inlineStr">
+        <is>
+          <t>pods</t>
+        </is>
+      </c>
+      <c r="B225" t="inlineStr">
+        <is>
+          <t>PODS</t>
+        </is>
+      </c>
+      <c r="C225" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D225" t="n">
+        <v>1</v>
+      </c>
+      <c r="E225" t="inlineStr">
+        <is>
+          <t>2025-12-10</t>
+        </is>
+      </c>
+      <c r="G225" t="inlineStr">
+        <is>
+          <t>2026-01-26</t>
+        </is>
+      </c>
+      <c r="H225" t="inlineStr">
+        <is>
+          <t>2026-01-29</t>
+        </is>
+      </c>
+      <c r="I225" t="inlineStr">
+        <is>
+          <t>2026-02-08</t>
+        </is>
+      </c>
+      <c r="K225" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+      <c r="L225" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="M225" t="inlineStr">
+        <is>
+          <t>Bengaluru, India</t>
+        </is>
+      </c>
+      <c r="N225" t="inlineStr">
+        <is>
+          <t>https://2026.sigmod.org/</t>
+        </is>
+      </c>
+      <c r="O225" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:R72"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Fix CHES 2026 dates from official ches.iacr.org/2026
</commit_message>
<xml_diff>
--- a/timeline_data.xlsx
+++ b/timeline_data.xlsx
@@ -1155,42 +1155,42 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
+          <t>2025-08-28</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
           <t>2025-08-31</t>
         </is>
       </c>
-      <c r="I12" t="inlineStr">
+      <c r="J12" t="inlineStr">
         <is>
           <t>2025-09-15</t>
         </is>
       </c>
-      <c r="J12" t="inlineStr">
+      <c r="K12" t="inlineStr">
         <is>
           <t>2025-10-14</t>
         </is>
       </c>
-      <c r="K12" t="inlineStr">
+      <c r="L12" t="inlineStr">
         <is>
           <t>2026-10-11</t>
         </is>
       </c>
-      <c r="L12" t="inlineStr">
+      <c r="M12" t="inlineStr">
         <is>
           <t>2026-10-15</t>
         </is>
       </c>
-      <c r="M12" t="inlineStr">
+      <c r="N12" t="inlineStr">
         <is>
           <t>Antalya, Turkiye</t>
         </is>
       </c>
-      <c r="N12" t="inlineStr">
+      <c r="O12" t="inlineStr">
         <is>
           <t>https://ches.iacr.org/2026/</t>
-        </is>
-      </c>
-      <c r="O12" t="inlineStr">
-        <is>
-          <t>AoE</t>
         </is>
       </c>
     </row>
@@ -1223,42 +1223,42 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2025-12-02</t>
+          <t>2025-11-27</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
+          <t>2025-11-30</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
           <t>2025-12-15</t>
         </is>
       </c>
-      <c r="J13" t="inlineStr">
+      <c r="K13" t="inlineStr">
         <is>
           <t>2026-01-14</t>
         </is>
       </c>
-      <c r="K13" t="inlineStr">
+      <c r="L13" t="inlineStr">
         <is>
           <t>2026-10-11</t>
         </is>
       </c>
-      <c r="L13" t="inlineStr">
+      <c r="M13" t="inlineStr">
         <is>
           <t>2026-10-15</t>
         </is>
       </c>
-      <c r="M13" t="inlineStr">
+      <c r="N13" t="inlineStr">
         <is>
           <t>Antalya, Turkiye</t>
         </is>
       </c>
-      <c r="N13" t="inlineStr">
+      <c r="O13" t="inlineStr">
         <is>
           <t>https://ches.iacr.org/2026/</t>
-        </is>
-      </c>
-      <c r="O13" t="inlineStr">
-        <is>
-          <t>AoE</t>
         </is>
       </c>
     </row>
@@ -1291,42 +1291,42 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
+          <t>2026-02-26</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
           <t>2026-03-01</t>
         </is>
       </c>
-      <c r="I14" t="inlineStr">
+      <c r="J14" t="inlineStr">
         <is>
           <t>2026-03-15</t>
         </is>
       </c>
-      <c r="J14" t="inlineStr">
+      <c r="K14" t="inlineStr">
         <is>
           <t>2026-04-14</t>
         </is>
       </c>
-      <c r="K14" t="inlineStr">
+      <c r="L14" t="inlineStr">
         <is>
           <t>2026-10-11</t>
         </is>
       </c>
-      <c r="L14" t="inlineStr">
+      <c r="M14" t="inlineStr">
         <is>
           <t>2026-10-15</t>
         </is>
       </c>
-      <c r="M14" t="inlineStr">
+      <c r="N14" t="inlineStr">
         <is>
           <t>Antalya, Turkiye</t>
         </is>
       </c>
-      <c r="N14" t="inlineStr">
+      <c r="O14" t="inlineStr">
         <is>
           <t>https://ches.iacr.org/2026/</t>
-        </is>
-      </c>
-      <c r="O14" t="inlineStr">
-        <is>
-          <t>AoE</t>
         </is>
       </c>
     </row>
@@ -1359,42 +1359,42 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
           <t>2026-05-31</t>
         </is>
       </c>
-      <c r="I15" t="inlineStr">
+      <c r="J15" t="inlineStr">
         <is>
           <t>2026-06-15</t>
         </is>
       </c>
-      <c r="J15" t="inlineStr">
+      <c r="K15" t="inlineStr">
         <is>
           <t>2026-07-14</t>
         </is>
       </c>
-      <c r="K15" t="inlineStr">
+      <c r="L15" t="inlineStr">
         <is>
           <t>2026-10-11</t>
         </is>
       </c>
-      <c r="L15" t="inlineStr">
+      <c r="M15" t="inlineStr">
         <is>
           <t>2026-10-15</t>
         </is>
       </c>
-      <c r="M15" t="inlineStr">
+      <c r="N15" t="inlineStr">
         <is>
           <t>Antalya, Turkiye</t>
         </is>
       </c>
-      <c r="N15" t="inlineStr">
+      <c r="O15" t="inlineStr">
         <is>
           <t>https://ches.iacr.org/2026/</t>
-        </is>
-      </c>
-      <c r="O15" t="inlineStr">
-        <is>
-          <t>AoE</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix S&P 2027 dates from official sp2027.ieee-security.org
</commit_message>
<xml_diff>
--- a/timeline_data.xlsx
+++ b/timeline_data.xlsx
@@ -6099,12 +6099,22 @@
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="H96" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="I96" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="J96" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="K96" t="inlineStr">
@@ -6114,22 +6124,22 @@
       </c>
       <c r="L96" t="inlineStr">
         <is>
-          <t>2027-05-21</t>
+          <t>2027-05-01</t>
         </is>
       </c>
       <c r="M96" t="inlineStr">
         <is>
-          <t>San Francisco, CA, USA</t>
+          <t>2027-05-04</t>
         </is>
       </c>
       <c r="N96" t="inlineStr">
         <is>
-          <t>https://www.ieee-security.org/TC/SP2027/</t>
+          <t>Montreal, Canada</t>
         </is>
       </c>
       <c r="O96" t="inlineStr">
         <is>
-          <t>AoE</t>
+          <t>https://sp2027.ieee-security.org/</t>
         </is>
       </c>
     </row>
@@ -6152,12 +6162,22 @@
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>2026-11-13</t>
+          <t>2026-11-17</t>
+        </is>
+      </c>
+      <c r="H97" t="inlineStr">
+        <is>
+          <t>2027-02-11</t>
         </is>
       </c>
       <c r="I97" t="inlineStr">
         <is>
-          <t>2027-02-01</t>
+          <t>2027-02-16</t>
+        </is>
+      </c>
+      <c r="J97" t="inlineStr">
+        <is>
+          <t>2027-03-05</t>
         </is>
       </c>
       <c r="K97" t="inlineStr">
@@ -6177,12 +6197,12 @@
       </c>
       <c r="N97" t="inlineStr">
         <is>
-          <t>https://www.ieee-security.org/TC/SP2027/</t>
+          <t>Montreal, Canada</t>
         </is>
       </c>
       <c r="O97" t="inlineStr">
         <is>
-          <t>AoE</t>
+          <t>https://sp2027.ieee-security.org/</t>
         </is>
       </c>
     </row>
@@ -8181,9 +8201,19 @@
           <t>2026-06-11</t>
         </is>
       </c>
+      <c r="H133" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
       <c r="I133" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="J133" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="K133" t="inlineStr">
@@ -8193,22 +8223,22 @@
       </c>
       <c r="L133" t="inlineStr">
         <is>
+          <t>2027-05-01</t>
+        </is>
+      </c>
+      <c r="M133" t="inlineStr">
+        <is>
           <t>2027-05-04</t>
         </is>
       </c>
-      <c r="M133" t="inlineStr">
-        <is>
-          <t>San Francisco, CA, USA</t>
-        </is>
-      </c>
       <c r="N133" t="inlineStr">
         <is>
-          <t>https://www.ieee-security.org/TC/SP2027/</t>
+          <t>Montreal, Canada</t>
         </is>
       </c>
       <c r="O133" t="inlineStr">
         <is>
-          <t>AoE</t>
+          <t>https://sp2027.ieee-security.org/</t>
         </is>
       </c>
     </row>
@@ -8234,8 +8264,18 @@
           <t>2026-11-17</t>
         </is>
       </c>
+      <c r="H134" t="inlineStr">
+        <is>
+          <t>2027-02-11</t>
+        </is>
+      </c>
       <c r="I134" t="inlineStr">
         <is>
+          <t>2027-02-16</t>
+        </is>
+      </c>
+      <c r="J134" t="inlineStr">
+        <is>
           <t>2027-03-05</t>
         </is>
       </c>
@@ -8256,12 +8296,12 @@
       </c>
       <c r="N134" t="inlineStr">
         <is>
-          <t>https://www.ieee-security.org/TC/SP2027/</t>
+          <t>Montreal, Canada</t>
         </is>
       </c>
       <c r="O134" t="inlineStr">
         <is>
-          <t>AoE</t>
+          <t>https://sp2027.ieee-security.org/</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix NDSS 2027: 2 cycles (May 6 + Aug 19 2026) from official site
</commit_message>
<xml_diff>
--- a/timeline_data.xlsx
+++ b/timeline_data.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R229"/>
+  <dimension ref="A1:R230"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -6331,7 +6331,7 @@
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="I100" t="inlineStr">
@@ -6339,6 +6339,7 @@
           <t>2026-10-15</t>
         </is>
       </c>
+      <c r="J100" t="inlineStr"/>
       <c r="K100" t="inlineStr">
         <is>
           <t>2027-02-23</t>
@@ -8430,7 +8431,7 @@
       </c>
       <c r="E137" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="I137" t="inlineStr">
@@ -8438,6 +8439,7 @@
           <t>2026-11-04</t>
         </is>
       </c>
+      <c r="J137" t="inlineStr"/>
       <c r="K137" t="inlineStr">
         <is>
           <t>2027-03-22</t>
@@ -13665,6 +13667,54 @@
         </is>
       </c>
       <c r="O229" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="inlineStr">
+        <is>
+          <t>ndss</t>
+        </is>
+      </c>
+      <c r="B230" t="inlineStr">
+        <is>
+          <t>NDSS</t>
+        </is>
+      </c>
+      <c r="C230" t="n">
+        <v>2027</v>
+      </c>
+      <c r="D230" t="n">
+        <v>2</v>
+      </c>
+      <c r="E230" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="K230" t="inlineStr">
+        <is>
+          <t>2027-03-22</t>
+        </is>
+      </c>
+      <c r="L230" t="inlineStr">
+        <is>
+          <t>2027-03-26</t>
+        </is>
+      </c>
+      <c r="M230" t="inlineStr">
+        <is>
+          <t>Seoul, South Korea</t>
+        </is>
+      </c>
+      <c r="N230" t="inlineStr">
+        <is>
+          <t>https://www.ndss-symposium.org/</t>
+        </is>
+      </c>
+      <c r="O230" t="inlineStr">
         <is>
           <t>AoE</t>
         </is>

</xml_diff>

<commit_message>
Fix CCS 2026 dates from official sigsac.org CFP
</commit_message>
<xml_diff>
--- a/timeline_data.xlsx
+++ b/timeline_data.xlsx
@@ -1028,34 +1028,44 @@
           <t>2026-01-14</t>
         </is>
       </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>2026-01-07</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>2026-03-17</t>
+        </is>
+      </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-03-20</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
           <t>2026-11-15</t>
         </is>
       </c>
-      <c r="L10" t="inlineStr">
+      <c r="M10" t="inlineStr">
         <is>
           <t>2026-11-19</t>
         </is>
       </c>
-      <c r="M10" t="inlineStr">
+      <c r="N10" t="inlineStr">
         <is>
           <t>The Hague, Netherlands</t>
-        </is>
-      </c>
-      <c r="N10" t="inlineStr">
-        <is>
-          <t>https://www.sigsac.org/ccs/CCS2026/</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
@@ -1095,29 +1105,44 @@
           <t>2026-04-29</t>
         </is>
       </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
       <c r="I11" t="inlineStr">
         <is>
           <t>2026-07-01</t>
         </is>
       </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
       <c r="K11" t="inlineStr">
         <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
           <t>2026-11-15</t>
         </is>
       </c>
-      <c r="L11" t="inlineStr">
+      <c r="M11" t="inlineStr">
         <is>
           <t>2026-11-19</t>
         </is>
       </c>
-      <c r="M11" t="inlineStr">
+      <c r="N11" t="inlineStr">
         <is>
           <t>The Hague, Netherlands</t>
-        </is>
-      </c>
-      <c r="N11" t="inlineStr">
-        <is>
-          <t>https://www.sigsac.org/ccs/CCS2026/</t>
         </is>
       </c>
       <c r="O11" t="inlineStr">
@@ -6339,7 +6364,6 @@
           <t>2026-10-15</t>
         </is>
       </c>
-      <c r="J100" t="inlineStr"/>
       <c r="K100" t="inlineStr">
         <is>
           <t>2027-02-23</t>
@@ -8439,7 +8463,6 @@
           <t>2026-11-04</t>
         </is>
       </c>
-      <c r="J137" t="inlineStr"/>
       <c r="K137" t="inlineStr">
         <is>
           <t>2027-03-22</t>

</xml_diff>

<commit_message>
Fix CHES 2025, USENIX Sec 2027, EUROCRYPT 2027 dates from official sources
</commit_message>
<xml_diff>
--- a/timeline_data.xlsx
+++ b/timeline_data.xlsx
@@ -6071,12 +6071,22 @@
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="H95" t="inlineStr">
+        <is>
+          <t>2026-11-05</t>
         </is>
       </c>
       <c r="I95" t="inlineStr">
         <is>
-          <t>2026-12-01</t>
+          <t>2026-11-12</t>
+        </is>
+      </c>
+      <c r="J95" t="inlineStr">
+        <is>
+          <t>2026-12-03</t>
         </is>
       </c>
       <c r="K95" t="inlineStr">
@@ -6086,22 +6096,22 @@
       </c>
       <c r="L95" t="inlineStr">
         <is>
-          <t>2027-08-14</t>
+          <t>2027-08-11</t>
         </is>
       </c>
       <c r="M95" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>2027-08-13</t>
         </is>
       </c>
       <c r="N95" t="inlineStr">
         <is>
+          <t>Denver, CO, USA</t>
+        </is>
+      </c>
+      <c r="O95" t="inlineStr">
+        <is>
           <t>https://www.usenix.org/conference/usenixsecurity27/</t>
-        </is>
-      </c>
-      <c r="O95" t="inlineStr">
-        <is>
-          <t>AoE</t>
         </is>
       </c>
     </row>
@@ -6127,9 +6137,19 @@
           <t>2027-01-26</t>
         </is>
       </c>
+      <c r="H96" t="inlineStr">
+        <is>
+          <t>2027-04-08</t>
+        </is>
+      </c>
       <c r="I96" t="inlineStr">
         <is>
-          <t>2027-05-01</t>
+          <t>2027-04-15</t>
+        </is>
+      </c>
+      <c r="J96" t="inlineStr">
+        <is>
+          <t>2027-05-06</t>
         </is>
       </c>
       <c r="K96" t="inlineStr">
@@ -6139,22 +6159,22 @@
       </c>
       <c r="L96" t="inlineStr">
         <is>
-          <t>2027-08-14</t>
+          <t>2027-08-11</t>
         </is>
       </c>
       <c r="M96" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>2027-08-13</t>
         </is>
       </c>
       <c r="N96" t="inlineStr">
         <is>
+          <t>Denver, CO, USA</t>
+        </is>
+      </c>
+      <c r="O96" t="inlineStr">
+        <is>
           <t>https://www.usenix.org/conference/usenixsecurity27/</t>
-        </is>
-      </c>
-      <c r="O96" t="inlineStr">
-        <is>
-          <t>AoE</t>
         </is>
       </c>
     </row>
@@ -7681,42 +7701,42 @@
       </c>
       <c r="H124" t="inlineStr">
         <is>
-          <t>2025-02-21</t>
+          <t>2025-02-24</t>
         </is>
       </c>
       <c r="I124" t="inlineStr">
         <is>
+          <t>2025-02-28</t>
+        </is>
+      </c>
+      <c r="J124" t="inlineStr">
+        <is>
           <t>2025-03-15</t>
         </is>
       </c>
-      <c r="J124" t="inlineStr">
+      <c r="K124" t="inlineStr">
         <is>
           <t>2025-04-14</t>
         </is>
       </c>
-      <c r="K124" t="inlineStr">
+      <c r="L124" t="inlineStr">
         <is>
           <t>2025-09-14</t>
         </is>
       </c>
-      <c r="L124" t="inlineStr">
+      <c r="M124" t="inlineStr">
         <is>
           <t>2025-09-18</t>
         </is>
       </c>
-      <c r="M124" t="inlineStr">
+      <c r="N124" t="inlineStr">
         <is>
           <t>Kuala Lumpur, Malaysia</t>
         </is>
       </c>
-      <c r="N124" t="inlineStr">
+      <c r="O124" t="inlineStr">
         <is>
           <t>https://ches.iacr.org/2025/</t>
-        </is>
-      </c>
-      <c r="O124" t="inlineStr">
-        <is>
-          <t>AoE</t>
         </is>
       </c>
     </row>
@@ -7749,42 +7769,42 @@
       </c>
       <c r="H125" t="inlineStr">
         <is>
-          <t>2025-05-23</t>
+          <t>2025-05-26</t>
         </is>
       </c>
       <c r="I125" t="inlineStr">
         <is>
+          <t>2025-05-30</t>
+        </is>
+      </c>
+      <c r="J125" t="inlineStr">
+        <is>
           <t>2025-06-15</t>
         </is>
       </c>
-      <c r="J125" t="inlineStr">
+      <c r="K125" t="inlineStr">
         <is>
           <t>2025-07-14</t>
         </is>
       </c>
-      <c r="K125" t="inlineStr">
+      <c r="L125" t="inlineStr">
         <is>
           <t>2025-09-14</t>
         </is>
       </c>
-      <c r="L125" t="inlineStr">
+      <c r="M125" t="inlineStr">
         <is>
           <t>2025-09-18</t>
         </is>
       </c>
-      <c r="M125" t="inlineStr">
+      <c r="N125" t="inlineStr">
         <is>
           <t>Kuala Lumpur, Malaysia</t>
         </is>
       </c>
-      <c r="N125" t="inlineStr">
+      <c r="O125" t="inlineStr">
         <is>
           <t>https://ches.iacr.org/2025/</t>
-        </is>
-      </c>
-      <c r="O125" t="inlineStr">
-        <is>
-          <t>AoE</t>
         </is>
       </c>
     </row>
@@ -7810,39 +7830,44 @@
           <t>2026-09-17</t>
         </is>
       </c>
+      <c r="H126" t="inlineStr">
+        <is>
+          <t>2026-11-30</t>
+        </is>
+      </c>
       <c r="I126" t="inlineStr">
         <is>
+          <t>2026-12-05</t>
+        </is>
+      </c>
+      <c r="J126" t="inlineStr">
+        <is>
           <t>2027-01-18</t>
         </is>
       </c>
-      <c r="J126" t="inlineStr">
+      <c r="K126" t="inlineStr">
         <is>
           <t>2027-02-08</t>
         </is>
       </c>
-      <c r="K126" t="inlineStr">
+      <c r="L126" t="inlineStr">
         <is>
           <t>2027-04-11</t>
         </is>
       </c>
-      <c r="L126" t="inlineStr">
+      <c r="M126" t="inlineStr">
         <is>
           <t>2027-04-15</t>
         </is>
       </c>
-      <c r="M126" t="inlineStr">
+      <c r="N126" t="inlineStr">
         <is>
           <t>Eindhoven, Netherlands</t>
         </is>
       </c>
-      <c r="N126" t="inlineStr">
+      <c r="O126" t="inlineStr">
         <is>
           <t>https://eurocrypt.iacr.org/2027/</t>
-        </is>
-      </c>
-      <c r="O126" t="inlineStr">
-        <is>
-          <t>AoE</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add NDSS 2027, EUROCRYPT 2026, USENIX Sec 2026/27, S&P 2026, DSN 2026, FC 2026, EuroS&P 2026
</commit_message>
<xml_diff>
--- a/timeline_data.xlsx
+++ b/timeline_data.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R50"/>
+  <dimension ref="A1:R63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -3715,6 +3715,810 @@
         </is>
       </c>
     </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>ndss</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>NDSS</t>
+        </is>
+      </c>
+      <c r="C51" t="n">
+        <v>2027</v>
+      </c>
+      <c r="D51" t="n">
+        <v>1</v>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>2027-03-22</t>
+        </is>
+      </c>
+      <c r="L51" t="inlineStr">
+        <is>
+          <t>2027-03-26</t>
+        </is>
+      </c>
+      <c r="M51" t="inlineStr">
+        <is>
+          <t>Seoul, South Korea</t>
+        </is>
+      </c>
+      <c r="N51" t="inlineStr">
+        <is>
+          <t>https://www.ndss-symposium.org/ndss2027/submissions/call-for-papers/</t>
+        </is>
+      </c>
+      <c r="O51" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>ndss</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>NDSS</t>
+        </is>
+      </c>
+      <c r="C52" t="n">
+        <v>2027</v>
+      </c>
+      <c r="D52" t="n">
+        <v>2</v>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>2026-11-04</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>2027-01-06</t>
+        </is>
+      </c>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>2027-03-22</t>
+        </is>
+      </c>
+      <c r="L52" t="inlineStr">
+        <is>
+          <t>2027-03-26</t>
+        </is>
+      </c>
+      <c r="M52" t="inlineStr">
+        <is>
+          <t>Seoul, South Korea</t>
+        </is>
+      </c>
+      <c r="N52" t="inlineStr">
+        <is>
+          <t>https://www.ndss-symposium.org/ndss2027/submissions/call-for-papers/</t>
+        </is>
+      </c>
+      <c r="O52" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>eurocrypt</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>EUROCRYPT</t>
+        </is>
+      </c>
+      <c r="C53" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D53" t="n">
+        <v>1</v>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>2025-10-02</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>2025-12-08</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>2025-12-12</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>2026-01-29</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>2026-02-27</t>
+        </is>
+      </c>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="L53" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="M53" t="inlineStr">
+        <is>
+          <t>Rome, Italy</t>
+        </is>
+      </c>
+      <c r="N53" t="inlineStr">
+        <is>
+          <t>https://eurocrypt.iacr.org/2026/</t>
+        </is>
+      </c>
+      <c r="O53" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>asiacrypt</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>ASIACRYPT</t>
+        </is>
+      </c>
+      <c r="C54" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D54" t="n">
+        <v>1</v>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>2025-05-16</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>2025-07-01</t>
+        </is>
+      </c>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t>2025-12-07</t>
+        </is>
+      </c>
+      <c r="L54" t="inlineStr">
+        <is>
+          <t>2025-12-11</t>
+        </is>
+      </c>
+      <c r="M54" t="inlineStr">
+        <is>
+          <t>Melbourne, Australia</t>
+        </is>
+      </c>
+      <c r="N54" t="inlineStr">
+        <is>
+          <t>https://asiacrypt.iacr.org/2025/</t>
+        </is>
+      </c>
+      <c r="O54" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>usenix-security</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>USENIX Security</t>
+        </is>
+      </c>
+      <c r="C55" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D55" t="n">
+        <v>1</v>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>2025-08-26</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>2025-11-06</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>2025-11-13</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>2025-12-04</t>
+        </is>
+      </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>2026-01-15</t>
+        </is>
+      </c>
+      <c r="K55" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="L55" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="M55" t="inlineStr">
+        <is>
+          <t>Baltimore, MD, USA</t>
+        </is>
+      </c>
+      <c r="N55" t="inlineStr">
+        <is>
+          <t>https://www.usenix.org/conference/usenixsecurity26/</t>
+        </is>
+      </c>
+      <c r="O55" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>usenix-security</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>USENIX Security</t>
+        </is>
+      </c>
+      <c r="C56" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D56" t="n">
+        <v>2</v>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>2026-02-05</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>2026-04-23</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="K56" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="L56" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="M56" t="inlineStr">
+        <is>
+          <t>Baltimore, MD, USA</t>
+        </is>
+      </c>
+      <c r="N56" t="inlineStr">
+        <is>
+          <t>https://www.usenix.org/conference/usenixsecurity26/</t>
+        </is>
+      </c>
+      <c r="O56" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>usenix-security</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>USENIX Security</t>
+        </is>
+      </c>
+      <c r="C57" t="n">
+        <v>2027</v>
+      </c>
+      <c r="D57" t="n">
+        <v>1</v>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>2026-11-05</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>2026-11-12</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>2026-12-03</t>
+        </is>
+      </c>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>2027-01-14</t>
+        </is>
+      </c>
+      <c r="K57" t="inlineStr">
+        <is>
+          <t>2027-08-11</t>
+        </is>
+      </c>
+      <c r="L57" t="inlineStr">
+        <is>
+          <t>2027-08-13</t>
+        </is>
+      </c>
+      <c r="M57" t="inlineStr">
+        <is>
+          <t>Denver, CO, USA</t>
+        </is>
+      </c>
+      <c r="N57" t="inlineStr">
+        <is>
+          <t>https://www.usenix.org/conference/usenixsecurity27/</t>
+        </is>
+      </c>
+      <c r="O57" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>usenix-security</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>USENIX Security</t>
+        </is>
+      </c>
+      <c r="C58" t="n">
+        <v>2027</v>
+      </c>
+      <c r="D58" t="n">
+        <v>2</v>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>2027-01-26</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>2027-04-08</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>2027-04-15</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>2027-05-06</t>
+        </is>
+      </c>
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>2027-06-03</t>
+        </is>
+      </c>
+      <c r="K58" t="inlineStr">
+        <is>
+          <t>2027-08-11</t>
+        </is>
+      </c>
+      <c r="L58" t="inlineStr">
+        <is>
+          <t>2027-08-13</t>
+        </is>
+      </c>
+      <c r="M58" t="inlineStr">
+        <is>
+          <t>Denver, CO, USA</t>
+        </is>
+      </c>
+      <c r="N58" t="inlineStr">
+        <is>
+          <t>https://www.usenix.org/conference/usenixsecurity27/</t>
+        </is>
+      </c>
+      <c r="O58" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>s-p</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>S&amp;P</t>
+        </is>
+      </c>
+      <c r="C59" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D59" t="n">
+        <v>1</v>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>2025-06-05</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>2025-09-01</t>
+        </is>
+      </c>
+      <c r="K59" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="L59" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="M59" t="inlineStr">
+        <is>
+          <t>San Francisco, CA, USA</t>
+        </is>
+      </c>
+      <c r="N59" t="inlineStr">
+        <is>
+          <t>https://www.ieee-security.org/TC/SP2026/</t>
+        </is>
+      </c>
+      <c r="O59" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>s-p</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>S&amp;P</t>
+        </is>
+      </c>
+      <c r="C60" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D60" t="n">
+        <v>2</v>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>2025-11-13</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>2026-02-01</t>
+        </is>
+      </c>
+      <c r="K60" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="L60" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="M60" t="inlineStr">
+        <is>
+          <t>San Francisco, CA, USA</t>
+        </is>
+      </c>
+      <c r="N60" t="inlineStr">
+        <is>
+          <t>https://www.ieee-security.org/TC/SP2026/</t>
+        </is>
+      </c>
+      <c r="O60" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>dsn</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>DSN</t>
+        </is>
+      </c>
+      <c r="C61" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D61" t="n">
+        <v>1</v>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>2025-12-04</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>2026-02-13</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>2026-02-27</t>
+        </is>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>2026-03-19</t>
+        </is>
+      </c>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="K61" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="L61" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="M61" t="inlineStr">
+        <is>
+          <t>Charlotte, NC, USA</t>
+        </is>
+      </c>
+      <c r="N61" t="inlineStr">
+        <is>
+          <t>https://dsn2026.github.io/</t>
+        </is>
+      </c>
+      <c r="O61" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>fc</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>FC</t>
+        </is>
+      </c>
+      <c r="C62" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D62" t="n">
+        <v>1</v>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>2025-09-20</t>
+        </is>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>2025-11-24</t>
+        </is>
+      </c>
+      <c r="J62" t="inlineStr">
+        <is>
+          <t>2026-01-12</t>
+        </is>
+      </c>
+      <c r="K62" t="inlineStr">
+        <is>
+          <t>2026-03-02</t>
+        </is>
+      </c>
+      <c r="L62" t="inlineStr">
+        <is>
+          <t>2026-03-06</t>
+        </is>
+      </c>
+      <c r="M62" t="inlineStr">
+        <is>
+          <t>St. Kitts</t>
+        </is>
+      </c>
+      <c r="N62" t="inlineStr">
+        <is>
+          <t>https://ifca.ai/fc26/</t>
+        </is>
+      </c>
+      <c r="O62" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>euros-p</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>EuroS&amp;P</t>
+        </is>
+      </c>
+      <c r="C63" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D63" t="n">
+        <v>1</v>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>2025-11-20</t>
+        </is>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>2026-02-15</t>
+        </is>
+      </c>
+      <c r="K63" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="L63" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="M63" t="inlineStr">
+        <is>
+          <t>Lisbon, Portugal</t>
+        </is>
+      </c>
+      <c r="N63" t="inlineStr">
+        <is>
+          <t>https://www.ieee-security.org/TC/EuroSP2026/</t>
+        </is>
+      </c>
+      <c r="O63" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:R72"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Clean rebuild from verified data only (4 sheets)
</commit_message>
<xml_diff>
--- a/timeline_data.xlsx
+++ b/timeline_data.xlsx
@@ -62,9 +62,7 @@
   </cellStyleXfs>
   <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -430,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R7"/>
+  <dimension ref="A1:O4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -509,71 +507,68 @@
           <t>timezone</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
-        <is>
-          <t>submissions</t>
-        </is>
-      </c>
-      <c r="Q1" s="1" t="inlineStr">
-        <is>
-          <t>accepted</t>
-        </is>
-      </c>
-      <c r="R1" s="1" t="inlineStr">
-        <is>
-          <t>acceptance_rate</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>asiacrypt</t>
+          <t>ches</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>ASIACRYPT</t>
+          <t>CHES</t>
         </is>
       </c>
       <c r="C2" t="n">
         <v>2025</v>
       </c>
       <c r="D2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2025-05-16</t>
+          <t>2025-01-15</t>
         </is>
       </c>
       <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr"/>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>2025-02-24</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>2025-02-28</t>
+        </is>
+      </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>2025-07-01</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr"/>
+          <t>2025-03-15</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>2025-04-14</t>
+        </is>
+      </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>2025-12-07</t>
+          <t>2025-09-14</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>2025-12-11</t>
+          <t>2025-09-18</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>Melbourne, Australia</t>
+          <t>Kuala Lumpur, Malaysia</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>https://asiacrypt.iacr.org/2025/</t>
+          <t>https://ches.iacr.org/2025/</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
@@ -581,9 +576,6 @@
           <t>AoE</t>
         </is>
       </c>
-      <c r="P2" t="inlineStr"/>
-      <c r="Q2" t="inlineStr"/>
-      <c r="R2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -600,124 +592,121 @@
         <v>2025</v>
       </c>
       <c r="D3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2025-01-15</t>
+          <t>2025-04-15</t>
         </is>
       </c>
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2025-02-17</t>
+          <t>2025-05-26</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>2025-02-24</t>
+          <t>2025-05-30</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>2025-02-28</t>
+          <t>2025-06-15</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>2025-03-15</t>
+          <t>2025-07-14</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>2025-04-14</t>
+          <t>2025-09-14</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>2025-09-14</t>
+          <t>2025-09-18</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2025-09-18</t>
+          <t>Kuala Lumpur, Malaysia</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>Kuala Lumpur, Malaysia</t>
+          <t>https://ches.iacr.org/2025/</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>https://ches.iacr.org/2025/</t>
-        </is>
-      </c>
-      <c r="P3" t="inlineStr"/>
-      <c r="Q3" t="inlineStr"/>
-      <c r="R3" t="inlineStr"/>
+          <t>AoE</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>ches</t>
+          <t>crypto</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>CHES</t>
+          <t>CRYPTO</t>
         </is>
       </c>
       <c r="C4" t="n">
         <v>2025</v>
       </c>
       <c r="D4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2025-01-15</t>
+          <t>2025-02-13</t>
         </is>
       </c>
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2025-02-24</t>
+          <t>2025-04-07</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>2025-02-28</t>
+          <t>2025-04-12</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>2025-03-15</t>
+          <t>2025-05-03</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>2025-04-14</t>
+          <t>2025-06-05</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>2025-09-14</t>
+          <t>2025-08-17</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>2025-09-18</t>
+          <t>2025-08-21</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>Kuala Lumpur, Malaysia</t>
+          <t>Santa Barbara, CA, USA</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>https://ches.iacr.org/2025/</t>
+          <t>https://crypto.iacr.org/2025/</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
@@ -725,225 +714,6 @@
           <t>AoE</t>
         </is>
       </c>
-      <c r="P4" t="inlineStr"/>
-      <c r="Q4" t="inlineStr"/>
-      <c r="R4" t="inlineStr"/>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>ches</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>CHES</t>
-        </is>
-      </c>
-      <c r="C5" t="n">
-        <v>2025</v>
-      </c>
-      <c r="D5" t="n">
-        <v>4</v>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>2025-04-15</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>2025-05-19</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>2025-05-26</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>2025-05-30</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>2025-06-15</t>
-        </is>
-      </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>2025-07-14</t>
-        </is>
-      </c>
-      <c r="L5" t="inlineStr">
-        <is>
-          <t>2025-09-14</t>
-        </is>
-      </c>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>2025-09-18</t>
-        </is>
-      </c>
-      <c r="N5" t="inlineStr">
-        <is>
-          <t>Kuala Lumpur, Malaysia</t>
-        </is>
-      </c>
-      <c r="O5" t="inlineStr">
-        <is>
-          <t>https://ches.iacr.org/2025/</t>
-        </is>
-      </c>
-      <c r="P5" t="inlineStr"/>
-      <c r="Q5" t="inlineStr"/>
-      <c r="R5" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>ches</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>CHES</t>
-        </is>
-      </c>
-      <c r="C6" t="n">
-        <v>2025</v>
-      </c>
-      <c r="D6" t="n">
-        <v>4</v>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>2025-04-15</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>2025-05-26</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>2025-05-30</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>2025-06-15</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>2025-07-14</t>
-        </is>
-      </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>2025-09-14</t>
-        </is>
-      </c>
-      <c r="L6" t="inlineStr">
-        <is>
-          <t>2025-09-18</t>
-        </is>
-      </c>
-      <c r="M6" t="inlineStr">
-        <is>
-          <t>Kuala Lumpur, Malaysia</t>
-        </is>
-      </c>
-      <c r="N6" t="inlineStr">
-        <is>
-          <t>https://ches.iacr.org/2025/</t>
-        </is>
-      </c>
-      <c r="O6" t="inlineStr">
-        <is>
-          <t>AoE</t>
-        </is>
-      </c>
-      <c r="P6" t="inlineStr"/>
-      <c r="Q6" t="inlineStr"/>
-      <c r="R6" t="inlineStr"/>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>crypto</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>CRYPTO</t>
-        </is>
-      </c>
-      <c r="C7" t="n">
-        <v>2025</v>
-      </c>
-      <c r="D7" t="n">
-        <v>1</v>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>2025-02-13</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr"/>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>2025-04-07</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>2025-04-12</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>2025-05-03</t>
-        </is>
-      </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>2025-06-05</t>
-        </is>
-      </c>
-      <c r="K7" t="inlineStr">
-        <is>
-          <t>2025-08-17</t>
-        </is>
-      </c>
-      <c r="L7" t="inlineStr">
-        <is>
-          <t>2025-08-21</t>
-        </is>
-      </c>
-      <c r="M7" t="inlineStr">
-        <is>
-          <t>Santa Barbara, CA, USA</t>
-        </is>
-      </c>
-      <c r="N7" t="inlineStr">
-        <is>
-          <t>https://crypto.iacr.org/2025/</t>
-        </is>
-      </c>
-      <c r="O7" t="inlineStr">
-        <is>
-          <t>AoE</t>
-        </is>
-      </c>
-      <c r="P7" t="inlineStr"/>
-      <c r="Q7" t="inlineStr"/>
-      <c r="R7" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -956,7 +726,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R25"/>
+  <dimension ref="A1:O17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1035,31 +805,16 @@
           <t>timezone</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
-        <is>
-          <t>submissions</t>
-        </is>
-      </c>
-      <c r="Q1" s="1" t="inlineStr">
-        <is>
-          <t>accepted</t>
-        </is>
-      </c>
-      <c r="R1" s="1" t="inlineStr">
-        <is>
-          <t>acceptance_rate</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>asplos</t>
+          <t>ches</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>ASPLOS</t>
+          <t>CHES</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -1070,56 +825,65 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2025-03-12</t>
+          <t>2025-07-15</t>
         </is>
       </c>
       <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr"/>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>2025-08-28</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>2025-08-31</t>
+        </is>
+      </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>2025-06-24</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr"/>
+          <t>2025-09-15</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>2025-10-14</t>
+        </is>
+      </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>2026-03-28</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>San Diego, CA, USA</t>
+          <t>Antalya, Turkiye</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>https://www.asplos-conference.org/asplos2026/</t>
+          <t>https://ches.iacr.org/2026/</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>US Eastern</t>
-        </is>
-      </c>
-      <c r="P2" t="inlineStr"/>
-      <c r="Q2" t="inlineStr"/>
-      <c r="R2" t="inlineStr"/>
+          <t>AoE</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>asplos</t>
+          <t>ches</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>ASPLOS</t>
+          <t>CHES</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -1130,56 +894,65 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2025-08-20</t>
+          <t>2025-10-15</t>
         </is>
       </c>
       <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr"/>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>2025-11-27</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>2025-11-30</t>
+        </is>
+      </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>2025-11-24</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr"/>
+          <t>2025-12-15</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>2026-01-14</t>
+        </is>
+      </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>2026-03-28</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>San Diego, CA, USA</t>
+          <t>Antalya, Turkiye</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>https://www.asplos-conference.org/asplos2026/</t>
+          <t>https://ches.iacr.org/2026/</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>US Eastern</t>
-        </is>
-      </c>
-      <c r="P3" t="inlineStr"/>
-      <c r="Q3" t="inlineStr"/>
-      <c r="R3" t="inlineStr"/>
+          <t>AoE</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>ches</t>
+          <t>fse</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>CHES</t>
+          <t>FSE</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -1190,120 +963,117 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2025-07-15</t>
+          <t>2025-09-01</t>
         </is>
       </c>
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2025-08-28</t>
+          <t>2025-10-05</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>2025-08-28</t>
+          <t>2025-10-08</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>2025-08-31</t>
+          <t>2025-11-01</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>2025-09-15</t>
+          <t>2025-11-28</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>2025-10-14</t>
+          <t>2026-03-23</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>Singapore</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>Antalya, Turkiye</t>
+          <t>https://fse.iacr.org/2026/</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>https://ches.iacr.org/2026/</t>
-        </is>
-      </c>
-      <c r="P4" t="inlineStr"/>
-      <c r="Q4" t="inlineStr"/>
-      <c r="R4" t="inlineStr"/>
+          <t>AoE</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>ches</t>
+          <t>fse</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>CHES</t>
+          <t>FSE</t>
         </is>
       </c>
       <c r="C5" t="n">
         <v>2026</v>
       </c>
       <c r="D5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2025-07-15</t>
+          <t>2025-11-23</t>
         </is>
       </c>
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2025-08-28</t>
+          <t>2026-01-02</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2025-08-31</t>
+          <t>2026-01-06</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>2025-09-15</t>
+          <t>2026-01-23</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2025-10-14</t>
+          <t>2026-02-20</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-03-23</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>Antalya, Turkiye</t>
+          <t>Singapore</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>https://ches.iacr.org/2026/</t>
+          <t>https://fse.iacr.org/2026/</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
@@ -1311,143 +1081,137 @@
           <t>AoE</t>
         </is>
       </c>
-      <c r="P5" t="inlineStr"/>
-      <c r="Q5" t="inlineStr"/>
-      <c r="R5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>ches</t>
+          <t>usenix-security</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>CHES</t>
+          <t>USENIX Security</t>
         </is>
       </c>
       <c r="C6" t="n">
         <v>2026</v>
       </c>
       <c r="D6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2025-10-15</t>
+          <t>2025-08-26</t>
         </is>
       </c>
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2025-11-27</t>
+          <t>2025-11-06</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2025-11-27</t>
+          <t>2025-11-13</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>2025-11-30</t>
+          <t>2025-12-04</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2025-12-15</t>
+          <t>2026-01-15</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>2026-01-14</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>Baltimore, MD, USA</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>Antalya, Turkiye</t>
+          <t>https://www.usenix.org/conference/usenixsecurity26/</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>https://ches.iacr.org/2026/</t>
-        </is>
-      </c>
-      <c r="P6" t="inlineStr"/>
-      <c r="Q6" t="inlineStr"/>
-      <c r="R6" t="inlineStr"/>
+          <t>AoE</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>ches</t>
+          <t>ndss</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>CHES</t>
+          <t>NDSS</t>
         </is>
       </c>
       <c r="C7" t="n">
         <v>2026</v>
       </c>
       <c r="D7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>2025-10-15</t>
+          <t>2025-07-10</t>
         </is>
       </c>
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2025-11-27</t>
+          <t>2025-09-22</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2025-11-30</t>
+          <t>2025-09-29</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>2025-12-15</t>
+          <t>2025-10-24</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2026-01-14</t>
+          <t>2025-12-05</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-02-23</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-02-26</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>Antalya, Turkiye</t>
+          <t>San Diego, CA, USA</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>https://ches.iacr.org/2026/</t>
+          <t>https://www.ndss-symposium.org/</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
@@ -1455,19 +1219,16 @@
           <t>AoE</t>
         </is>
       </c>
-      <c r="P7" t="inlineStr"/>
-      <c r="Q7" t="inlineStr"/>
-      <c r="R7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>csf</t>
+          <t>s-p</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>CSF</t>
+          <t>S&amp;P</t>
         </is>
       </c>
       <c r="C8" t="n">
@@ -1478,7 +1239,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>2025-07-24</t>
+          <t>2025-06-05</t>
         </is>
       </c>
       <c r="F8" t="inlineStr"/>
@@ -1486,28 +1247,28 @@
       <c r="H8" t="inlineStr"/>
       <c r="I8" t="inlineStr">
         <is>
-          <t>2025-09-25</t>
+          <t>2025-09-01</t>
         </is>
       </c>
       <c r="J8" t="inlineStr"/>
       <c r="K8" t="inlineStr">
         <is>
-          <t>2026-07-26</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>Lisbon, Portugal</t>
+          <t>San Francisco, CA, USA</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>https://www.ieee-security.org/TC/CSF2026/</t>
+          <t>https://www.ieee-security.org/TC/SP2026/</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
@@ -1515,19 +1276,16 @@
           <t>AoE</t>
         </is>
       </c>
-      <c r="P8" t="inlineStr"/>
-      <c r="Q8" t="inlineStr"/>
-      <c r="R8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>csf</t>
+          <t>s-p</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>CSF</t>
+          <t>S&amp;P</t>
         </is>
       </c>
       <c r="C9" t="n">
@@ -1538,7 +1296,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2025-10-09</t>
+          <t>2025-11-13</t>
         </is>
       </c>
       <c r="F9" t="inlineStr"/>
@@ -1546,28 +1304,28 @@
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="inlineStr">
         <is>
-          <t>2025-12-11</t>
+          <t>2026-02-01</t>
         </is>
       </c>
       <c r="J9" t="inlineStr"/>
       <c r="K9" t="inlineStr">
         <is>
-          <t>2026-07-26</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>Lisbon, Portugal</t>
+          <t>San Francisco, CA, USA</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>https://www.ieee-security.org/TC/CSF2026/</t>
+          <t>https://www.ieee-security.org/TC/SP2026/</t>
         </is>
       </c>
       <c r="O9" t="inlineStr">
@@ -1575,19 +1333,16 @@
           <t>AoE</t>
         </is>
       </c>
-      <c r="P9" t="inlineStr"/>
-      <c r="Q9" t="inlineStr"/>
-      <c r="R9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>dsn</t>
+          <t>eurocrypt</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>DSN</t>
+          <t>EUROCRYPT</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -1598,48 +1353,48 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>2025-12-04</t>
+          <t>2025-10-02</t>
         </is>
       </c>
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
         <is>
-          <t>2026-02-13</t>
+          <t>2025-12-08</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
+          <t>2025-12-12</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>2026-01-29</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
           <t>2026-02-27</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>2026-03-19</t>
-        </is>
-      </c>
-      <c r="J10" t="inlineStr">
-        <is>
-          <t>2026-04-28</t>
-        </is>
-      </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>Charlotte, NC, USA</t>
+          <t>Rome, Italy</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>https://dsn2026.github.io/</t>
+          <t>https://eurocrypt.iacr.org/2026/</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
@@ -1647,19 +1402,16 @@
           <t>AoE</t>
         </is>
       </c>
-      <c r="P10" t="inlineStr"/>
-      <c r="Q10" t="inlineStr"/>
-      <c r="R10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>eurocrypt</t>
+          <t>dsn</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>EUROCRYPT</t>
+          <t>DSN</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -1670,48 +1422,48 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>2025-10-02</t>
+          <t>2025-12-04</t>
         </is>
       </c>
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr">
         <is>
-          <t>2025-12-08</t>
+          <t>2026-02-13</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2025-12-12</t>
+          <t>2026-02-27</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>2026-01-29</t>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>2026-02-27</t>
+          <t>2026-04-28</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>Rome, Italy</t>
+          <t>Charlotte, NC, USA</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>https://eurocrypt.iacr.org/2026/</t>
+          <t>https://dsn2026.github.io/</t>
         </is>
       </c>
       <c r="O11" t="inlineStr">
@@ -1719,19 +1471,16 @@
           <t>AoE</t>
         </is>
       </c>
-      <c r="P11" t="inlineStr"/>
-      <c r="Q11" t="inlineStr"/>
-      <c r="R11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>euros-p</t>
+          <t>fc</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>EuroS&amp;P</t>
+          <t>FC</t>
         </is>
       </c>
       <c r="C12" t="n">
@@ -1742,7 +1491,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>2025-11-20</t>
+          <t>2025-09-20</t>
         </is>
       </c>
       <c r="F12" t="inlineStr"/>
@@ -1750,28 +1499,32 @@
       <c r="H12" t="inlineStr"/>
       <c r="I12" t="inlineStr">
         <is>
-          <t>2026-02-15</t>
-        </is>
-      </c>
-      <c r="J12" t="inlineStr"/>
+          <t>2025-11-24</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>2026-01-12</t>
+        </is>
+      </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-03-02</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-03-06</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>Lisbon, Portugal</t>
+          <t>St. Kitts</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>https://www.ieee-security.org/TC/EuroSP2026/</t>
+          <t>https://ifca.ai/fc26/</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
@@ -1779,19 +1532,16 @@
           <t>AoE</t>
         </is>
       </c>
-      <c r="P12" t="inlineStr"/>
-      <c r="Q12" t="inlineStr"/>
-      <c r="R12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>fc</t>
+          <t>euros-p</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>FC</t>
+          <t>EuroS&amp;P</t>
         </is>
       </c>
       <c r="C13" t="n">
@@ -1802,7 +1552,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>2025-09-20</t>
+          <t>2025-11-20</t>
         </is>
       </c>
       <c r="F13" t="inlineStr"/>
@@ -1810,32 +1560,28 @@
       <c r="H13" t="inlineStr"/>
       <c r="I13" t="inlineStr">
         <is>
-          <t>2025-11-24</t>
-        </is>
-      </c>
-      <c r="J13" t="inlineStr">
-        <is>
-          <t>2026-01-12</t>
-        </is>
-      </c>
+          <t>2026-02-15</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr"/>
       <c r="K13" t="inlineStr">
         <is>
-          <t>2026-03-02</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>St. Kitts</t>
+          <t>Lisbon, Portugal</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>https://ifca.ai/fc26/</t>
+          <t>https://www.ieee-security.org/TC/EuroSP2026/</t>
         </is>
       </c>
       <c r="O13" t="inlineStr">
@@ -1843,19 +1589,16 @@
           <t>AoE</t>
         </is>
       </c>
-      <c r="P13" t="inlineStr"/>
-      <c r="Q13" t="inlineStr"/>
-      <c r="R13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>fse</t>
+          <t>pkc</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>FSE</t>
+          <t>PKC</t>
         </is>
       </c>
       <c r="C14" t="n">
@@ -1866,48 +1609,48 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>2025-09-01</t>
+          <t>2025-10-24</t>
         </is>
       </c>
       <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr">
         <is>
-          <t>2025-10-05</t>
+          <t>2025-12-16</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2025-10-08</t>
+          <t>2025-12-23</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>2025-11-01</t>
+          <t>2026-02-13</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>2025-11-28</t>
+          <t>2026-03-06</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>2026-03-23</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>Singapore</t>
+          <t>West Palm Beach, FL, USA</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>https://fse.iacr.org/2026/</t>
+          <t>https://pkc.iacr.org/2026/</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
@@ -1915,71 +1658,56 @@
           <t>AoE</t>
         </is>
       </c>
-      <c r="P14" t="inlineStr"/>
-      <c r="Q14" t="inlineStr"/>
-      <c r="R14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>fse</t>
+          <t>csf</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>FSE</t>
+          <t>CSF</t>
         </is>
       </c>
       <c r="C15" t="n">
         <v>2026</v>
       </c>
       <c r="D15" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>2025-11-23</t>
+          <t>2025-07-24</t>
         </is>
       </c>
       <c r="F15" t="inlineStr"/>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>2026-01-02</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>2026-01-06</t>
-        </is>
-      </c>
+      <c r="G15" t="inlineStr"/>
+      <c r="H15" t="inlineStr"/>
       <c r="I15" t="inlineStr">
         <is>
-          <t>2026-01-23</t>
-        </is>
-      </c>
-      <c r="J15" t="inlineStr">
-        <is>
-          <t>2026-02-20</t>
-        </is>
-      </c>
+          <t>2025-09-25</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr"/>
       <c r="K15" t="inlineStr">
         <is>
-          <t>2026-03-23</t>
+          <t>2026-07-26</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>Singapore</t>
+          <t>Lisbon, Portugal</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>https://fse.iacr.org/2026/</t>
+          <t>https://www.ieee-security.org/TC/CSF2026/</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
@@ -1987,30 +1715,27 @@
           <t>AoE</t>
         </is>
       </c>
-      <c r="P15" t="inlineStr"/>
-      <c r="Q15" t="inlineStr"/>
-      <c r="R15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>icde</t>
+          <t>csf</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>ICDE</t>
+          <t>CSF</t>
         </is>
       </c>
       <c r="C16" t="n">
         <v>2026</v>
       </c>
       <c r="D16" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>2025-06-18</t>
+          <t>2025-10-09</t>
         </is>
       </c>
       <c r="F16" t="inlineStr"/>
@@ -2018,48 +1743,45 @@
       <c r="H16" t="inlineStr"/>
       <c r="I16" t="inlineStr">
         <is>
-          <t>2025-10-20</t>
+          <t>2025-12-11</t>
         </is>
       </c>
       <c r="J16" t="inlineStr"/>
       <c r="K16" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-07-26</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>Hong Kong, China</t>
+          <t>Lisbon, Portugal</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>https://icde2026.github.io/</t>
+          <t>https://www.ieee-security.org/TC/CSF2026/</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>US Pacific</t>
-        </is>
-      </c>
-      <c r="P16" t="inlineStr"/>
-      <c r="Q16" t="inlineStr"/>
-      <c r="R16" t="inlineStr"/>
+          <t>AoE</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>nsdi</t>
+          <t>www</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>NSDI</t>
+          <t>WWW</t>
         </is>
       </c>
       <c r="C17" t="n">
@@ -2070,574 +1792,55 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>2025-04-25</t>
+          <t>2025-10-24</t>
         </is>
       </c>
       <c r="F17" t="inlineStr"/>
-      <c r="G17" t="inlineStr"/>
-      <c r="H17" t="inlineStr"/>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>2026-01-06</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>2026-01-13</t>
+        </is>
+      </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>2025-07-24</t>
+          <t>2026-01-24</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>2025-10-21</t>
+          <t>2026-02-14</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-04-19</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-04-24</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>Renton, WA, USA</t>
+          <t>Perth, Australia</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>https://www.usenix.org/conference/nsdi26/</t>
+          <t>https://www2026.thewebconf.org/</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>US PDT</t>
-        </is>
-      </c>
-      <c r="P17" t="inlineStr"/>
-      <c r="Q17" t="inlineStr"/>
-      <c r="R17" t="inlineStr"/>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>nsdi</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>NSDI</t>
-        </is>
-      </c>
-      <c r="C18" t="n">
-        <v>2026</v>
-      </c>
-      <c r="D18" t="n">
-        <v>2</v>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>2025-09-18</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr"/>
-      <c r="G18" t="inlineStr"/>
-      <c r="H18" t="inlineStr"/>
-      <c r="I18" t="inlineStr">
-        <is>
-          <t>2025-12-09</t>
-        </is>
-      </c>
-      <c r="J18" t="inlineStr">
-        <is>
-          <t>2026-03-05</t>
-        </is>
-      </c>
-      <c r="K18" t="inlineStr">
-        <is>
-          <t>2026-05-04</t>
-        </is>
-      </c>
-      <c r="L18" t="inlineStr">
-        <is>
-          <t>2026-05-06</t>
-        </is>
-      </c>
-      <c r="M18" t="inlineStr">
-        <is>
-          <t>Renton, WA, USA</t>
-        </is>
-      </c>
-      <c r="N18" t="inlineStr">
-        <is>
-          <t>https://www.usenix.org/conference/nsdi26/</t>
-        </is>
-      </c>
-      <c r="O18" t="inlineStr">
-        <is>
-          <t>US PDT</t>
-        </is>
-      </c>
-      <c r="P18" t="inlineStr"/>
-      <c r="Q18" t="inlineStr"/>
-      <c r="R18" t="inlineStr"/>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>pakdd</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>PAKDD</t>
-        </is>
-      </c>
-      <c r="C19" t="n">
-        <v>2026</v>
-      </c>
-      <c r="D19" t="n">
-        <v>1</v>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>2025-11-25</t>
-        </is>
-      </c>
-      <c r="F19" t="inlineStr"/>
-      <c r="G19" t="inlineStr"/>
-      <c r="H19" t="inlineStr"/>
-      <c r="I19" t="inlineStr">
-        <is>
-          <t>2026-02-08</t>
-        </is>
-      </c>
-      <c r="J19" t="inlineStr">
-        <is>
-          <t>2026-03-01</t>
-        </is>
-      </c>
-      <c r="K19" t="inlineStr">
-        <is>
-          <t>2026-06-09</t>
-        </is>
-      </c>
-      <c r="L19" t="inlineStr">
-        <is>
-          <t>2026-06-12</t>
-        </is>
-      </c>
-      <c r="M19" t="inlineStr">
-        <is>
-          <t>Hong Kong SAR, China</t>
-        </is>
-      </c>
-      <c r="N19" t="inlineStr">
-        <is>
-          <t>https://www.pakdd2026.org/</t>
-        </is>
-      </c>
-      <c r="O19" t="inlineStr">
-        <is>
-          <t>US PST</t>
-        </is>
-      </c>
-      <c r="P19" t="inlineStr"/>
-      <c r="Q19" t="inlineStr"/>
-      <c r="R19" t="inlineStr"/>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>pkc</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>PKC</t>
-        </is>
-      </c>
-      <c r="C20" t="n">
-        <v>2026</v>
-      </c>
-      <c r="D20" t="n">
-        <v>1</v>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>2025-10-24</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr"/>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>2025-12-16</t>
-        </is>
-      </c>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>2025-12-23</t>
-        </is>
-      </c>
-      <c r="I20" t="inlineStr">
-        <is>
-          <t>2026-02-13</t>
-        </is>
-      </c>
-      <c r="J20" t="inlineStr">
-        <is>
-          <t>2026-03-06</t>
-        </is>
-      </c>
-      <c r="K20" t="inlineStr">
-        <is>
-          <t>2026-05-25</t>
-        </is>
-      </c>
-      <c r="L20" t="inlineStr">
-        <is>
-          <t>2026-05-28</t>
-        </is>
-      </c>
-      <c r="M20" t="inlineStr">
-        <is>
-          <t>West Palm Beach, FL, USA</t>
-        </is>
-      </c>
-      <c r="N20" t="inlineStr">
-        <is>
-          <t>https://pkc.iacr.org/2026/</t>
-        </is>
-      </c>
-      <c r="O20" t="inlineStr">
-        <is>
-          <t>AoE</t>
-        </is>
-      </c>
-      <c r="P20" t="inlineStr"/>
-      <c r="Q20" t="inlineStr"/>
-      <c r="R20" t="inlineStr"/>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>s-p</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>S&amp;P</t>
-        </is>
-      </c>
-      <c r="C21" t="n">
-        <v>2026</v>
-      </c>
-      <c r="D21" t="n">
-        <v>1</v>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>2025-06-05</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr"/>
-      <c r="G21" t="inlineStr"/>
-      <c r="H21" t="inlineStr"/>
-      <c r="I21" t="inlineStr">
-        <is>
-          <t>2025-09-01</t>
-        </is>
-      </c>
-      <c r="J21" t="inlineStr"/>
-      <c r="K21" t="inlineStr">
-        <is>
-          <t>2026-05-18</t>
-        </is>
-      </c>
-      <c r="L21" t="inlineStr">
-        <is>
-          <t>2026-05-21</t>
-        </is>
-      </c>
-      <c r="M21" t="inlineStr">
-        <is>
-          <t>San Francisco, CA, USA</t>
-        </is>
-      </c>
-      <c r="N21" t="inlineStr">
-        <is>
-          <t>https://www.ieee-security.org/TC/SP2026/</t>
-        </is>
-      </c>
-      <c r="O21" t="inlineStr">
-        <is>
-          <t>AoE</t>
-        </is>
-      </c>
-      <c r="P21" t="inlineStr"/>
-      <c r="Q21" t="inlineStr"/>
-      <c r="R21" t="inlineStr"/>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>s-p</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>S&amp;P</t>
-        </is>
-      </c>
-      <c r="C22" t="n">
-        <v>2026</v>
-      </c>
-      <c r="D22" t="n">
-        <v>2</v>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>2025-11-13</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr"/>
-      <c r="G22" t="inlineStr"/>
-      <c r="H22" t="inlineStr"/>
-      <c r="I22" t="inlineStr">
-        <is>
-          <t>2026-02-01</t>
-        </is>
-      </c>
-      <c r="J22" t="inlineStr"/>
-      <c r="K22" t="inlineStr">
-        <is>
-          <t>2026-05-18</t>
-        </is>
-      </c>
-      <c r="L22" t="inlineStr">
-        <is>
-          <t>2026-05-21</t>
-        </is>
-      </c>
-      <c r="M22" t="inlineStr">
-        <is>
-          <t>San Francisco, CA, USA</t>
-        </is>
-      </c>
-      <c r="N22" t="inlineStr">
-        <is>
-          <t>https://www.ieee-security.org/TC/SP2026/</t>
-        </is>
-      </c>
-      <c r="O22" t="inlineStr">
-        <is>
-          <t>AoE</t>
-        </is>
-      </c>
-      <c r="P22" t="inlineStr"/>
-      <c r="Q22" t="inlineStr"/>
-      <c r="R22" t="inlineStr"/>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>stoc</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>STOC</t>
-        </is>
-      </c>
-      <c r="C23" t="n">
-        <v>2026</v>
-      </c>
-      <c r="D23" t="n">
-        <v>1</v>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>2025-11-04</t>
-        </is>
-      </c>
-      <c r="F23" t="inlineStr"/>
-      <c r="G23" t="inlineStr"/>
-      <c r="H23" t="inlineStr"/>
-      <c r="I23" t="inlineStr">
-        <is>
-          <t>2026-02-01</t>
-        </is>
-      </c>
-      <c r="J23" t="inlineStr"/>
-      <c r="K23" t="inlineStr">
-        <is>
-          <t>2026-06-22</t>
-        </is>
-      </c>
-      <c r="L23" t="inlineStr">
-        <is>
-          <t>2026-06-27</t>
-        </is>
-      </c>
-      <c r="M23" t="inlineStr">
-        <is>
-          <t>Salt Lake City, UT, USA</t>
-        </is>
-      </c>
-      <c r="N23" t="inlineStr">
-        <is>
-          <t>https://acm-stoc.org/stoc2026/</t>
-        </is>
-      </c>
-      <c r="O23" t="inlineStr">
-        <is>
-          <t>US EST</t>
-        </is>
-      </c>
-      <c r="P23" t="inlineStr"/>
-      <c r="Q23" t="inlineStr"/>
-      <c r="R23" t="inlineStr"/>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>usenix-security</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>USENIX Security</t>
-        </is>
-      </c>
-      <c r="C24" t="n">
-        <v>2026</v>
-      </c>
-      <c r="D24" t="n">
-        <v>1</v>
-      </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>2025-08-26</t>
-        </is>
-      </c>
-      <c r="F24" t="inlineStr"/>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t>2025-11-06</t>
-        </is>
-      </c>
-      <c r="H24" t="inlineStr">
-        <is>
-          <t>2025-11-13</t>
-        </is>
-      </c>
-      <c r="I24" t="inlineStr">
-        <is>
-          <t>2025-12-04</t>
-        </is>
-      </c>
-      <c r="J24" t="inlineStr">
-        <is>
-          <t>2026-01-15</t>
-        </is>
-      </c>
-      <c r="K24" t="inlineStr">
-        <is>
-          <t>2026-08-12</t>
-        </is>
-      </c>
-      <c r="L24" t="inlineStr">
-        <is>
-          <t>2026-08-14</t>
-        </is>
-      </c>
-      <c r="M24" t="inlineStr">
-        <is>
-          <t>Baltimore, MD, USA</t>
-        </is>
-      </c>
-      <c r="N24" t="inlineStr">
-        <is>
-          <t>https://www.usenix.org/conference/usenixsecurity26/</t>
-        </is>
-      </c>
-      <c r="O24" t="inlineStr">
-        <is>
-          <t>AoE</t>
-        </is>
-      </c>
-      <c r="P24" t="inlineStr"/>
-      <c r="Q24" t="inlineStr"/>
-      <c r="R24" t="inlineStr"/>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>www</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>WWW</t>
-        </is>
-      </c>
-      <c r="C25" t="n">
-        <v>2026</v>
-      </c>
-      <c r="D25" t="n">
-        <v>1</v>
-      </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>2025-10-24</t>
-        </is>
-      </c>
-      <c r="F25" t="inlineStr"/>
-      <c r="G25" t="inlineStr">
-        <is>
-          <t>2026-01-06</t>
-        </is>
-      </c>
-      <c r="H25" t="inlineStr">
-        <is>
-          <t>2026-01-13</t>
-        </is>
-      </c>
-      <c r="I25" t="inlineStr">
-        <is>
-          <t>2026-01-24</t>
-        </is>
-      </c>
-      <c r="J25" t="inlineStr">
-        <is>
-          <t>2026-02-14</t>
-        </is>
-      </c>
-      <c r="K25" t="inlineStr">
-        <is>
-          <t>2026-04-19</t>
-        </is>
-      </c>
-      <c r="L25" t="inlineStr">
-        <is>
-          <t>2026-04-24</t>
-        </is>
-      </c>
-      <c r="M25" t="inlineStr">
-        <is>
-          <t>Perth, Australia</t>
-        </is>
-      </c>
-      <c r="N25" t="inlineStr">
-        <is>
-          <t>https://www2026.thewebconf.org/</t>
-        </is>
-      </c>
-      <c r="O25" t="inlineStr">
-        <is>
-          <t>AoE</t>
-        </is>
-      </c>
-      <c r="P25" t="inlineStr"/>
-      <c r="Q25" t="inlineStr"/>
-      <c r="R25" t="inlineStr"/>
+          <t>AoE</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2650,7 +1853,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R15"/>
+  <dimension ref="A1:O11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2729,83 +1932,68 @@
           <t>timezone</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
-        <is>
-          <t>submissions</t>
-        </is>
-      </c>
-      <c r="Q1" s="1" t="inlineStr">
-        <is>
-          <t>accepted</t>
-        </is>
-      </c>
-      <c r="R1" s="1" t="inlineStr">
-        <is>
-          <t>acceptance_rate</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>asiacrypt</t>
+          <t>ches</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>ASIACRYPT</t>
+          <t>CHES</t>
         </is>
       </c>
       <c r="C2" t="n">
         <v>2026</v>
       </c>
       <c r="D2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-01-15</t>
         </is>
       </c>
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-02-26</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-03-01</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-03-15</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-04-14</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>2026-12-07</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>2026-12-11</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>Hong Kong, China</t>
+          <t>Antalya, Turkiye</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>https://asiacrypt.iacr.org/2026/</t>
+          <t>https://ches.iacr.org/2026/</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
@@ -2813,75 +2001,68 @@
           <t>AoE</t>
         </is>
       </c>
-      <c r="P2" t="inlineStr"/>
-      <c r="Q2" t="inlineStr"/>
-      <c r="R2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>ccs</t>
+          <t>ches</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>CCS</t>
+          <t>CHES</t>
         </is>
       </c>
       <c r="C3" t="n">
         <v>2026</v>
       </c>
       <c r="D3" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-01-14</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>2026-01-07</t>
-        </is>
-      </c>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2026-03-17</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>2026-03-20</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>2026-11-15</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>2026-11-19</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>The Hague, Netherlands</t>
+          <t>Antalya, Turkiye</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>https://www.sigsac.org/ccs/CCS2026/</t>
+          <t>https://ches.iacr.org/2026/</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
@@ -2889,75 +2070,68 @@
           <t>AoE</t>
         </is>
       </c>
-      <c r="P3" t="inlineStr"/>
-      <c r="Q3" t="inlineStr"/>
-      <c r="R3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>ccs</t>
+          <t>crypto</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>CCS</t>
+          <t>CRYPTO</t>
         </is>
       </c>
       <c r="C4" t="n">
         <v>2026</v>
       </c>
       <c r="D4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2026-04-29</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>2026-04-22</t>
-        </is>
-      </c>
+          <t>2026-02-12</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-04-07</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>2026-11-15</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>2026-11-19</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>The Hague, Netherlands</t>
+          <t>Santa Barbara, CA, USA</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>https://www.sigsac.org/ccs/CCS2026/</t>
+          <t>https://crypto.iacr.org/2026/</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
@@ -2965,143 +2139,129 @@
           <t>AoE</t>
         </is>
       </c>
-      <c r="P4" t="inlineStr"/>
-      <c r="Q4" t="inlineStr"/>
-      <c r="R4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>ches</t>
+          <t>asiacrypt</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>CHES</t>
+          <t>ASIACRYPT</t>
         </is>
       </c>
       <c r="C5" t="n">
         <v>2026</v>
       </c>
       <c r="D5" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2026-01-15</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-02-26</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-02-26</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>2026-03-01</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2026-03-15</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-12-07</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-12-11</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>Hong Kong, China</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>Antalya, Turkiye</t>
+          <t>https://asiacrypt.iacr.org/2026/</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>https://ches.iacr.org/2026/</t>
-        </is>
-      </c>
-      <c r="P5" t="inlineStr"/>
-      <c r="Q5" t="inlineStr"/>
-      <c r="R5" t="inlineStr"/>
+          <t>AoE</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>ches</t>
+          <t>tcc</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>CHES</t>
+          <t>TCC</t>
         </is>
       </c>
       <c r="C6" t="n">
         <v>2026</v>
       </c>
       <c r="D6" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2026-01-15</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>2026-02-26</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>2026-03-01</t>
-        </is>
-      </c>
+      <c r="G6" t="inlineStr"/>
+      <c r="H6" t="inlineStr"/>
       <c r="I6" t="inlineStr">
         <is>
-          <t>2026-03-15</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-11-10</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-11-13</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>Antalya, Turkiye</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>https://ches.iacr.org/2026/</t>
+          <t>https://tcc.iacr.org/2026/</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
@@ -3109,143 +2269,145 @@
           <t>AoE</t>
         </is>
       </c>
-      <c r="P6" t="inlineStr"/>
-      <c r="Q6" t="inlineStr"/>
-      <c r="R6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>ches</t>
+          <t>ccs</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>CHES</t>
+          <t>CCS</t>
         </is>
       </c>
       <c r="C7" t="n">
         <v>2026</v>
       </c>
       <c r="D7" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr"/>
+          <t>2026-01-14</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>2026-01-07</t>
+        </is>
+      </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-03-20</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-11-15</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-11-19</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>The Hague, Netherlands</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>Antalya, Turkiye</t>
+          <t>https://www.sigsac.org/ccs/CCS2026/</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>https://ches.iacr.org/2026/</t>
-        </is>
-      </c>
-      <c r="P7" t="inlineStr"/>
-      <c r="Q7" t="inlineStr"/>
-      <c r="R7" t="inlineStr"/>
+          <t>AoE</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>ches</t>
+          <t>ccs</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>CHES</t>
+          <t>CCS</t>
         </is>
       </c>
       <c r="C8" t="n">
         <v>2026</v>
       </c>
       <c r="D8" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr"/>
+          <t>2026-04-29</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-11-15</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-11-19</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>Antalya, Turkiye</t>
+          <t>The Hague, Netherlands</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>https://ches.iacr.org/2026/</t>
+          <t>https://www.sigsac.org/ccs/CCS2026/</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
@@ -3253,19 +2415,16 @@
           <t>AoE</t>
         </is>
       </c>
-      <c r="P8" t="inlineStr"/>
-      <c r="Q8" t="inlineStr"/>
-      <c r="R8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>crypto</t>
+          <t>sigcomm</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>CRYPTO</t>
+          <t>SIGCOMM</t>
         </is>
       </c>
       <c r="C9" t="n">
@@ -3276,30 +2435,26 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2026-02-12</t>
+          <t>2026-02-06</t>
         </is>
       </c>
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-04-13</t>
+          <t>2026-04-29</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
-        </is>
-      </c>
-      <c r="J9" t="inlineStr">
-        <is>
-          <t>2026-06-08</t>
-        </is>
-      </c>
+          <t>2026-05-11</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr"/>
       <c r="K9" t="inlineStr">
         <is>
           <t>2026-08-17</t>
@@ -3307,89 +2462,74 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>Santa Barbara, CA, USA</t>
+          <t>Denver, CO, USA</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>https://crypto.iacr.org/2026/</t>
+          <t>https://conferences.sigcomm.org/sigcomm/2026/</t>
         </is>
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>US Pacific</t>
-        </is>
-      </c>
-      <c r="P9" t="inlineStr"/>
-      <c r="Q9" t="inlineStr"/>
-      <c r="R9" t="inlineStr"/>
+          <t>AoE</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>crypto</t>
+          <t>csf</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>CRYPTO</t>
+          <t>CSF</t>
         </is>
       </c>
       <c r="C10" t="n">
         <v>2026</v>
       </c>
       <c r="D10" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>2026-02-12</t>
+          <t>2026-01-29</t>
         </is>
       </c>
       <c r="F10" t="inlineStr"/>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>2026-04-07</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>2026-04-13</t>
-        </is>
-      </c>
+      <c r="G10" t="inlineStr"/>
+      <c r="H10" t="inlineStr"/>
       <c r="I10" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
-        </is>
-      </c>
-      <c r="J10" t="inlineStr">
-        <is>
-          <t>2026-06-08</t>
-        </is>
-      </c>
+          <t>2026-04-01</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr"/>
       <c r="K10" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-07-26</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>Santa Barbara, CA, USA</t>
+          <t>Lisbon, Portugal</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>https://crypto.iacr.org/2026/</t>
+          <t>https://www.ieee-security.org/TC/CSF2026/</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
@@ -3397,59 +2537,68 @@
           <t>AoE</t>
         </is>
       </c>
-      <c r="P10" t="inlineStr"/>
-      <c r="Q10" t="inlineStr"/>
-      <c r="R10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>csf</t>
+          <t>usenix-security</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>CSF</t>
+          <t>USENIX Security</t>
         </is>
       </c>
       <c r="C11" t="n">
         <v>2026</v>
       </c>
       <c r="D11" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>2026-01-29</t>
+          <t>2026-02-05</t>
         </is>
       </c>
       <c r="F11" t="inlineStr"/>
-      <c r="G11" t="inlineStr"/>
-      <c r="H11" t="inlineStr"/>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>2026-04-23</t>
+        </is>
+      </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
-        </is>
-      </c>
-      <c r="J11" t="inlineStr"/>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>2026-07-26</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>Lisbon, Portugal</t>
+          <t>Baltimore, MD, USA</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>https://www.ieee-security.org/TC/CSF2026/</t>
+          <t>https://www.usenix.org/conference/usenixsecurity26/</t>
         </is>
       </c>
       <c r="O11" t="inlineStr">
@@ -3457,273 +2606,6 @@
           <t>AoE</t>
         </is>
       </c>
-      <c r="P11" t="inlineStr"/>
-      <c r="Q11" t="inlineStr"/>
-      <c r="R11" t="inlineStr"/>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>miccai</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>MICCAI</t>
-        </is>
-      </c>
-      <c r="C12" t="n">
-        <v>2026</v>
-      </c>
-      <c r="D12" t="n">
-        <v>1</v>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>2026-02-26</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr"/>
-      <c r="G12" t="inlineStr"/>
-      <c r="H12" t="inlineStr"/>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t>2026-05-15</t>
-        </is>
-      </c>
-      <c r="J12" t="inlineStr"/>
-      <c r="K12" t="inlineStr">
-        <is>
-          <t>2026-10-04</t>
-        </is>
-      </c>
-      <c r="L12" t="inlineStr">
-        <is>
-          <t>2026-10-08</t>
-        </is>
-      </c>
-      <c r="M12" t="inlineStr">
-        <is>
-          <t>Munich, Germany</t>
-        </is>
-      </c>
-      <c r="N12" t="inlineStr">
-        <is>
-          <t>https://conferences.miccai.org/2026/</t>
-        </is>
-      </c>
-      <c r="O12" t="inlineStr">
-        <is>
-          <t>US Pacific</t>
-        </is>
-      </c>
-      <c r="P12" t="inlineStr"/>
-      <c r="Q12" t="inlineStr"/>
-      <c r="R12" t="inlineStr"/>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>sigcomm</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>SIGCOMM</t>
-        </is>
-      </c>
-      <c r="C13" t="n">
-        <v>2026</v>
-      </c>
-      <c r="D13" t="n">
-        <v>1</v>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>2026-02-06</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr"/>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>2026-04-27</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>2026-04-29</t>
-        </is>
-      </c>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>2026-05-11</t>
-        </is>
-      </c>
-      <c r="J13" t="inlineStr"/>
-      <c r="K13" t="inlineStr">
-        <is>
-          <t>2026-08-17</t>
-        </is>
-      </c>
-      <c r="L13" t="inlineStr">
-        <is>
-          <t>2026-08-21</t>
-        </is>
-      </c>
-      <c r="M13" t="inlineStr">
-        <is>
-          <t>Denver, CO, USA</t>
-        </is>
-      </c>
-      <c r="N13" t="inlineStr">
-        <is>
-          <t>https://conferences.sigcomm.org/sigcomm/2026/</t>
-        </is>
-      </c>
-      <c r="O13" t="inlineStr">
-        <is>
-          <t>AoE</t>
-        </is>
-      </c>
-      <c r="P13" t="inlineStr"/>
-      <c r="Q13" t="inlineStr"/>
-      <c r="R13" t="inlineStr"/>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>tcc</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>TCC</t>
-        </is>
-      </c>
-      <c r="C14" t="n">
-        <v>2026</v>
-      </c>
-      <c r="D14" t="n">
-        <v>1</v>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>2026-05-19</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr"/>
-      <c r="G14" t="inlineStr"/>
-      <c r="H14" t="inlineStr"/>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t>2026-08-20</t>
-        </is>
-      </c>
-      <c r="J14" t="inlineStr">
-        <is>
-          <t>2026-09-15</t>
-        </is>
-      </c>
-      <c r="K14" t="inlineStr">
-        <is>
-          <t>2026-11-10</t>
-        </is>
-      </c>
-      <c r="L14" t="inlineStr">
-        <is>
-          <t>2026-11-13</t>
-        </is>
-      </c>
-      <c r="M14" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="N14" t="inlineStr">
-        <is>
-          <t>https://tcc.iacr.org/2026/</t>
-        </is>
-      </c>
-      <c r="O14" t="inlineStr">
-        <is>
-          <t>AoE</t>
-        </is>
-      </c>
-      <c r="P14" t="inlineStr"/>
-      <c r="Q14" t="inlineStr"/>
-      <c r="R14" t="inlineStr"/>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>usenix-security</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>USENIX Security</t>
-        </is>
-      </c>
-      <c r="C15" t="n">
-        <v>2026</v>
-      </c>
-      <c r="D15" t="n">
-        <v>2</v>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>2026-02-05</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr"/>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>2026-04-16</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>2026-04-23</t>
-        </is>
-      </c>
-      <c r="I15" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="J15" t="inlineStr">
-        <is>
-          <t>2026-06-11</t>
-        </is>
-      </c>
-      <c r="K15" t="inlineStr">
-        <is>
-          <t>2026-08-12</t>
-        </is>
-      </c>
-      <c r="L15" t="inlineStr">
-        <is>
-          <t>2026-08-14</t>
-        </is>
-      </c>
-      <c r="M15" t="inlineStr">
-        <is>
-          <t>Baltimore, MD, USA</t>
-        </is>
-      </c>
-      <c r="N15" t="inlineStr">
-        <is>
-          <t>https://www.usenix.org/conference/usenixsecurity26/</t>
-        </is>
-      </c>
-      <c r="O15" t="inlineStr">
-        <is>
-          <t>AoE</t>
-        </is>
-      </c>
-      <c r="P15" t="inlineStr"/>
-      <c r="Q15" t="inlineStr"/>
-      <c r="R15" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3736,7 +2618,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R15"/>
+  <dimension ref="A1:O16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3815,21 +2697,6 @@
           <t>timezone</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
-        <is>
-          <t>submissions</t>
-        </is>
-      </c>
-      <c r="Q1" s="1" t="inlineStr">
-        <is>
-          <t>accepted</t>
-        </is>
-      </c>
-      <c r="R1" s="1" t="inlineStr">
-        <is>
-          <t>acceptance_rate</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -3899,9 +2766,6 @@
           <t>AoE</t>
         </is>
       </c>
-      <c r="P2" t="inlineStr"/>
-      <c r="Q2" t="inlineStr"/>
-      <c r="R2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -3971,139 +2835,137 @@
           <t>AoE</t>
         </is>
       </c>
-      <c r="P3" t="inlineStr"/>
-      <c r="Q3" t="inlineStr"/>
-      <c r="R3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>eurocrypt</t>
+          <t>ches</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>EUROCRYPT</t>
+          <t>CHES</t>
         </is>
       </c>
       <c r="C4" t="n">
         <v>2027</v>
       </c>
       <c r="D4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2027-01-15</t>
         </is>
       </c>
       <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr"/>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>2027-02-23</t>
+        </is>
+      </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>2026-11-30</t>
+          <t>2027-02-28</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>2026-12-05</t>
+          <t>2027-03-15</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>2027-01-18</t>
+          <t>2027-04-14</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>2027-02-08</t>
+          <t>2027-09-06</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>2027-04-11</t>
+          <t>2027-09-09</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>2027-04-15</t>
+          <t>Cancun, Mexico</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>Eindhoven, Netherlands</t>
+          <t>https://ches.iacr.org/2027/</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>https://eurocrypt.iacr.org/2027/</t>
-        </is>
-      </c>
-      <c r="P4" t="inlineStr"/>
-      <c r="Q4" t="inlineStr"/>
-      <c r="R4" t="inlineStr"/>
+          <t>AoE</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>eurocrypt</t>
+          <t>ches</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>EUROCRYPT</t>
+          <t>CHES</t>
         </is>
       </c>
       <c r="C5" t="n">
         <v>2027</v>
       </c>
       <c r="D5" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2027-04-15</t>
         </is>
       </c>
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-11-30</t>
+          <t>2027-05-23</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-12-05</t>
+          <t>2027-05-28</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>2027-01-18</t>
+          <t>2027-06-15</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2027-02-08</t>
+          <t>2027-07-14</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>2027-04-11</t>
+          <t>2027-09-06</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>2027-04-15</t>
+          <t>2027-09-09</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>Eindhoven, Netherlands</t>
+          <t>Cancun, Mexico</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>https://eurocrypt.iacr.org/2027/</t>
+          <t>https://ches.iacr.org/2027/</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
@@ -4111,9 +2973,6 @@
           <t>AoE</t>
         </is>
       </c>
-      <c r="P5" t="inlineStr"/>
-      <c r="Q5" t="inlineStr"/>
-      <c r="R5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -4183,9 +3042,6 @@
           <t>AoE</t>
         </is>
       </c>
-      <c r="P6" t="inlineStr"/>
-      <c r="Q6" t="inlineStr"/>
-      <c r="R6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -4255,9 +3111,6 @@
           <t>AoE</t>
         </is>
       </c>
-      <c r="P7" t="inlineStr"/>
-      <c r="Q7" t="inlineStr"/>
-      <c r="R7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -4327,9 +3180,6 @@
           <t>AoE</t>
         </is>
       </c>
-      <c r="P8" t="inlineStr"/>
-      <c r="Q8" t="inlineStr"/>
-      <c r="R8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -4399,19 +3249,16 @@
           <t>AoE</t>
         </is>
       </c>
-      <c r="P9" t="inlineStr"/>
-      <c r="Q9" t="inlineStr"/>
-      <c r="R9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>ndss</t>
+          <t>eurocrypt</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>NDSS</t>
+          <t>EUROCRYPT</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -4422,48 +3269,48 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-11-30</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-12-05</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2027-01-18</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2027-02-08</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>2027-03-22</t>
+          <t>2027-04-11</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>2027-03-26</t>
+          <t>2027-04-15</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>Seoul, South Korea</t>
+          <t>Eindhoven, Netherlands</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>https://www.ndss-symposium.org/ndss2027/submissions/call-for-papers/</t>
+          <t>https://eurocrypt.iacr.org/2027/</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
@@ -4471,63 +3318,68 @@
           <t>AoE</t>
         </is>
       </c>
-      <c r="P10" t="inlineStr"/>
-      <c r="Q10" t="inlineStr"/>
-      <c r="R10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>ndss</t>
+          <t>s-p</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>NDSS</t>
+          <t>S&amp;P</t>
         </is>
       </c>
       <c r="C11" t="n">
         <v>2027</v>
       </c>
       <c r="D11" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="F11" t="inlineStr"/>
-      <c r="G11" t="inlineStr"/>
-      <c r="H11" t="inlineStr"/>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>2026-11-04</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>2027-01-06</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>2027-03-22</t>
+          <t>2027-05-01</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>2027-03-26</t>
+          <t>2027-05-04</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>Seoul, South Korea</t>
+          <t>Montreal, Canada</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>https://www.ndss-symposium.org/ndss2027/submissions/call-for-papers/</t>
+          <t>https://sp2027.ieee-security.org/</t>
         </is>
       </c>
       <c r="O11" t="inlineStr">
@@ -4535,9 +3387,6 @@
           <t>AoE</t>
         </is>
       </c>
-      <c r="P11" t="inlineStr"/>
-      <c r="Q11" t="inlineStr"/>
-      <c r="R11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -4554,32 +3403,32 @@
         <v>2027</v>
       </c>
       <c r="D12" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-11-17</t>
         </is>
       </c>
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2027-02-11</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2027-02-16</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2027-03-05</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2027-04-08</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
@@ -4607,71 +3456,68 @@
           <t>AoE</t>
         </is>
       </c>
-      <c r="P12" t="inlineStr"/>
-      <c r="Q12" t="inlineStr"/>
-      <c r="R12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>s-p</t>
+          <t>usenix-security</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>S&amp;P</t>
+          <t>USENIX Security</t>
         </is>
       </c>
       <c r="C13" t="n">
         <v>2027</v>
       </c>
       <c r="D13" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>2026-11-17</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr">
         <is>
-          <t>2027-02-11</t>
+          <t>2026-11-05</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2027-02-16</t>
+          <t>2026-11-12</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>2027-03-05</t>
+          <t>2026-12-03</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>2027-04-08</t>
+          <t>2027-01-14</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>2027-05-01</t>
+          <t>2027-08-11</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>2027-05-04</t>
+          <t>2027-08-13</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>Montreal, Canada</t>
+          <t>Denver, CO, USA</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>https://sp2027.ieee-security.org/</t>
+          <t>https://www.usenix.org/conference/usenixsecurity27/</t>
         </is>
       </c>
       <c r="O13" t="inlineStr">
@@ -4679,9 +3525,6 @@
           <t>AoE</t>
         </is>
       </c>
-      <c r="P13" t="inlineStr"/>
-      <c r="Q13" t="inlineStr"/>
-      <c r="R13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -4698,68 +3541,69 @@
         <v>2027</v>
       </c>
       <c r="D14" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2027-01-26</t>
         </is>
       </c>
       <c r="F14" t="inlineStr"/>
-      <c r="G14" t="inlineStr"/>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>2027-04-08</t>
+        </is>
+      </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-11-05</t>
+          <t>2027-04-15</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>2026-11-12</t>
+          <t>2027-05-06</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>2026-12-03</t>
+          <t>2027-06-03</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>2027-08-12</t>
+          <t>2027-08-11</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>2027-08-11</t>
+          <t>2027-08-13</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>2027-08-13</t>
+          <t>Denver, CO, USA</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>Denver, CO, USA</t>
+          <t>https://www.usenix.org/conference/usenixsecurity27/</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>https://www.usenix.org/conference/usenixsecurity27/</t>
-        </is>
-      </c>
-      <c r="P14" t="inlineStr"/>
-      <c r="Q14" t="inlineStr"/>
-      <c r="R14" t="inlineStr"/>
+          <t>AoE</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>usenix-security</t>
+          <t>ndss</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>USENIX Security</t>
+          <t>NDSS</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -4770,48 +3614,48 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr">
         <is>
-          <t>2026-11-05</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-11-12</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>2026-12-03</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>2027-01-14</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>2027-08-11</t>
+          <t>2027-03-22</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>2027-08-13</t>
+          <t>2027-03-26</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>Denver, CO, USA</t>
+          <t>Seoul, South Korea</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>https://www.usenix.org/conference/usenixsecurity27/</t>
+          <t>https://www.ndss-symposium.org/ndss2027/submissions/call-for-papers/</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
@@ -4819,9 +3663,67 @@
           <t>AoE</t>
         </is>
       </c>
-      <c r="P15" t="inlineStr"/>
-      <c r="Q15" t="inlineStr"/>
-      <c r="R15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>ndss</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>NDSS</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>2027</v>
+      </c>
+      <c r="D16" t="n">
+        <v>2</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr"/>
+      <c r="G16" t="inlineStr"/>
+      <c r="H16" t="inlineStr"/>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>2026-11-04</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>2027-01-06</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>2027-03-22</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>2027-03-26</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>Seoul, South Korea</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>https://www.ndss-symposium.org/ndss2027/submissions/call-for-papers/</t>
+        </is>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add ICML, NeurIPS, ICLR, ACL 2026 from official sources
</commit_message>
<xml_diff>
--- a/timeline_data.xlsx
+++ b/timeline_data.xlsx
@@ -726,7 +726,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O17"/>
+  <dimension ref="A1:O18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1837,6 +1837,67 @@
         </is>
       </c>
       <c r="O17" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>iclr</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>ICLR</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D18" t="n">
+        <v>1</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>2025-09-24</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>2025-09-19</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr"/>
+      <c r="H18" t="inlineStr"/>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>2026-01-25</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr"/>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>2026-04-23</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>2026-04-25</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>https://iclr.cc/Conferences/2026/</t>
+        </is>
+      </c>
+      <c r="O18" t="inlineStr">
         <is>
           <t>AoE</t>
         </is>
@@ -1853,7 +1914,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O11"/>
+  <dimension ref="A1:O14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2602,6 +2663,193 @@
         </is>
       </c>
       <c r="O11" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>icml</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>ICML</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D12" t="n">
+        <v>1</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>2026-01-28</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>2026-01-23</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr"/>
+      <c r="H12" t="inlineStr"/>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>2026-04-30</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>Seoul, South Korea</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>https://icml.cc/Conferences/2026/</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>neurips</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>NeurIPS</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D13" t="n">
+        <v>1</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>2026-05-04</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr"/>
+      <c r="H13" t="inlineStr"/>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr"/>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>2026-12-11</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>2026-12-13</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>Sydney, Australia</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>https://neurips.cc/Conferences/2026/</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>acl</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>ACL</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D14" t="n">
+        <v>1</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>2026-01-05</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr"/>
+      <c r="G14" t="inlineStr"/>
+      <c r="H14" t="inlineStr"/>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>2026-04-04</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>2026-04-19</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>San Diego, CA, USA</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>https://2026.aclweb.org/</t>
+        </is>
+      </c>
+      <c r="O14" t="inlineStr">
         <is>
           <t>AoE</t>
         </is>

</xml_diff>

<commit_message>
Add CVPR 2026, ICCV 2025 from official sources
</commit_message>
<xml_diff>
--- a/timeline_data.xlsx
+++ b/timeline_data.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O4"/>
+  <dimension ref="A1:O5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -710,6 +710,71 @@
         </is>
       </c>
       <c r="O4" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>iccv</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>ICCV</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>2025-03-07</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>2025-05-09</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>2025-05-16</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>2025-06-25</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>2025-10-19</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>2025-10-23</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>Honolulu, HI, USA</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>https://iccv.thecvf.com/Conferences/2025/</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
         <is>
           <t>AoE</t>
         </is>
@@ -726,7 +791,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O18"/>
+  <dimension ref="A1:O19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1898,6 +1963,75 @@
         </is>
       </c>
       <c r="O18" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>cvpr</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>CVPR</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D19" t="n">
+        <v>1</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>2025-11-13</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>2025-11-07</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>2026-01-22</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>2026-01-29</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>2026-02-20</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr"/>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>https://cvpr.thecvf.com/Conferences/2026/</t>
+        </is>
+      </c>
+      <c r="O19" t="inlineStr">
         <is>
           <t>AoE</t>
         </is>

</xml_diff>

<commit_message>
Add EMNLP 2026, IJCAI 2026
</commit_message>
<xml_diff>
--- a/timeline_data.xlsx
+++ b/timeline_data.xlsx
@@ -2048,7 +2048,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O14"/>
+  <dimension ref="A1:O16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2984,6 +2984,120 @@
         </is>
       </c>
       <c r="O14" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>emnlp</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>EMNLP</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D15" t="n">
+        <v>1</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr"/>
+      <c r="G15" t="inlineStr"/>
+      <c r="H15" t="inlineStr"/>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr"/>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>Budapest, Hungary</t>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>https://2026.emnlp.org/</t>
+        </is>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>ijcai</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>IJCAI</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D16" t="n">
+        <v>1</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>2026-01-19</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr"/>
+      <c r="G16" t="inlineStr"/>
+      <c r="H16" t="inlineStr"/>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr"/>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>Bremen, Germany</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>https://ijcai-26.org/</t>
+        </is>
+      </c>
+      <c r="O16" t="inlineStr">
         <is>
           <t>AoE</t>
         </is>

</xml_diff>

<commit_message>
Add STOC 2026, ICRA 2026
</commit_message>
<xml_diff>
--- a/timeline_data.xlsx
+++ b/timeline_data.xlsx
@@ -791,7 +791,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O19"/>
+  <dimension ref="A1:O21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2013,25 +2013,143 @@
       <c r="J19" t="inlineStr"/>
       <c r="K19" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
+          <t>Nashville, TN, USA</t>
+        </is>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>https://cvpr.thecvf.com/Conferences/2026/</t>
+        </is>
+      </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>stoc</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>STOC</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D20" t="n">
+        <v>1</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>2025-11-04</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr"/>
+      <c r="G20" t="inlineStr"/>
+      <c r="H20" t="inlineStr"/>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>2026-02-01</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>2026-03-31</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>Salt Lake City, UT, USA</t>
+        </is>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>https://acm-stoc.org/stoc2026/</t>
+        </is>
+      </c>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>US EST</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>icra</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>ICRA</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D21" t="n">
+        <v>1</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>2025-09-15</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr"/>
+      <c r="G21" t="inlineStr"/>
+      <c r="H21" t="inlineStr"/>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>2026-01-15</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr"/>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
           <t>TBD</t>
         </is>
       </c>
-      <c r="N19" t="inlineStr">
-        <is>
-          <t>https://cvpr.thecvf.com/Conferences/2026/</t>
-        </is>
-      </c>
-      <c r="O19" t="inlineStr">
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>https://2026.ieee-icra.org/</t>
+        </is>
+      </c>
+      <c r="O21" t="inlineStr">
         <is>
           <t>AoE</t>
         </is>

</xml_diff>

<commit_message>
Add PLDI 2026, POPL 2026 (2025submit-2026conf group)
</commit_message>
<xml_diff>
--- a/timeline_data.xlsx
+++ b/timeline_data.xlsx
@@ -791,7 +791,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O21"/>
+  <dimension ref="A1:O23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2150,6 +2150,120 @@
         </is>
       </c>
       <c r="O21" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>pldi</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>PLDI</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D22" t="n">
+        <v>1</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>2025-11-13</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr"/>
+      <c r="G22" t="inlineStr"/>
+      <c r="H22" t="inlineStr"/>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>2026-03-05</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr"/>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>Boulder, CO, USA</t>
+        </is>
+      </c>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>https://pldi26.sigplan.org/</t>
+        </is>
+      </c>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>popl</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>POPL</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D23" t="n">
+        <v>1</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>2025-07-11</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr"/>
+      <c r="G23" t="inlineStr"/>
+      <c r="H23" t="inlineStr"/>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>2025-10-01</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr"/>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>2026-01-20</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>2026-01-22</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>Philadelphia, PA, USA</t>
+        </is>
+      </c>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>https://popl.sigplan.org/</t>
+        </is>
+      </c>
+      <c r="O23" t="inlineStr">
         <is>
           <t>AoE</t>
         </is>

</xml_diff>

<commit_message>
Add OSDI 2026, CHI 2027 from official sources
</commit_message>
<xml_diff>
--- a/timeline_data.xlsx
+++ b/timeline_data.xlsx
@@ -791,7 +791,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O23"/>
+  <dimension ref="A1:O24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2266,6 +2266,71 @@
       <c r="O23" t="inlineStr">
         <is>
           <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>osdi</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>OSDI</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D24" t="n">
+        <v>1</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>2025-12-11</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>2025-12-04</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr"/>
+      <c r="H24" t="inlineStr"/>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>Seattle, WA, USA</t>
+        </is>
+      </c>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>https://www.usenix.org/conference/osdi26/</t>
+        </is>
+      </c>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>US EST</t>
         </is>
       </c>
     </row>
@@ -3476,7 +3541,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O16"/>
+  <dimension ref="A1:O17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4583,6 +4648,63 @@
         </is>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>chi</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>CHI</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>2027</v>
+      </c>
+      <c r="D17" t="n">
+        <v>1</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr"/>
+      <c r="G17" t="inlineStr"/>
+      <c r="H17" t="inlineStr"/>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>2026-12-01</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr"/>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>2027-05-10</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>2027-05-14</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>Pittsburgh, PA, USA</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>https://chi2027.acm.org/</t>
+        </is>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add ISCA 2026, SIGMOD 2026 (4 rounds) from official sources
</commit_message>
<xml_diff>
--- a/timeline_data.xlsx
+++ b/timeline_data.xlsx
@@ -791,7 +791,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O24"/>
+  <dimension ref="A1:O29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2331,6 +2331,327 @@
       <c r="O24" t="inlineStr">
         <is>
           <t>US EST</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>isca</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>ISCA</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D25" t="n">
+        <v>1</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>2025-11-17</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>2025-11-10</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>2026-02-16</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>2026-03-06</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr"/>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>Raleigh, NC, USA</t>
+        </is>
+      </c>
+      <c r="N25" t="inlineStr">
+        <is>
+          <t>https://www.iscaconf.org/isca2026/</t>
+        </is>
+      </c>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>sigmod</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>SIGMOD</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D26" t="n">
+        <v>1</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>2025-01-17</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>2025-01-10</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr"/>
+      <c r="H26" t="inlineStr"/>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>2025-05-02</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr"/>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>Bengaluru, India</t>
+        </is>
+      </c>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t>https://2026.sigmod.org/</t>
+        </is>
+      </c>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>sigmod</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>SIGMOD</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D27" t="n">
+        <v>2</v>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>2025-04-17</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>2025-04-10</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr"/>
+      <c r="H27" t="inlineStr"/>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>2025-08-01</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr"/>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>Bengaluru, India</t>
+        </is>
+      </c>
+      <c r="N27" t="inlineStr">
+        <is>
+          <t>https://2026.sigmod.org/</t>
+        </is>
+      </c>
+      <c r="O27" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>sigmod</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>SIGMOD</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D28" t="n">
+        <v>3</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>2025-07-17</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>2025-07-10</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr"/>
+      <c r="H28" t="inlineStr"/>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>2025-11-01</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr"/>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>Bengaluru, India</t>
+        </is>
+      </c>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>https://2026.sigmod.org/</t>
+        </is>
+      </c>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>sigmod</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>SIGMOD</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D29" t="n">
+        <v>4</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>2025-10-17</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>2025-10-10</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>2025-12-01</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>2025-12-08</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>2026-01-30</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr"/>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>Bengaluru, India</t>
+        </is>
+      </c>
+      <c r="N29" t="inlineStr">
+        <is>
+          <t>https://2026.sigmod.org/</t>
+        </is>
+      </c>
+      <c r="O29" t="inlineStr">
+        <is>
+          <t>AoE</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add SIGGRAPH 2026 from official source
</commit_message>
<xml_diff>
--- a/timeline_data.xlsx
+++ b/timeline_data.xlsx
@@ -2666,7 +2666,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O18"/>
+  <dimension ref="A1:O19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3846,6 +3846,63 @@
         </is>
       </c>
       <c r="O18" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>siggraph</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>SIGGRAPH</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D19" t="n">
+        <v>1</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>2026-01-15</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr"/>
+      <c r="G19" t="inlineStr"/>
+      <c r="H19" t="inlineStr"/>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>2026-03-01</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr"/>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>2026-07-19</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>Los Angeles, CA, USA</t>
+        </is>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>https://siggraph2026.nnja.co/</t>
+        </is>
+      </c>
+      <c r="O19" t="inlineStr">
         <is>
           <t>AoE</t>
         </is>

</xml_diff>

<commit_message>
Add FAST 2026 (2x), NSDI 2026 (2x) from official sources
</commit_message>
<xml_diff>
--- a/timeline_data.xlsx
+++ b/timeline_data.xlsx
@@ -791,7 +791,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O29"/>
+  <dimension ref="A1:O33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2406,12 +2406,12 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>sigmod</t>
+          <t>fast</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>SIGMOD</t>
+          <t>FAST</t>
         </is>
       </c>
       <c r="C26" t="n">
@@ -2422,40 +2422,48 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>2025-01-17</t>
-        </is>
-      </c>
-      <c r="F26" t="inlineStr">
-        <is>
-          <t>2025-01-10</t>
-        </is>
-      </c>
-      <c r="G26" t="inlineStr"/>
-      <c r="H26" t="inlineStr"/>
+          <t>2025-03-18</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr"/>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>2025-05-20</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>2025-05-22</t>
+        </is>
+      </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>2025-05-02</t>
-        </is>
-      </c>
-      <c r="J26" t="inlineStr"/>
+          <t>2025-06-05</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>2025-07-29</t>
+        </is>
+      </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-02-24</t>
         </is>
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-02-26</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>Bengaluru, India</t>
+          <t>Santa Clara, CA, USA</t>
         </is>
       </c>
       <c r="N26" t="inlineStr">
         <is>
-          <t>https://2026.sigmod.org/</t>
+          <t>https://www.usenix.org/conference/fast26/</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
@@ -2467,12 +2475,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>sigmod</t>
+          <t>fast</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>SIGMOD</t>
+          <t>FAST</t>
         </is>
       </c>
       <c r="C27" t="n">
@@ -2483,40 +2491,48 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>2025-04-17</t>
-        </is>
-      </c>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>2025-04-10</t>
-        </is>
-      </c>
-      <c r="G27" t="inlineStr"/>
-      <c r="H27" t="inlineStr"/>
+          <t>2025-09-16</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr"/>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>2025-11-18</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>2025-11-20</t>
+        </is>
+      </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>2025-08-01</t>
-        </is>
-      </c>
-      <c r="J27" t="inlineStr"/>
+          <t>2025-12-08</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>2026-01-27</t>
+        </is>
+      </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-02-24</t>
         </is>
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-02-26</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>Bengaluru, India</t>
+          <t>Santa Clara, CA, USA</t>
         </is>
       </c>
       <c r="N27" t="inlineStr">
         <is>
-          <t>https://2026.sigmod.org/</t>
+          <t>https://www.usenix.org/conference/fast26/</t>
         </is>
       </c>
       <c r="O27" t="inlineStr">
@@ -2528,128 +2544,380 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>sigmod</t>
+          <t>nsdi</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>SIGMOD</t>
+          <t>NSDI</t>
         </is>
       </c>
       <c r="C28" t="n">
         <v>2026</v>
       </c>
       <c r="D28" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>2025-07-17</t>
+          <t>2025-04-25</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>2025-07-10</t>
+          <t>2025-04-18</t>
         </is>
       </c>
       <c r="G28" t="inlineStr"/>
       <c r="H28" t="inlineStr"/>
       <c r="I28" t="inlineStr">
         <is>
-          <t>2025-11-01</t>
-        </is>
-      </c>
-      <c r="J28" t="inlineStr"/>
+          <t>2025-07-24</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>2025-10-21</t>
+        </is>
+      </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t>Bengaluru, India</t>
+          <t>Renton, WA, USA</t>
         </is>
       </c>
       <c r="N28" t="inlineStr">
         <is>
-          <t>https://2026.sigmod.org/</t>
+          <t>https://www.usenix.org/conference/nsdi26/</t>
         </is>
       </c>
       <c r="O28" t="inlineStr">
         <is>
-          <t>AoE</t>
+          <t>US PDT</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>sigmod</t>
+          <t>nsdi</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>SIGMOD</t>
+          <t>NSDI</t>
         </is>
       </c>
       <c r="C29" t="n">
         <v>2026</v>
       </c>
       <c r="D29" t="n">
+        <v>2</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>2025-09-18</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>2025-09-11</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr"/>
+      <c r="H29" t="inlineStr"/>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>2025-12-09</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>2026-03-05</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>2026-05-04</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>Renton, WA, USA</t>
+        </is>
+      </c>
+      <c r="N29" t="inlineStr">
+        <is>
+          <t>https://www.usenix.org/conference/nsdi26/</t>
+        </is>
+      </c>
+      <c r="O29" t="inlineStr">
+        <is>
+          <t>US PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>sigmod</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>SIGMOD</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D30" t="n">
+        <v>1</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>2025-01-17</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>2025-01-10</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr"/>
+      <c r="H30" t="inlineStr"/>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>2025-05-02</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr"/>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t>Bengaluru, India</t>
+        </is>
+      </c>
+      <c r="N30" t="inlineStr">
+        <is>
+          <t>https://2026.sigmod.org/</t>
+        </is>
+      </c>
+      <c r="O30" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>sigmod</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>SIGMOD</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D31" t="n">
+        <v>2</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>2025-04-17</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>2025-04-10</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr"/>
+      <c r="H31" t="inlineStr"/>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>2025-08-01</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr"/>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>Bengaluru, India</t>
+        </is>
+      </c>
+      <c r="N31" t="inlineStr">
+        <is>
+          <t>https://2026.sigmod.org/</t>
+        </is>
+      </c>
+      <c r="O31" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>sigmod</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>SIGMOD</t>
+        </is>
+      </c>
+      <c r="C32" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D32" t="n">
+        <v>3</v>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>2025-07-17</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>2025-07-10</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr"/>
+      <c r="H32" t="inlineStr"/>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>2025-11-01</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr"/>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>Bengaluru, India</t>
+        </is>
+      </c>
+      <c r="N32" t="inlineStr">
+        <is>
+          <t>https://2026.sigmod.org/</t>
+        </is>
+      </c>
+      <c r="O32" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>sigmod</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>SIGMOD</t>
+        </is>
+      </c>
+      <c r="C33" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D33" t="n">
         <v>4</v>
       </c>
-      <c r="E29" t="inlineStr">
+      <c r="E33" t="inlineStr">
         <is>
           <t>2025-10-17</t>
         </is>
       </c>
-      <c r="F29" t="inlineStr">
+      <c r="F33" t="inlineStr">
         <is>
           <t>2025-10-10</t>
         </is>
       </c>
-      <c r="G29" t="inlineStr">
+      <c r="G33" t="inlineStr">
         <is>
           <t>2025-12-01</t>
         </is>
       </c>
-      <c r="H29" t="inlineStr">
+      <c r="H33" t="inlineStr">
         <is>
           <t>2025-12-08</t>
         </is>
       </c>
-      <c r="I29" t="inlineStr">
+      <c r="I33" t="inlineStr">
         <is>
           <t>2026-01-30</t>
         </is>
       </c>
-      <c r="J29" t="inlineStr"/>
-      <c r="K29" t="inlineStr">
+      <c r="J33" t="inlineStr"/>
+      <c r="K33" t="inlineStr">
         <is>
           <t>2026-05-31</t>
         </is>
       </c>
-      <c r="L29" t="inlineStr">
+      <c r="L33" t="inlineStr">
         <is>
           <t>2026-06-05</t>
         </is>
       </c>
-      <c r="M29" t="inlineStr">
+      <c r="M33" t="inlineStr">
         <is>
           <t>Bengaluru, India</t>
         </is>
       </c>
-      <c r="N29" t="inlineStr">
+      <c r="N33" t="inlineStr">
         <is>
           <t>https://2026.sigmod.org/</t>
         </is>
       </c>
-      <c r="O29" t="inlineStr">
+      <c r="O33" t="inlineStr">
         <is>
           <t>AoE</t>
         </is>

</xml_diff>

<commit_message>
Add SC 2026 from official source
</commit_message>
<xml_diff>
--- a/timeline_data.xlsx
+++ b/timeline_data.xlsx
@@ -2934,7 +2934,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O21"/>
+  <dimension ref="A1:O22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4299,6 +4299,79 @@
       <c r="O21" t="inlineStr">
         <is>
           <t>US Pacific</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>sc</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D22" t="n">
+        <v>1</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>2026-04-08</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>2026-04-01</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>2026-11-15</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>2026-11-20</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>Chicago, IL, USA</t>
+        </is>
+      </c>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>https://sc26.supercomputing.org/</t>
+        </is>
+      </c>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>AoE</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add HPCA 2026 from official source
</commit_message>
<xml_diff>
--- a/timeline_data.xlsx
+++ b/timeline_data.xlsx
@@ -791,7 +791,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O33"/>
+  <dimension ref="A1:O34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2674,12 +2674,12 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>sigmod</t>
+          <t>hpca</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>SIGMOD</t>
+          <t>HPCA</t>
         </is>
       </c>
       <c r="C30" t="n">
@@ -2690,40 +2690,52 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>2025-01-17</t>
+          <t>2025-08-01</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>2025-01-10</t>
-        </is>
-      </c>
-      <c r="G30" t="inlineStr"/>
-      <c r="H30" t="inlineStr"/>
+          <t>2025-07-25</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>2025-10-07</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>2025-10-20</t>
+        </is>
+      </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>2025-05-02</t>
-        </is>
-      </c>
-      <c r="J30" t="inlineStr"/>
+          <t>2025-11-07</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>2025-12-04</t>
+        </is>
+      </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-02-25</t>
         </is>
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-03-01</t>
         </is>
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t>Bengaluru, India</t>
+          <t>Sydney, Australia</t>
         </is>
       </c>
       <c r="N30" t="inlineStr">
         <is>
-          <t>https://2026.sigmod.org/</t>
+          <t>https://hpca-conf.org/</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
@@ -2747,23 +2759,23 @@
         <v>2026</v>
       </c>
       <c r="D31" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>2025-04-17</t>
+          <t>2025-01-17</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>2025-04-10</t>
+          <t>2025-01-10</t>
         </is>
       </c>
       <c r="G31" t="inlineStr"/>
       <c r="H31" t="inlineStr"/>
       <c r="I31" t="inlineStr">
         <is>
-          <t>2025-08-01</t>
+          <t>2025-05-02</t>
         </is>
       </c>
       <c r="J31" t="inlineStr"/>
@@ -2808,23 +2820,23 @@
         <v>2026</v>
       </c>
       <c r="D32" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>2025-07-17</t>
+          <t>2025-04-17</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>2025-07-10</t>
+          <t>2025-04-10</t>
         </is>
       </c>
       <c r="G32" t="inlineStr"/>
       <c r="H32" t="inlineStr"/>
       <c r="I32" t="inlineStr">
         <is>
-          <t>2025-11-01</t>
+          <t>2025-08-01</t>
         </is>
       </c>
       <c r="J32" t="inlineStr"/>
@@ -2869,31 +2881,23 @@
         <v>2026</v>
       </c>
       <c r="D33" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>2025-10-17</t>
+          <t>2025-07-17</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>2025-10-10</t>
-        </is>
-      </c>
-      <c r="G33" t="inlineStr">
-        <is>
-          <t>2025-12-01</t>
-        </is>
-      </c>
-      <c r="H33" t="inlineStr">
-        <is>
-          <t>2025-12-08</t>
-        </is>
-      </c>
+          <t>2025-07-10</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr"/>
+      <c r="H33" t="inlineStr"/>
       <c r="I33" t="inlineStr">
         <is>
-          <t>2026-01-30</t>
+          <t>2025-11-01</t>
         </is>
       </c>
       <c r="J33" t="inlineStr"/>
@@ -2918,6 +2922,75 @@
         </is>
       </c>
       <c r="O33" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>sigmod</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>SIGMOD</t>
+        </is>
+      </c>
+      <c r="C34" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D34" t="n">
+        <v>4</v>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>2025-10-17</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>2025-10-10</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>2025-12-01</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>2025-12-08</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>2026-01-30</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr"/>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="M34" t="inlineStr">
+        <is>
+          <t>Bengaluru, India</t>
+        </is>
+      </c>
+      <c r="N34" t="inlineStr">
+        <is>
+          <t>https://2026.sigmod.org/</t>
+        </is>
+      </c>
+      <c r="O34" t="inlineStr">
         <is>
           <t>AoE</t>
         </is>

</xml_diff>

<commit_message>
Add VLDB 2026 from official source
</commit_message>
<xml_diff>
--- a/timeline_data.xlsx
+++ b/timeline_data.xlsx
@@ -3007,7 +3007,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O22"/>
+  <dimension ref="A1:O23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4443,6 +4443,63 @@
         </is>
       </c>
       <c r="O22" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>vldb</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>VLDB</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D23" t="n">
+        <v>1</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>2026-04-01</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr"/>
+      <c r="G23" t="inlineStr"/>
+      <c r="H23" t="inlineStr"/>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr"/>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>Boston, MA, USA</t>
+        </is>
+      </c>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>https://vldb.org/2026/</t>
+        </is>
+      </c>
+      <c r="O23" t="inlineStr">
         <is>
           <t>AoE</t>
         </is>

</xml_diff>

<commit_message>
Add SOSP 2026 from official source
</commit_message>
<xml_diff>
--- a/timeline_data.xlsx
+++ b/timeline_data.xlsx
@@ -3007,7 +3007,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O23"/>
+  <dimension ref="A1:O24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4500,6 +4500,71 @@
         </is>
       </c>
       <c r="O23" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>sosp</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>SOSP</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D24" t="n">
+        <v>1</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>2026-04-01</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr"/>
+      <c r="H24" t="inlineStr"/>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>Prague, Czech Republic</t>
+        </is>
+      </c>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>https://sigops.org/s/conferences/sosp/2026/</t>
+        </is>
+      </c>
+      <c r="O24" t="inlineStr">
         <is>
           <t>AoE</t>
         </is>

</xml_diff>

<commit_message>
Add OOPSLA 2026 (2x), ISSTA 2026 from official sources
</commit_message>
<xml_diff>
--- a/timeline_data.xlsx
+++ b/timeline_data.xlsx
@@ -3007,7 +3007,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O24"/>
+  <dimension ref="A1:O27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4565,6 +4565,181 @@
         </is>
       </c>
       <c r="O24" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>oopsla</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>OOPSLA</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D25" t="n">
+        <v>1</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>2025-10-10</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr"/>
+      <c r="G25" t="inlineStr"/>
+      <c r="H25" t="inlineStr"/>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>2026-02-17</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr"/>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>Oakland, CA, USA</t>
+        </is>
+      </c>
+      <c r="N25" t="inlineStr">
+        <is>
+          <t>https://2026.splashcon.org/track/splash-2026/oopsla-2026</t>
+        </is>
+      </c>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>oopsla</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>OOPSLA</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D26" t="n">
+        <v>2</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>2026-03-17</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr"/>
+      <c r="G26" t="inlineStr"/>
+      <c r="H26" t="inlineStr"/>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>Oakland, CA, USA</t>
+        </is>
+      </c>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t>https://2026.splashcon.org/track/splash-2026/oopsla-2026</t>
+        </is>
+      </c>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>issta</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>ISSTA</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D27" t="n">
+        <v>1</v>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>2026-01-29</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr"/>
+      <c r="G27" t="inlineStr"/>
+      <c r="H27" t="inlineStr"/>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr"/>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>Nanjing, China</t>
+        </is>
+      </c>
+      <c r="N27" t="inlineStr">
+        <is>
+          <t>https://conf.researchr.org/home/issta-2026</t>
+        </is>
+      </c>
+      <c r="O27" t="inlineStr">
         <is>
           <t>AoE</t>
         </is>

</xml_diff>

<commit_message>
Add DAC 2026 from official source
</commit_message>
<xml_diff>
--- a/timeline_data.xlsx
+++ b/timeline_data.xlsx
@@ -3007,7 +3007,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O27"/>
+  <dimension ref="A1:O28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4740,6 +4740,63 @@
         </is>
       </c>
       <c r="O27" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>dac</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>DAC</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D28" t="n">
+        <v>1</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>2026-01-20</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr"/>
+      <c r="G28" t="inlineStr"/>
+      <c r="H28" t="inlineStr"/>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>2026-03-01</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr"/>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>Long Beach, CA, USA</t>
+        </is>
+      </c>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>https://dac.com/2026</t>
+        </is>
+      </c>
+      <c r="O28" t="inlineStr">
         <is>
           <t>AoE</t>
         </is>

</xml_diff>

<commit_message>
Combined: CSCW 2026 + ICCAD 2026
</commit_message>
<xml_diff>
--- a/timeline_data.xlsx
+++ b/timeline_data.xlsx
@@ -791,7 +791,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O34"/>
+  <dimension ref="A1:O35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2991,6 +2991,63 @@
         </is>
       </c>
       <c r="O34" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>cscw</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>CSCW</t>
+        </is>
+      </c>
+      <c r="C35" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D35" t="n">
+        <v>1</v>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>2025-05-14</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr"/>
+      <c r="G35" t="inlineStr"/>
+      <c r="H35" t="inlineStr"/>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>2025-08-19</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr"/>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="M35" t="inlineStr">
+        <is>
+          <t>Salt Lake City, UT, USA</t>
+        </is>
+      </c>
+      <c r="N35" t="inlineStr">
+        <is>
+          <t>https://cscw.acm.org/2026/</t>
+        </is>
+      </c>
+      <c r="O35" t="inlineStr">
         <is>
           <t>AoE</t>
         </is>

</xml_diff>

<commit_message>
Combined: CSCW 2026 + ICCAD 2026 + ECCV 2026
</commit_message>
<xml_diff>
--- a/timeline_data.xlsx
+++ b/timeline_data.xlsx
@@ -791,7 +791,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O34"/>
+  <dimension ref="A1:O35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2991,6 +2991,63 @@
         </is>
       </c>
       <c r="O34" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>cscw</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>CSCW</t>
+        </is>
+      </c>
+      <c r="C35" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D35" t="n">
+        <v>1</v>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>2025-05-14</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr"/>
+      <c r="G35" t="inlineStr"/>
+      <c r="H35" t="inlineStr"/>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>2025-08-19</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr"/>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="M35" t="inlineStr">
+        <is>
+          <t>Salt Lake City, UT, USA</t>
+        </is>
+      </c>
+      <c r="N35" t="inlineStr">
+        <is>
+          <t>https://cscw.acm.org/2026/</t>
+        </is>
+      </c>
+      <c r="O35" t="inlineStr">
         <is>
           <t>AoE</t>
         </is>
@@ -3007,7 +3064,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O29"/>
+  <dimension ref="A1:O30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4805,12 +4862,12 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>eccv</t>
+          <t>iccad</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>ECCV</t>
+          <t>ICCAD</t>
         </is>
       </c>
       <c r="C29" t="n">
@@ -4821,55 +4878,120 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>2026-04-07</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr"/>
+      <c r="H29" t="inlineStr"/>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>2026-11-08</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>2026-11-12</t>
+        </is>
+      </c>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>San Jose, CA, USA</t>
+        </is>
+      </c>
+      <c r="N29" t="inlineStr">
+        <is>
+          <t>https://iccad.com/2026</t>
+        </is>
+      </c>
+      <c r="O29" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>eccv</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>ECCV</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D30" t="n">
+        <v>1</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
           <t>2026-03-05</t>
         </is>
       </c>
-      <c r="F29" t="inlineStr">
+      <c r="F30" t="inlineStr">
         <is>
           <t>2026-02-26</t>
         </is>
       </c>
-      <c r="G29" t="inlineStr">
+      <c r="G30" t="inlineStr">
         <is>
           <t>2026-05-02</t>
         </is>
       </c>
-      <c r="H29" t="inlineStr">
+      <c r="H30" t="inlineStr">
         <is>
           <t>2026-05-11</t>
         </is>
       </c>
-      <c r="I29" t="inlineStr">
+      <c r="I30" t="inlineStr">
         <is>
           <t>2026-06-17</t>
         </is>
       </c>
-      <c r="J29" t="inlineStr">
+      <c r="J30" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
       </c>
-      <c r="K29" t="inlineStr">
+      <c r="K30" t="inlineStr">
         <is>
           <t>2026-09-08</t>
         </is>
       </c>
-      <c r="L29" t="inlineStr">
+      <c r="L30" t="inlineStr">
         <is>
           <t>2026-09-11</t>
         </is>
       </c>
-      <c r="M29" t="inlineStr">
+      <c r="M30" t="inlineStr">
         <is>
           <t>Glasgow, UK</t>
         </is>
       </c>
-      <c r="N29" t="inlineStr">
+      <c r="N30" t="inlineStr">
         <is>
           <t>https://eccv.ecva.net/Conferences/2026/</t>
         </is>
       </c>
-      <c r="O29" t="inlineStr">
+      <c r="O30" t="inlineStr">
         <is>
           <t>CET</t>
         </is>

</xml_diff>

<commit_message>
All 4: CSCW+ICCAD+ECCV+AAAI 2027
</commit_message>
<xml_diff>
--- a/timeline_data.xlsx
+++ b/timeline_data.xlsx
@@ -791,7 +791,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O34"/>
+  <dimension ref="A1:O35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2991,6 +2991,63 @@
         </is>
       </c>
       <c r="O34" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>cscw</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>CSCW</t>
+        </is>
+      </c>
+      <c r="C35" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D35" t="n">
+        <v>1</v>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>2025-05-14</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr"/>
+      <c r="G35" t="inlineStr"/>
+      <c r="H35" t="inlineStr"/>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>2025-08-19</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr"/>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="M35" t="inlineStr">
+        <is>
+          <t>Salt Lake City, UT, USA</t>
+        </is>
+      </c>
+      <c r="N35" t="inlineStr">
+        <is>
+          <t>https://cscw.acm.org/2026/</t>
+        </is>
+      </c>
+      <c r="O35" t="inlineStr">
         <is>
           <t>AoE</t>
         </is>
@@ -3007,7 +3064,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O28"/>
+  <dimension ref="A1:O30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4799,6 +4856,144 @@
       <c r="O28" t="inlineStr">
         <is>
           <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>iccad</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>ICCAD</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D29" t="n">
+        <v>1</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>2026-04-07</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr"/>
+      <c r="H29" t="inlineStr"/>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>2026-11-08</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>2026-11-12</t>
+        </is>
+      </c>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>San Jose, CA, USA</t>
+        </is>
+      </c>
+      <c r="N29" t="inlineStr">
+        <is>
+          <t>https://iccad.com/2026</t>
+        </is>
+      </c>
+      <c r="O29" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>eccv</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>ECCV</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D30" t="n">
+        <v>1</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>2026-03-05</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>2026-02-26</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>2026-05-02</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>2026-05-11</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t>Glasgow, UK</t>
+        </is>
+      </c>
+      <c r="N30" t="inlineStr">
+        <is>
+          <t>https://eccv.ecva.net/Conferences/2026/</t>
+        </is>
+      </c>
+      <c r="O30" t="inlineStr">
+        <is>
+          <t>CET</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add ACM MM 2026
</commit_message>
<xml_diff>
--- a/timeline_data.xlsx
+++ b/timeline_data.xlsx
@@ -791,7 +791,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O35"/>
+  <dimension ref="A1:O34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2991,63 +2991,6 @@
         </is>
       </c>
       <c r="O34" t="inlineStr">
-        <is>
-          <t>AoE</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>cscw</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>CSCW</t>
-        </is>
-      </c>
-      <c r="C35" t="n">
-        <v>2026</v>
-      </c>
-      <c r="D35" t="n">
-        <v>1</v>
-      </c>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t>2025-05-14</t>
-        </is>
-      </c>
-      <c r="F35" t="inlineStr"/>
-      <c r="G35" t="inlineStr"/>
-      <c r="H35" t="inlineStr"/>
-      <c r="I35" t="inlineStr">
-        <is>
-          <t>2025-08-19</t>
-        </is>
-      </c>
-      <c r="J35" t="inlineStr"/>
-      <c r="K35" t="inlineStr">
-        <is>
-          <t>2026-10-10</t>
-        </is>
-      </c>
-      <c r="L35" t="inlineStr">
-        <is>
-          <t>2026-10-14</t>
-        </is>
-      </c>
-      <c r="M35" t="inlineStr">
-        <is>
-          <t>Salt Lake City, UT, USA</t>
-        </is>
-      </c>
-      <c r="N35" t="inlineStr">
-        <is>
-          <t>https://cscw.acm.org/2026/</t>
-        </is>
-      </c>
-      <c r="O35" t="inlineStr">
         <is>
           <t>AoE</t>
         </is>
@@ -3064,7 +3007,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O30"/>
+  <dimension ref="A1:O29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4862,12 +4805,12 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>iccad</t>
+          <t>acm-mm</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>ICCAD</t>
+          <t>ACM MM</t>
         </is>
       </c>
       <c r="C29" t="n">
@@ -4878,122 +4821,49 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="G29" t="inlineStr"/>
       <c r="H29" t="inlineStr"/>
       <c r="I29" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>2026-11-08</t>
+          <t>2026-11-10</t>
         </is>
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>2026-11-12</t>
+          <t>2026-11-14</t>
         </is>
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>San Jose, CA, USA</t>
+          <t>Rio de Janeiro, Brazil</t>
         </is>
       </c>
       <c r="N29" t="inlineStr">
         <is>
-          <t>https://iccad.com/2026</t>
+          <t>https://2026.acmmm.org/</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
         <is>
           <t>AoE</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>eccv</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>ECCV</t>
-        </is>
-      </c>
-      <c r="C30" t="n">
-        <v>2026</v>
-      </c>
-      <c r="D30" t="n">
-        <v>1</v>
-      </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>2026-03-05</t>
-        </is>
-      </c>
-      <c r="F30" t="inlineStr">
-        <is>
-          <t>2026-02-26</t>
-        </is>
-      </c>
-      <c r="G30" t="inlineStr">
-        <is>
-          <t>2026-05-02</t>
-        </is>
-      </c>
-      <c r="H30" t="inlineStr">
-        <is>
-          <t>2026-05-11</t>
-        </is>
-      </c>
-      <c r="I30" t="inlineStr">
-        <is>
-          <t>2026-06-17</t>
-        </is>
-      </c>
-      <c r="J30" t="inlineStr">
-        <is>
-          <t>2026-06-30</t>
-        </is>
-      </c>
-      <c r="K30" t="inlineStr">
-        <is>
-          <t>2026-09-08</t>
-        </is>
-      </c>
-      <c r="L30" t="inlineStr">
-        <is>
-          <t>2026-09-11</t>
-        </is>
-      </c>
-      <c r="M30" t="inlineStr">
-        <is>
-          <t>Glasgow, UK</t>
-        </is>
-      </c>
-      <c r="N30" t="inlineStr">
-        <is>
-          <t>https://eccv.ecva.net/Conferences/2026/</t>
-        </is>
-      </c>
-      <c r="O30" t="inlineStr">
-        <is>
-          <t>CET</t>
         </is>
       </c>
     </row>
@@ -5008,7 +4878,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O18"/>
+  <dimension ref="A1:O17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6172,71 +6042,6 @@
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>aaai</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>AAAI</t>
-        </is>
-      </c>
-      <c r="C18" t="n">
-        <v>2027</v>
-      </c>
-      <c r="D18" t="n">
-        <v>1</v>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>2026-07-28</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>2026-07-21</t>
-        </is>
-      </c>
-      <c r="G18" t="inlineStr"/>
-      <c r="H18" t="inlineStr"/>
-      <c r="I18" t="inlineStr">
-        <is>
-          <t>2026-11-30</t>
-        </is>
-      </c>
-      <c r="J18" t="inlineStr">
-        <is>
-          <t>2026-12-14</t>
-        </is>
-      </c>
-      <c r="K18" t="inlineStr">
-        <is>
-          <t>2027-02-16</t>
-        </is>
-      </c>
-      <c r="L18" t="inlineStr">
-        <is>
-          <t>2027-02-23</t>
-        </is>
-      </c>
-      <c r="M18" t="inlineStr">
-        <is>
-          <t>Montreal, Canada</t>
-        </is>
-      </c>
-      <c r="N18" t="inlineStr">
-        <is>
-          <t>https://aaai.org/conference/aaai/aaai-27/</t>
-        </is>
-      </c>
-      <c r="O18" t="inlineStr">
-        <is>
-          <t>AoE</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add CSCW, RECOMB, ICCAD, ECCV, ACM MM, AAAI - 87 total verified entries
</commit_message>
<xml_diff>
--- a/timeline_data.xlsx
+++ b/timeline_data.xlsx
@@ -530,7 +530,6 @@
           <t>2025-01-15</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
           <t>2025-02-24</t>
@@ -599,7 +598,6 @@
           <t>2025-04-15</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
           <t>2025-05-26</t>
@@ -668,7 +666,6 @@
           <t>2025-02-13</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
           <t>2025-04-07</t>
@@ -737,7 +734,6 @@
           <t>2025-03-07</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
           <t>2025-05-09</t>
@@ -753,7 +749,6 @@
           <t>2025-06-25</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr"/>
       <c r="K5" t="inlineStr">
         <is>
           <t>2025-10-19</t>
@@ -791,7 +786,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O35"/>
+  <dimension ref="A1:O37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -893,7 +888,6 @@
           <t>2025-07-15</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
           <t>2025-08-28</t>
@@ -962,7 +956,6 @@
           <t>2025-10-15</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
           <t>2025-11-27</t>
@@ -1031,7 +1024,6 @@
           <t>2025-09-01</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
           <t>2025-10-05</t>
@@ -1100,7 +1092,6 @@
           <t>2025-11-23</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
           <t>2026-01-02</t>
@@ -1169,7 +1160,6 @@
           <t>2025-08-26</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
           <t>2025-11-06</t>
@@ -1238,7 +1228,6 @@
           <t>2025-07-10</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
           <t>2025-09-22</t>
@@ -1307,15 +1296,11 @@
           <t>2025-06-05</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr"/>
       <c r="I8" t="inlineStr">
         <is>
           <t>2025-09-01</t>
         </is>
       </c>
-      <c r="J8" t="inlineStr"/>
       <c r="K8" t="inlineStr">
         <is>
           <t>2026-05-18</t>
@@ -1364,15 +1349,11 @@
           <t>2025-11-13</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr"/>
-      <c r="G9" t="inlineStr"/>
-      <c r="H9" t="inlineStr"/>
       <c r="I9" t="inlineStr">
         <is>
           <t>2026-02-01</t>
         </is>
       </c>
-      <c r="J9" t="inlineStr"/>
       <c r="K9" t="inlineStr">
         <is>
           <t>2026-05-18</t>
@@ -1421,7 +1402,6 @@
           <t>2025-10-02</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
         <is>
           <t>2025-12-08</t>
@@ -1490,7 +1470,6 @@
           <t>2025-12-04</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr">
         <is>
           <t>2026-02-13</t>
@@ -1559,9 +1538,6 @@
           <t>2025-09-20</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr"/>
-      <c r="G12" t="inlineStr"/>
-      <c r="H12" t="inlineStr"/>
       <c r="I12" t="inlineStr">
         <is>
           <t>2025-11-24</t>
@@ -1620,15 +1596,11 @@
           <t>2025-11-20</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr"/>
-      <c r="G13" t="inlineStr"/>
-      <c r="H13" t="inlineStr"/>
       <c r="I13" t="inlineStr">
         <is>
           <t>2026-02-15</t>
         </is>
       </c>
-      <c r="J13" t="inlineStr"/>
       <c r="K13" t="inlineStr">
         <is>
           <t>2026-07-06</t>
@@ -1677,7 +1649,6 @@
           <t>2025-10-24</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr">
         <is>
           <t>2025-12-16</t>
@@ -1746,15 +1717,11 @@
           <t>2025-07-24</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr"/>
-      <c r="G15" t="inlineStr"/>
-      <c r="H15" t="inlineStr"/>
       <c r="I15" t="inlineStr">
         <is>
           <t>2025-09-25</t>
         </is>
       </c>
-      <c r="J15" t="inlineStr"/>
       <c r="K15" t="inlineStr">
         <is>
           <t>2026-07-26</t>
@@ -1803,15 +1770,11 @@
           <t>2025-10-09</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr"/>
-      <c r="G16" t="inlineStr"/>
-      <c r="H16" t="inlineStr"/>
       <c r="I16" t="inlineStr">
         <is>
           <t>2025-12-11</t>
         </is>
       </c>
-      <c r="J16" t="inlineStr"/>
       <c r="K16" t="inlineStr">
         <is>
           <t>2026-07-26</t>
@@ -1860,7 +1823,6 @@
           <t>2025-10-24</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr"/>
       <c r="G17" t="inlineStr">
         <is>
           <t>2026-01-06</t>
@@ -1934,14 +1896,11 @@
           <t>2025-09-19</t>
         </is>
       </c>
-      <c r="G18" t="inlineStr"/>
-      <c r="H18" t="inlineStr"/>
       <c r="I18" t="inlineStr">
         <is>
           <t>2026-01-25</t>
         </is>
       </c>
-      <c r="J18" t="inlineStr"/>
       <c r="K18" t="inlineStr">
         <is>
           <t>2026-04-23</t>
@@ -2010,7 +1969,6 @@
           <t>2026-02-20</t>
         </is>
       </c>
-      <c r="J19" t="inlineStr"/>
       <c r="K19" t="inlineStr">
         <is>
           <t>2026-06-11</t>
@@ -2059,9 +2017,6 @@
           <t>2025-11-04</t>
         </is>
       </c>
-      <c r="F20" t="inlineStr"/>
-      <c r="G20" t="inlineStr"/>
-      <c r="H20" t="inlineStr"/>
       <c r="I20" t="inlineStr">
         <is>
           <t>2026-02-01</t>
@@ -2120,15 +2075,11 @@
           <t>2025-09-15</t>
         </is>
       </c>
-      <c r="F21" t="inlineStr"/>
-      <c r="G21" t="inlineStr"/>
-      <c r="H21" t="inlineStr"/>
       <c r="I21" t="inlineStr">
         <is>
           <t>2026-01-15</t>
         </is>
       </c>
-      <c r="J21" t="inlineStr"/>
       <c r="K21" t="inlineStr">
         <is>
           <t>2026-05-18</t>
@@ -2177,15 +2128,11 @@
           <t>2025-11-13</t>
         </is>
       </c>
-      <c r="F22" t="inlineStr"/>
-      <c r="G22" t="inlineStr"/>
-      <c r="H22" t="inlineStr"/>
       <c r="I22" t="inlineStr">
         <is>
           <t>2026-03-05</t>
         </is>
       </c>
-      <c r="J22" t="inlineStr"/>
       <c r="K22" t="inlineStr">
         <is>
           <t>2026-06-15</t>
@@ -2234,15 +2181,11 @@
           <t>2025-07-11</t>
         </is>
       </c>
-      <c r="F23" t="inlineStr"/>
-      <c r="G23" t="inlineStr"/>
-      <c r="H23" t="inlineStr"/>
       <c r="I23" t="inlineStr">
         <is>
           <t>2025-10-01</t>
         </is>
       </c>
-      <c r="J23" t="inlineStr"/>
       <c r="K23" t="inlineStr">
         <is>
           <t>2026-01-20</t>
@@ -2296,8 +2239,6 @@
           <t>2025-12-04</t>
         </is>
       </c>
-      <c r="G24" t="inlineStr"/>
-      <c r="H24" t="inlineStr"/>
       <c r="I24" t="inlineStr">
         <is>
           <t>2026-03-26</t>
@@ -2376,7 +2317,6 @@
           <t>2026-03-27</t>
         </is>
       </c>
-      <c r="J25" t="inlineStr"/>
       <c r="K25" t="inlineStr">
         <is>
           <t>2026-06-27</t>
@@ -2425,7 +2365,6 @@
           <t>2025-03-18</t>
         </is>
       </c>
-      <c r="F26" t="inlineStr"/>
       <c r="G26" t="inlineStr">
         <is>
           <t>2025-05-20</t>
@@ -2494,7 +2433,6 @@
           <t>2025-09-16</t>
         </is>
       </c>
-      <c r="F27" t="inlineStr"/>
       <c r="G27" t="inlineStr">
         <is>
           <t>2025-11-18</t>
@@ -2568,8 +2506,6 @@
           <t>2025-04-18</t>
         </is>
       </c>
-      <c r="G28" t="inlineStr"/>
-      <c r="H28" t="inlineStr"/>
       <c r="I28" t="inlineStr">
         <is>
           <t>2025-07-24</t>
@@ -2633,8 +2569,6 @@
           <t>2025-09-11</t>
         </is>
       </c>
-      <c r="G29" t="inlineStr"/>
-      <c r="H29" t="inlineStr"/>
       <c r="I29" t="inlineStr">
         <is>
           <t>2025-12-09</t>
@@ -2771,14 +2705,11 @@
           <t>2025-01-10</t>
         </is>
       </c>
-      <c r="G31" t="inlineStr"/>
-      <c r="H31" t="inlineStr"/>
       <c r="I31" t="inlineStr">
         <is>
           <t>2025-05-02</t>
         </is>
       </c>
-      <c r="J31" t="inlineStr"/>
       <c r="K31" t="inlineStr">
         <is>
           <t>2026-05-31</t>
@@ -2832,14 +2763,11 @@
           <t>2025-04-10</t>
         </is>
       </c>
-      <c r="G32" t="inlineStr"/>
-      <c r="H32" t="inlineStr"/>
       <c r="I32" t="inlineStr">
         <is>
           <t>2025-08-01</t>
         </is>
       </c>
-      <c r="J32" t="inlineStr"/>
       <c r="K32" t="inlineStr">
         <is>
           <t>2026-05-31</t>
@@ -2893,14 +2821,11 @@
           <t>2025-07-10</t>
         </is>
       </c>
-      <c r="G33" t="inlineStr"/>
-      <c r="H33" t="inlineStr"/>
       <c r="I33" t="inlineStr">
         <is>
           <t>2025-11-01</t>
         </is>
       </c>
-      <c r="J33" t="inlineStr"/>
       <c r="K33" t="inlineStr">
         <is>
           <t>2026-05-31</t>
@@ -2969,7 +2894,6 @@
           <t>2026-01-30</t>
         </is>
       </c>
-      <c r="J34" t="inlineStr"/>
       <c r="K34" t="inlineStr">
         <is>
           <t>2026-05-31</t>
@@ -3018,9 +2942,6 @@
           <t>2025-11-20</t>
         </is>
       </c>
-      <c r="F35" t="inlineStr"/>
-      <c r="G35" t="inlineStr"/>
-      <c r="H35" t="inlineStr"/>
       <c r="I35" t="inlineStr">
         <is>
           <t>2026-01-16</t>
@@ -3052,6 +2973,117 @@
         </is>
       </c>
       <c r="O35" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>cscw</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>CSCW</t>
+        </is>
+      </c>
+      <c r="C36" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D36" t="n">
+        <v>1</v>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>2025-05-14</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>2025-08-19</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="M36" t="inlineStr">
+        <is>
+          <t>Salt Lake City, UT, USA</t>
+        </is>
+      </c>
+      <c r="N36" t="inlineStr">
+        <is>
+          <t>https://cscw.acm.org/2026/</t>
+        </is>
+      </c>
+      <c r="O36" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>recomb</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>RECOMB</t>
+        </is>
+      </c>
+      <c r="C37" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D37" t="n">
+        <v>1</v>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>2025-11-20</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>2026-01-16</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>2026-02-25</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="M37" t="inlineStr">
+        <is>
+          <t>Thessaloniki, Greece</t>
+        </is>
+      </c>
+      <c r="N37" t="inlineStr">
+        <is>
+          <t>http://recomb.org/recomb2026/</t>
+        </is>
+      </c>
+      <c r="O37" t="inlineStr">
         <is>
           <t>AoE</t>
         </is>
@@ -3068,7 +3100,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O28"/>
+  <dimension ref="A1:O31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3170,7 +3202,6 @@
           <t>2026-01-15</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
           <t>2026-02-26</t>
@@ -3239,7 +3270,6 @@
           <t>2026-04-15</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
           <t>2026-05-28</t>
@@ -3308,7 +3338,6 @@
           <t>2026-02-12</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
           <t>2026-04-07</t>
@@ -3377,7 +3406,6 @@
           <t>2026-05-21</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
           <t>2026-07-17</t>
@@ -3446,9 +3474,6 @@
           <t>2026-05-19</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr"/>
-      <c r="H6" t="inlineStr"/>
       <c r="I6" t="inlineStr">
         <is>
           <t>2026-08-20</t>
@@ -3653,7 +3678,6 @@
           <t>2026-02-06</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
           <t>2026-04-27</t>
@@ -3669,7 +3693,6 @@
           <t>2026-05-11</t>
         </is>
       </c>
-      <c r="J9" t="inlineStr"/>
       <c r="K9" t="inlineStr">
         <is>
           <t>2026-08-17</t>
@@ -3718,15 +3741,11 @@
           <t>2026-01-29</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr"/>
-      <c r="G10" t="inlineStr"/>
-      <c r="H10" t="inlineStr"/>
       <c r="I10" t="inlineStr">
         <is>
           <t>2026-04-01</t>
         </is>
       </c>
-      <c r="J10" t="inlineStr"/>
       <c r="K10" t="inlineStr">
         <is>
           <t>2026-07-26</t>
@@ -3775,7 +3794,6 @@
           <t>2026-02-05</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr">
         <is>
           <t>2026-04-16</t>
@@ -3849,8 +3867,6 @@
           <t>2026-01-23</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr"/>
-      <c r="H12" t="inlineStr"/>
       <c r="I12" t="inlineStr">
         <is>
           <t>2026-04-30</t>
@@ -3914,14 +3930,11 @@
           <t>2026-05-04</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr"/>
-      <c r="H13" t="inlineStr"/>
       <c r="I13" t="inlineStr">
         <is>
           <t>2026-09-24</t>
         </is>
       </c>
-      <c r="J13" t="inlineStr"/>
       <c r="K13" t="inlineStr">
         <is>
           <t>2026-12-11</t>
@@ -3970,9 +3983,6 @@
           <t>2026-01-05</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr"/>
-      <c r="G14" t="inlineStr"/>
-      <c r="H14" t="inlineStr"/>
       <c r="I14" t="inlineStr">
         <is>
           <t>2026-04-04</t>
@@ -4031,15 +4041,11 @@
           <t>2026-05-25</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr"/>
-      <c r="G15" t="inlineStr"/>
-      <c r="H15" t="inlineStr"/>
       <c r="I15" t="inlineStr">
         <is>
           <t>2026-08-20</t>
         </is>
       </c>
-      <c r="J15" t="inlineStr"/>
       <c r="K15" t="inlineStr">
         <is>
           <t>2026-10-24</t>
@@ -4088,15 +4094,11 @@
           <t>2026-01-19</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr"/>
-      <c r="G16" t="inlineStr"/>
-      <c r="H16" t="inlineStr"/>
       <c r="I16" t="inlineStr">
         <is>
           <t>2026-04-15</t>
         </is>
       </c>
-      <c r="J16" t="inlineStr"/>
       <c r="K16" t="inlineStr">
         <is>
           <t>2026-08-15</t>
@@ -4218,15 +4220,11 @@
           <t>2026-04-01</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr"/>
-      <c r="G18" t="inlineStr"/>
-      <c r="H18" t="inlineStr"/>
       <c r="I18" t="inlineStr">
         <is>
           <t>2026-07-03</t>
         </is>
       </c>
-      <c r="J18" t="inlineStr"/>
       <c r="K18" t="inlineStr">
         <is>
           <t>2026-11-08</t>
@@ -4275,15 +4273,11 @@
           <t>2026-01-15</t>
         </is>
       </c>
-      <c r="F19" t="inlineStr"/>
-      <c r="G19" t="inlineStr"/>
-      <c r="H19" t="inlineStr"/>
       <c r="I19" t="inlineStr">
         <is>
           <t>2026-03-01</t>
         </is>
       </c>
-      <c r="J19" t="inlineStr"/>
       <c r="K19" t="inlineStr">
         <is>
           <t>2026-07-19</t>
@@ -4337,14 +4331,11 @@
           <t>2026-03-24</t>
         </is>
       </c>
-      <c r="G20" t="inlineStr"/>
-      <c r="H20" t="inlineStr"/>
       <c r="I20" t="inlineStr">
         <is>
           <t>2026-08-07</t>
         </is>
       </c>
-      <c r="J20" t="inlineStr"/>
       <c r="K20" t="inlineStr">
         <is>
           <t>2026-11-02</t>
@@ -4398,8 +4389,6 @@
           <t>2026-02-12</t>
         </is>
       </c>
-      <c r="G21" t="inlineStr"/>
-      <c r="H21" t="inlineStr"/>
       <c r="I21" t="inlineStr">
         <is>
           <t>2026-05-01</t>
@@ -4531,15 +4520,11 @@
           <t>2026-04-01</t>
         </is>
       </c>
-      <c r="F23" t="inlineStr"/>
-      <c r="G23" t="inlineStr"/>
-      <c r="H23" t="inlineStr"/>
       <c r="I23" t="inlineStr">
         <is>
           <t>2026-05-15</t>
         </is>
       </c>
-      <c r="J23" t="inlineStr"/>
       <c r="K23" t="inlineStr">
         <is>
           <t>2026-08-31</t>
@@ -4593,8 +4578,6 @@
           <t>2026-03-26</t>
         </is>
       </c>
-      <c r="G24" t="inlineStr"/>
-      <c r="H24" t="inlineStr"/>
       <c r="I24" t="inlineStr">
         <is>
           <t>2026-07-03</t>
@@ -4653,15 +4636,11 @@
           <t>2025-10-10</t>
         </is>
       </c>
-      <c r="F25" t="inlineStr"/>
-      <c r="G25" t="inlineStr"/>
-      <c r="H25" t="inlineStr"/>
       <c r="I25" t="inlineStr">
         <is>
           <t>2026-02-17</t>
         </is>
       </c>
-      <c r="J25" t="inlineStr"/>
       <c r="K25" t="inlineStr">
         <is>
           <t>2026-10-03</t>
@@ -4710,9 +4689,6 @@
           <t>2026-03-17</t>
         </is>
       </c>
-      <c r="F26" t="inlineStr"/>
-      <c r="G26" t="inlineStr"/>
-      <c r="H26" t="inlineStr"/>
       <c r="I26" t="inlineStr">
         <is>
           <t>2026-06-10</t>
@@ -4771,15 +4747,11 @@
           <t>2026-01-29</t>
         </is>
       </c>
-      <c r="F27" t="inlineStr"/>
-      <c r="G27" t="inlineStr"/>
-      <c r="H27" t="inlineStr"/>
       <c r="I27" t="inlineStr">
         <is>
           <t>2026-04-15</t>
         </is>
       </c>
-      <c r="J27" t="inlineStr"/>
       <c r="K27" t="inlineStr">
         <is>
           <t>2026-09-21</t>
@@ -4828,15 +4800,11 @@
           <t>2026-01-20</t>
         </is>
       </c>
-      <c r="F28" t="inlineStr"/>
-      <c r="G28" t="inlineStr"/>
-      <c r="H28" t="inlineStr"/>
       <c r="I28" t="inlineStr">
         <is>
           <t>2026-03-01</t>
         </is>
       </c>
-      <c r="J28" t="inlineStr"/>
       <c r="K28" t="inlineStr">
         <is>
           <t>2026-07-26</t>
@@ -4858,6 +4826,205 @@
         </is>
       </c>
       <c r="O28" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>iccad</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>ICCAD</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D29" t="n">
+        <v>1</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>2026-04-07</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>2026-11-08</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>2026-11-12</t>
+        </is>
+      </c>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>San Jose, CA, USA</t>
+        </is>
+      </c>
+      <c r="N29" t="inlineStr">
+        <is>
+          <t>https://iccad.com/2026</t>
+        </is>
+      </c>
+      <c r="O29" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>eccv</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>ECCV</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D30" t="n">
+        <v>1</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>2026-03-05</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>2026-02-26</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>2026-05-02</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>2026-05-11</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t>Glasgow, UK</t>
+        </is>
+      </c>
+      <c r="N30" t="inlineStr">
+        <is>
+          <t>https://eccv.ecva.net/Conferences/2026/</t>
+        </is>
+      </c>
+      <c r="O30" t="inlineStr">
+        <is>
+          <t>CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>acm-mm</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>ACM MM</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D31" t="n">
+        <v>1</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>2026-04-01</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>2026-11-10</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>2026-11-14</t>
+        </is>
+      </c>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>Rio de Janeiro, Brazil</t>
+        </is>
+      </c>
+      <c r="N31" t="inlineStr">
+        <is>
+          <t>https://2026.acmmm.org/</t>
+        </is>
+      </c>
+      <c r="O31" t="inlineStr">
         <is>
           <t>AoE</t>
         </is>
@@ -4874,7 +5041,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O17"/>
+  <dimension ref="A1:O18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4976,7 +5143,6 @@
           <t>2026-07-15</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
           <t>2026-08-23</t>
@@ -5045,7 +5211,6 @@
           <t>2026-10-15</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
           <t>2026-11-23</t>
@@ -5114,7 +5279,6 @@
           <t>2027-01-15</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
           <t>2027-02-23</t>
@@ -5183,7 +5347,6 @@
           <t>2027-04-15</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
           <t>2027-05-23</t>
@@ -5252,7 +5415,6 @@
           <t>2026-03-01</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
           <t>2026-04-05</t>
@@ -5321,7 +5483,6 @@
           <t>2026-06-01</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
           <t>2026-07-05</t>
@@ -5390,7 +5551,6 @@
           <t>2026-09-01</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
           <t>2026-10-05</t>
@@ -5459,7 +5619,6 @@
           <t>2026-12-01</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
           <t>2027-01-05</t>
@@ -5528,7 +5687,6 @@
           <t>2026-09-17</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
         <is>
           <t>2026-11-30</t>
@@ -5597,7 +5755,6 @@
           <t>2026-06-11</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr">
         <is>
           <t>2026-08-20</t>
@@ -5666,7 +5823,6 @@
           <t>2026-11-17</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr">
         <is>
           <t>2027-02-11</t>
@@ -5735,7 +5891,6 @@
           <t>2026-08-25</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr">
         <is>
           <t>2026-11-05</t>
@@ -5804,7 +5959,6 @@
           <t>2027-01-26</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr">
         <is>
           <t>2027-04-08</t>
@@ -5873,7 +6027,6 @@
           <t>2026-05-06</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr">
         <is>
           <t>2026-07-15</t>
@@ -5942,9 +6095,6 @@
           <t>2026-08-19</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr"/>
-      <c r="G16" t="inlineStr"/>
-      <c r="H16" t="inlineStr"/>
       <c r="I16" t="inlineStr">
         <is>
           <t>2026-11-04</t>
@@ -6003,15 +6153,11 @@
           <t>2026-09-01</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr"/>
-      <c r="G17" t="inlineStr"/>
-      <c r="H17" t="inlineStr"/>
       <c r="I17" t="inlineStr">
         <is>
           <t>2026-12-01</t>
         </is>
       </c>
-      <c r="J17" t="inlineStr"/>
       <c r="K17" t="inlineStr">
         <is>
           <t>2027-05-10</t>
@@ -6033,6 +6179,69 @@
         </is>
       </c>
       <c r="O17" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>aaai</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>AAAI</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>2027</v>
+      </c>
+      <c r="D18" t="n">
+        <v>1</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>2026-11-30</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>2026-12-14</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>2027-02-16</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>2027-02-23</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>Montreal, Canada</t>
+        </is>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>https://aaai.org/conference/aaai/aaai-27/</t>
+        </is>
+      </c>
+      <c r="O18" t="inlineStr">
         <is>
           <t>AoE</t>
         </is>

</xml_diff>

<commit_message>
Add ICDE 2026 (2 rounds)
</commit_message>
<xml_diff>
--- a/timeline_data.xlsx
+++ b/timeline_data.xlsx
@@ -786,7 +786,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O37"/>
+  <dimension ref="A1:O39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3086,6 +3086,112 @@
       <c r="O37" t="inlineStr">
         <is>
           <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>icde</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>ICDE</t>
+        </is>
+      </c>
+      <c r="C38" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D38" t="n">
+        <v>1</v>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>2025-06-18</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>2025-10-20</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>2026-05-04</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>2026-05-08</t>
+        </is>
+      </c>
+      <c r="M38" t="inlineStr">
+        <is>
+          <t>Montreal, Canada</t>
+        </is>
+      </c>
+      <c r="N38" t="inlineStr">
+        <is>
+          <t>https://icde2026.github.io/</t>
+        </is>
+      </c>
+      <c r="O38" t="inlineStr">
+        <is>
+          <t>US Pacific</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>icde</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>ICDE</t>
+        </is>
+      </c>
+      <c r="C39" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D39" t="n">
+        <v>2</v>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>2025-10-27</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>2026-02-23</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>2026-05-04</t>
+        </is>
+      </c>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>2026-05-08</t>
+        </is>
+      </c>
+      <c r="M39" t="inlineStr">
+        <is>
+          <t>Montreal, Canada</t>
+        </is>
+      </c>
+      <c r="N39" t="inlineStr">
+        <is>
+          <t>https://icde2026.github.io/</t>
+        </is>
+      </c>
+      <c r="O39" t="inlineStr">
+        <is>
+          <t>US Pacific</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add UbiComp 2026 - reached 90 verified entries!
</commit_message>
<xml_diff>
--- a/timeline_data.xlsx
+++ b/timeline_data.xlsx
@@ -3206,7 +3206,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O31"/>
+  <dimension ref="A1:O32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5131,6 +5131,59 @@
         </is>
       </c>
       <c r="O31" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>ubicomp</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>UbiComp</t>
+        </is>
+      </c>
+      <c r="C32" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D32" t="n">
+        <v>1</v>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>2026-05-01</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>Shanghai, China</t>
+        </is>
+      </c>
+      <c r="N32" t="inlineStr">
+        <is>
+          <t>https://www.ubicomp.org/ubicomp-iswc-2026/</t>
+        </is>
+      </c>
+      <c r="O32" t="inlineStr">
         <is>
           <t>AoE</t>
         </is>

</xml_diff>

<commit_message>
Add RecSys 2026 - 91 total
</commit_message>
<xml_diff>
--- a/timeline_data.xlsx
+++ b/timeline_data.xlsx
@@ -3206,7 +3206,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O32"/>
+  <dimension ref="A1:O33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5184,6 +5184,79 @@
         </is>
       </c>
       <c r="O32" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>recsys</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>RecSys</t>
+        </is>
+      </c>
+      <c r="C33" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D33" t="n">
+        <v>1</v>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>2026-04-21</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="M33" t="inlineStr">
+        <is>
+          <t>Minneapolis, MN, USA</t>
+        </is>
+      </c>
+      <c r="N33" t="inlineStr">
+        <is>
+          <t>https://recsys.acm.org/recsys26/</t>
+        </is>
+      </c>
+      <c r="O33" t="inlineStr">
         <is>
           <t>AoE</t>
         </is>

</xml_diff>

<commit_message>
Add SIGMETRICS 2026 (3 rounds)
</commit_message>
<xml_diff>
--- a/timeline_data.xlsx
+++ b/timeline_data.xlsx
@@ -786,7 +786,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O39"/>
+  <dimension ref="A1:O41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3192,6 +3192,112 @@
       <c r="O39" t="inlineStr">
         <is>
           <t>US Pacific</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>sigmetrics</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>SIGMETRICS</t>
+        </is>
+      </c>
+      <c r="C40" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D40" t="n">
+        <v>1</v>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>2025-07-29</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>2025-09-26</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>2026-06-12</t>
+        </is>
+      </c>
+      <c r="M40" t="inlineStr">
+        <is>
+          <t>Ann Arbor, MI, USA</t>
+        </is>
+      </c>
+      <c r="N40" t="inlineStr">
+        <is>
+          <t>https://www.sigmetrics.org/sigmetrics2026/</t>
+        </is>
+      </c>
+      <c r="O40" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>sigmetrics</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>SIGMETRICS</t>
+        </is>
+      </c>
+      <c r="C41" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D41" t="n">
+        <v>2</v>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>2025-10-14</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>2025-12-12</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>2026-06-12</t>
+        </is>
+      </c>
+      <c r="M41" t="inlineStr">
+        <is>
+          <t>Ann Arbor, MI, USA</t>
+        </is>
+      </c>
+      <c r="N41" t="inlineStr">
+        <is>
+          <t>https://www.sigmetrics.org/sigmetrics2026/</t>
+        </is>
+      </c>
+      <c r="O41" t="inlineStr">
+        <is>
+          <t>AoE</t>
         </is>
       </c>
     </row>
@@ -3206,7 +3312,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O33"/>
+  <dimension ref="A1:O34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5257,6 +5363,59 @@
         </is>
       </c>
       <c r="O33" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>sigmetrics</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>SIGMETRICS</t>
+        </is>
+      </c>
+      <c r="C34" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D34" t="n">
+        <v>3</v>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>2026-01-13</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>2026-03-13</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>2026-06-12</t>
+        </is>
+      </c>
+      <c r="M34" t="inlineStr">
+        <is>
+          <t>Ann Arbor, MI, USA</t>
+        </is>
+      </c>
+      <c r="N34" t="inlineStr">
+        <is>
+          <t>https://www.sigmetrics.org/sigmetrics2026/</t>
+        </is>
+      </c>
+      <c r="O34" t="inlineStr">
         <is>
           <t>AoE</t>
         </is>

</xml_diff>

<commit_message>
Add ICPP 2026 - 95 total
</commit_message>
<xml_diff>
--- a/timeline_data.xlsx
+++ b/timeline_data.xlsx
@@ -3312,7 +3312,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O34"/>
+  <dimension ref="A1:O35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5416,6 +5416,69 @@
         </is>
       </c>
       <c r="O34" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>icpp</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>ICPP</t>
+        </is>
+      </c>
+      <c r="C35" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D35" t="n">
+        <v>1</v>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>2026-05-01</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>2026-04-24</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="M35" t="inlineStr">
+        <is>
+          <t>Singapore</t>
+        </is>
+      </c>
+      <c r="N35" t="inlineStr">
+        <is>
+          <t>https://icpp2026.github.io/</t>
+        </is>
+      </c>
+      <c r="O35" t="inlineStr">
         <is>
           <t>AoE</t>
         </is>

</xml_diff>

<commit_message>
Add WSDM 2027 - 96 total
</commit_message>
<xml_diff>
--- a/timeline_data.xlsx
+++ b/timeline_data.xlsx
@@ -5495,7 +5495,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O18"/>
+  <dimension ref="A1:O19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6701,6 +6701,64 @@
         </is>
       </c>
     </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>wsdm</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>WSDM</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>2027</v>
+      </c>
+      <c r="D19" t="n">
+        <v>1</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>2026-11-02</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>2027-02-15</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>2027-02-19</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>Hong Kong, China</t>
+        </is>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>https://wsdm-conference.org/2027/</t>
+        </is>
+      </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add ICWSM 2027 (2 rounds) - 98 total
</commit_message>
<xml_diff>
--- a/timeline_data.xlsx
+++ b/timeline_data.xlsx
@@ -5495,7 +5495,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O19"/>
+  <dimension ref="A1:O21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6759,6 +6759,112 @@
         </is>
       </c>
     </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>icwsm</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>ICWSM</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>2027</v>
+      </c>
+      <c r="D20" t="n">
+        <v>1</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>2027-05-01</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>2027-05-31</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>Edinburgh, Scotland, UK</t>
+        </is>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>https://icwsm.org/2027/</t>
+        </is>
+      </c>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>icwsm</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>ICWSM</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>2027</v>
+      </c>
+      <c r="D21" t="n">
+        <v>2</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>2026-11-15</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>2027-05-01</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>2027-05-31</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>Edinburgh, Scotland, UK</t>
+        </is>
+      </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>https://icwsm.org/2027/</t>
+        </is>
+      </c>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add ISSRE 2026 - 99 total
</commit_message>
<xml_diff>
--- a/timeline_data.xlsx
+++ b/timeline_data.xlsx
@@ -3312,7 +3312,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O35"/>
+  <dimension ref="A1:O36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5479,6 +5479,74 @@
         </is>
       </c>
       <c r="O35" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>issre</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>ISSRE</t>
+        </is>
+      </c>
+      <c r="C36" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D36" t="n">
+        <v>1</v>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>2026-04-24</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="M36" t="inlineStr">
+        <is>
+          <t>Limassol, Cyprus</t>
+        </is>
+      </c>
+      <c r="N36" t="inlineStr">
+        <is>
+          <t>https://easychair.org/conferences?conf=issre2026</t>
+        </is>
+      </c>
+      <c r="O36" t="inlineStr">
         <is>
           <t>AoE</t>
         </is>

</xml_diff>

<commit_message>
Add COLT 2026 - reached 100 verified entries!
</commit_message>
<xml_diff>
--- a/timeline_data.xlsx
+++ b/timeline_data.xlsx
@@ -3312,7 +3312,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O36"/>
+  <dimension ref="A1:O37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5547,6 +5547,69 @@
         </is>
       </c>
       <c r="O36" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>colt</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>COLT</t>
+        </is>
+      </c>
+      <c r="C37" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D37" t="n">
+        <v>1</v>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>2026-02-04</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>2026-04-03</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>2026-04-20</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>2026-05-04</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="M37" t="inlineStr">
+        <is>
+          <t>San Diego, CA, USA</t>
+        </is>
+      </c>
+      <c r="N37" t="inlineStr">
+        <is>
+          <t>https://learningtheory.org/colt2026/</t>
+        </is>
+      </c>
+      <c r="O37" t="inlineStr">
         <is>
           <t>AoE</t>
         </is>

</xml_diff>

<commit_message>
Add AAMAS 2026 + 2027 - 102 total
</commit_message>
<xml_diff>
--- a/timeline_data.xlsx
+++ b/timeline_data.xlsx
@@ -786,7 +786,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O41"/>
+  <dimension ref="A1:O42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3296,6 +3296,79 @@
         </is>
       </c>
       <c r="O41" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>aamas</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>AAMAS</t>
+        </is>
+      </c>
+      <c r="C42" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D42" t="n">
+        <v>1</v>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>2025-10-08</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>2025-10-01</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>2025-11-21</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>2025-11-25</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>2025-12-22</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>2026-02-11</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="M42" t="inlineStr">
+        <is>
+          <t>Paphos, Cyprus</t>
+        </is>
+      </c>
+      <c r="N42" t="inlineStr">
+        <is>
+          <t>https://cyprusconferences.org/aamas2026/</t>
+        </is>
+      </c>
+      <c r="O42" t="inlineStr">
         <is>
           <t>AoE</t>
         </is>
@@ -5626,7 +5699,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O21"/>
+  <dimension ref="A1:O22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6996,6 +7069,64 @@
         </is>
       </c>
     </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>aamas</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>AAMAS</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>2027</v>
+      </c>
+      <c r="D22" t="n">
+        <v>1</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>2027-02-01</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>2027-05-03</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>2027-05-07</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>Hanoi, Vietnam</t>
+        </is>
+      </c>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>https://warwick.ac.uk/fac/sci/dcs/aamas2027/</t>
+        </is>
+      </c>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add GECCO 2026 - 103 total
</commit_message>
<xml_diff>
--- a/timeline_data.xlsx
+++ b/timeline_data.xlsx
@@ -3385,7 +3385,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O37"/>
+  <dimension ref="A1:O38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5683,6 +5683,69 @@
         </is>
       </c>
       <c r="O37" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>gecco</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>GECCO</t>
+        </is>
+      </c>
+      <c r="C38" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D38" t="n">
+        <v>1</v>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>2026-01-26</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>2026-01-19</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>2026-03-20</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>2026-04-10</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="M38" t="inlineStr">
+        <is>
+          <t>San Jose, Costa Rica</t>
+        </is>
+      </c>
+      <c r="N38" t="inlineStr">
+        <is>
+          <t>http://gecco-2026.sigevo.org/</t>
+        </is>
+      </c>
+      <c r="O38" t="inlineStr">
         <is>
           <t>AoE</t>
         </is>

</xml_diff>

<commit_message>
Add FAST 2027 (2x) + NSDI 2027 - 107 total
</commit_message>
<xml_diff>
--- a/timeline_data.xlsx
+++ b/timeline_data.xlsx
@@ -5835,7 +5835,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O22"/>
+  <dimension ref="A1:O25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7263,6 +7263,165 @@
         </is>
       </c>
     </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>fast</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>FAST</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>2027</v>
+      </c>
+      <c r="D23" t="n">
+        <v>1</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>2026-03-17</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>2027-02-23</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>2027-02-25</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>Renton, WA, USA</t>
+        </is>
+      </c>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>https://www.usenix.org/conference/fast27/</t>
+        </is>
+      </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>fast</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>FAST</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>2027</v>
+      </c>
+      <c r="D24" t="n">
+        <v>2</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>2026-12-08</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>2027-02-23</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>2027-02-25</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>Renton, WA, USA</t>
+        </is>
+      </c>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>https://www.usenix.org/conference/fast27/</t>
+        </is>
+      </c>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>nsdi</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>NSDI</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>2027</v>
+      </c>
+      <c r="D25" t="n">
+        <v>1</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>2026-12-08</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>2027-05-11</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>2027-05-13</t>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>Providence, RI, USA</t>
+        </is>
+      </c>
+      <c r="N25" t="inlineStr">
+        <is>
+          <t>https://www.usenix.org/conference/nsdi27/</t>
+        </is>
+      </c>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add HOT CHIPS 2026
</commit_message>
<xml_diff>
--- a/timeline_data.xlsx
+++ b/timeline_data.xlsx
@@ -3458,7 +3458,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O38"/>
+  <dimension ref="A1:O39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5819,6 +5819,64 @@
         </is>
       </c>
       <c r="O38" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>hotchips</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>HOT CHIPS</t>
+        </is>
+      </c>
+      <c r="C39" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D39" t="n">
+        <v>1</v>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>2026-04-08</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>2026-05-01</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
+      </c>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="M39" t="inlineStr">
+        <is>
+          <t>Stanford, CA, USA</t>
+        </is>
+      </c>
+      <c r="N39" t="inlineStr">
+        <is>
+          <t>https://www.hotchips.org/</t>
+        </is>
+      </c>
+      <c r="O39" t="inlineStr">
         <is>
           <t>AoE</t>
         </is>

</xml_diff>

<commit_message>
Add PPSN 2026 - 109 total
</commit_message>
<xml_diff>
--- a/timeline_data.xlsx
+++ b/timeline_data.xlsx
@@ -3458,7 +3458,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O39"/>
+  <dimension ref="A1:O40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5877,6 +5877,59 @@
         </is>
       </c>
       <c r="O39" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>ppsn</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>PPSN</t>
+        </is>
+      </c>
+      <c r="C40" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D40" t="n">
+        <v>1</v>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>2026-03-28</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="M40" t="inlineStr">
+        <is>
+          <t>Trento, Italy</t>
+        </is>
+      </c>
+      <c r="N40" t="inlineStr">
+        <is>
+          <t>https://ppsn2026.science.unitn.it/</t>
+        </is>
+      </c>
+      <c r="O40" t="inlineStr">
         <is>
           <t>AoE</t>
         </is>

</xml_diff>

<commit_message>
Add ICLR 2027 - reached 110 verified entries!
</commit_message>
<xml_diff>
--- a/timeline_data.xlsx
+++ b/timeline_data.xlsx
@@ -5946,7 +5946,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O25"/>
+  <dimension ref="A1:O26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7533,6 +7533,59 @@
         </is>
       </c>
     </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>iclr</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>ICLR</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>2027</v>
+      </c>
+      <c r="D26" t="n">
+        <v>1</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>2027-01-25</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>2027-04-24</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>2027-04-28</t>
+        </is>
+      </c>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>West Coast, USA</t>
+        </is>
+      </c>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t>https://iclr.cc/Conferences/2027/</t>
+        </is>
+      </c>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add CGO 2026 R2 + CGO 2027 (2 rounds) - 113 total
</commit_message>
<xml_diff>
--- a/timeline_data.xlsx
+++ b/timeline_data.xlsx
@@ -786,7 +786,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O43"/>
+  <dimension ref="A1:O44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3442,6 +3442,69 @@
         </is>
       </c>
       <c r="O43" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>cgo</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>CGO</t>
+        </is>
+      </c>
+      <c r="C44" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D44" t="n">
+        <v>2</v>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>2025-09-11</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>2025-10-21</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>2025-10-23</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>2025-11-03</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>2026-01-31</t>
+        </is>
+      </c>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>2026-02-04</t>
+        </is>
+      </c>
+      <c r="M44" t="inlineStr">
+        <is>
+          <t>Sydney, Australia</t>
+        </is>
+      </c>
+      <c r="N44" t="inlineStr">
+        <is>
+          <t>https://2026.cgo.org/</t>
+        </is>
+      </c>
+      <c r="O44" t="inlineStr">
         <is>
           <t>AoE</t>
         </is>
@@ -5946,7 +6009,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O26"/>
+  <dimension ref="A1:O28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7586,6 +7649,92 @@
         </is>
       </c>
     </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>cgo</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>CGO</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>2027</v>
+      </c>
+      <c r="D27" t="n">
+        <v>1</v>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="N27" t="inlineStr">
+        <is>
+          <t>https://conf.researchr.org/home/cgo-2027</t>
+        </is>
+      </c>
+      <c r="O27" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>cgo</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>CGO</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>2027</v>
+      </c>
+      <c r="D28" t="n">
+        <v>2</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>2026-11-09</t>
+        </is>
+      </c>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>https://conf.researchr.org/home/cgo-2027</t>
+        </is>
+      </c>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add Eurographics 2027 - 114 total
</commit_message>
<xml_diff>
--- a/timeline_data.xlsx
+++ b/timeline_data.xlsx
@@ -6009,7 +6009,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O28"/>
+  <dimension ref="A1:O29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7735,6 +7735,69 @@
         </is>
       </c>
     </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>eurographics</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Eurographics</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>2027</v>
+      </c>
+      <c r="D29" t="n">
+        <v>1</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>2026-12-18</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>2027-02-23</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>2027-05-10</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>2027-05-14</t>
+        </is>
+      </c>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>Pisa, Italy</t>
+        </is>
+      </c>
+      <c r="N29" t="inlineStr">
+        <is>
+          <t>https://www.eg.org/</t>
+        </is>
+      </c>
+      <c r="O29" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add DIS 2026 + SLT 2026 - 116 total
</commit_message>
<xml_diff>
--- a/timeline_data.xlsx
+++ b/timeline_data.xlsx
@@ -3521,7 +3521,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O40"/>
+  <dimension ref="A1:O41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5993,6 +5993,69 @@
         </is>
       </c>
       <c r="O40" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>slt</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>SLT</t>
+        </is>
+      </c>
+      <c r="C41" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D41" t="n">
+        <v>1</v>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>2026-01-09</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>2026-12-13</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>2026-12-16</t>
+        </is>
+      </c>
+      <c r="M41" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="N41" t="inlineStr">
+        <is>
+          <t>https://attend.ieee.org/slt-2026/</t>
+        </is>
+      </c>
+      <c r="O41" t="inlineStr">
         <is>
           <t>AoE</t>
         </is>

</xml_diff>

<commit_message>
Add IJCNN + FUZZ-IEEE + IEEE CEC 2026 - 119 total
</commit_message>
<xml_diff>
--- a/timeline_data.xlsx
+++ b/timeline_data.xlsx
@@ -3521,7 +3521,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O41"/>
+  <dimension ref="A1:O44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6056,6 +6056,180 @@
         </is>
       </c>
       <c r="O41" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>ijcnn</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>IJCNN</t>
+        </is>
+      </c>
+      <c r="C42" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D42" t="n">
+        <v>1</v>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>2026-01-31</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>2026-03-15</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="M42" t="inlineStr">
+        <is>
+          <t>Maastricht, Netherlands</t>
+        </is>
+      </c>
+      <c r="N42" t="inlineStr">
+        <is>
+          <t>https://attend.ieee.org/wcci-2026/</t>
+        </is>
+      </c>
+      <c r="O42" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>fuzz-ieee</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>FUZZ-IEEE</t>
+        </is>
+      </c>
+      <c r="C43" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D43" t="n">
+        <v>1</v>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>2026-01-31</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>2026-03-15</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="M43" t="inlineStr">
+        <is>
+          <t>Maastricht, Netherlands</t>
+        </is>
+      </c>
+      <c r="N43" t="inlineStr">
+        <is>
+          <t>https://attend.ieee.org/wcci-2026/</t>
+        </is>
+      </c>
+      <c r="O43" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>ieee-cec</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>IEEE CEC</t>
+        </is>
+      </c>
+      <c r="C44" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D44" t="n">
+        <v>1</v>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>2026-01-31</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>2026-03-15</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="M44" t="inlineStr">
+        <is>
+          <t>Maastricht, Netherlands</t>
+        </is>
+      </c>
+      <c r="N44" t="inlineStr">
+        <is>
+          <t>https://attend.ieee.org/wcci-2026/</t>
+        </is>
+      </c>
+      <c r="O44" t="inlineStr">
         <is>
           <t>AoE</t>
         </is>

</xml_diff>

<commit_message>
Add ICSE 2027 - reached 120 entries!
</commit_message>
<xml_diff>
--- a/timeline_data.xlsx
+++ b/timeline_data.xlsx
@@ -6246,7 +6246,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O29"/>
+  <dimension ref="A1:O30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8035,6 +8035,79 @@
         </is>
       </c>
     </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>icse</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>ICSE</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>2027</v>
+      </c>
+      <c r="D30" t="n">
+        <v>1</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>2026-11-24</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>2027-04-25</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>2027-05-01</t>
+        </is>
+      </c>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t>Dublin, Ireland</t>
+        </is>
+      </c>
+      <c r="N30" t="inlineStr">
+        <is>
+          <t>https://conf.researchr.org/home/icse-2027</t>
+        </is>
+      </c>
+      <c r="O30" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add ASPLOS 2027 (2 rounds) - 121 total
</commit_message>
<xml_diff>
--- a/timeline_data.xlsx
+++ b/timeline_data.xlsx
@@ -6246,7 +6246,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O30"/>
+  <dimension ref="A1:O32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8108,6 +8108,112 @@
         </is>
       </c>
     </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>asplos</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>ASPLOS</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>2027</v>
+      </c>
+      <c r="D31" t="n">
+        <v>1</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>2027-04-11</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>2027-04-15</t>
+        </is>
+      </c>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>Heraklion, Crete, Greece</t>
+        </is>
+      </c>
+      <c r="N31" t="inlineStr">
+        <is>
+          <t>https://www.asplos-conference.org/asplos2027/</t>
+        </is>
+      </c>
+      <c r="O31" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>asplos</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>ASPLOS</t>
+        </is>
+      </c>
+      <c r="C32" t="n">
+        <v>2027</v>
+      </c>
+      <c r="D32" t="n">
+        <v>2</v>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>2026-12-21</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>2027-04-11</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>2027-04-15</t>
+        </is>
+      </c>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>Heraklion, Crete, Greece</t>
+        </is>
+      </c>
+      <c r="N32" t="inlineStr">
+        <is>
+          <t>https://www.asplos-conference.org/asplos2027/</t>
+        </is>
+      </c>
+      <c r="O32" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add SOUPS 2026 - 122 total
</commit_message>
<xml_diff>
--- a/timeline_data.xlsx
+++ b/timeline_data.xlsx
@@ -3521,7 +3521,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O44"/>
+  <dimension ref="A1:O45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6230,6 +6230,64 @@
         </is>
       </c>
       <c r="O44" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>soups</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>SOUPS</t>
+        </is>
+      </c>
+      <c r="C45" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D45" t="n">
+        <v>1</v>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>2026-02-19</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>2026-02-12</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
+      </c>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="M45" t="inlineStr">
+        <is>
+          <t>Hannover, Germany</t>
+        </is>
+      </c>
+      <c r="N45" t="inlineStr">
+        <is>
+          <t>https://www.usenix.org/conference/soups2026/</t>
+        </is>
+      </c>
+      <c r="O45" t="inlineStr">
         <is>
           <t>AoE</t>
         </is>

</xml_diff>

<commit_message>
Add ICME 2026 - 123 total
</commit_message>
<xml_diff>
--- a/timeline_data.xlsx
+++ b/timeline_data.xlsx
@@ -786,7 +786,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O44"/>
+  <dimension ref="A1:O45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3505,6 +3505,54 @@
         </is>
       </c>
       <c r="O44" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>icme</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>ICME</t>
+        </is>
+      </c>
+      <c r="C45" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D45" t="n">
+        <v>1</v>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>2025-12-15</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>2026-03-01</t>
+        </is>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="M45" t="inlineStr">
+        <is>
+          <t>Bangkok, Thailand</t>
+        </is>
+      </c>
+      <c r="O45" t="inlineStr">
         <is>
           <t>AoE</t>
         </is>

</xml_diff>

<commit_message>
Add FM 2026 - 124 total
</commit_message>
<xml_diff>
--- a/timeline_data.xlsx
+++ b/timeline_data.xlsx
@@ -786,7 +786,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O45"/>
+  <dimension ref="A1:O46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3553,6 +3553,69 @@
         </is>
       </c>
       <c r="O45" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>fm</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>FM</t>
+        </is>
+      </c>
+      <c r="C46" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D46" t="n">
+        <v>1</v>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>2025-12-02</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>2025-11-25</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>2026-01-30</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>2026-02-23</t>
+        </is>
+      </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="M46" t="inlineStr">
+        <is>
+          <t>Tokyo, Japan</t>
+        </is>
+      </c>
+      <c r="N46" t="inlineStr">
+        <is>
+          <t>https://conf.researchr.org/home/fm-2026</t>
+        </is>
+      </c>
+      <c r="O46" t="inlineStr">
         <is>
           <t>AoE</t>
         </is>

</xml_diff>

<commit_message>
Add ICPR+ICDAR+FG+BMVC 2026 - 128 total
</commit_message>
<xml_diff>
--- a/timeline_data.xlsx
+++ b/timeline_data.xlsx
@@ -786,7 +786,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O46"/>
+  <dimension ref="A1:O47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3616,6 +3616,54 @@
         </is>
       </c>
       <c r="O46" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>icpr</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>ICPR</t>
+        </is>
+      </c>
+      <c r="C47" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D47" t="n">
+        <v>1</v>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>2025-12-21</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>2026-03-01</t>
+        </is>
+      </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="M47" t="inlineStr">
+        <is>
+          <t>Lyon, France</t>
+        </is>
+      </c>
+      <c r="O47" t="inlineStr">
         <is>
           <t>AoE</t>
         </is>
@@ -3632,7 +3680,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O45"/>
+  <dimension ref="A1:P48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6399,6 +6447,135 @@
         </is>
       </c>
       <c r="O45" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>icdar</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>ICDAR</t>
+        </is>
+      </c>
+      <c r="C46" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D46" t="n">
+        <v>1</v>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>2026-02-27</t>
+        </is>
+      </c>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="M46" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="N46" t="inlineStr">
+        <is>
+          <t>Vienna, Austria</t>
+        </is>
+      </c>
+      <c r="P46" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>fg</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>FG</t>
+        </is>
+      </c>
+      <c r="C47" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D47" t="n">
+        <v>1</v>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>2026-01-09</t>
+        </is>
+      </c>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="M47" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="N47" t="inlineStr">
+        <is>
+          <t>Kyoto, Japan</t>
+        </is>
+      </c>
+      <c r="P47" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>bmvc</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>BMVC</t>
+        </is>
+      </c>
+      <c r="C48" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D48" t="n">
+        <v>1</v>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="L48" t="inlineStr">
+        <is>
+          <t>2026-11-23</t>
+        </is>
+      </c>
+      <c r="M48" t="inlineStr">
+        <is>
+          <t>2026-11-26</t>
+        </is>
+      </c>
+      <c r="N48" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="P48" t="inlineStr">
         <is>
           <t>AoE</t>
         </is>

</xml_diff>

<commit_message>
Add ICECCS 2026 - 129 total
</commit_message>
<xml_diff>
--- a/timeline_data.xlsx
+++ b/timeline_data.xlsx
@@ -3680,7 +3680,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P48"/>
+  <dimension ref="A1:P49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6576,6 +6576,69 @@
         </is>
       </c>
       <c r="P48" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>iceccs</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>ICECCS</t>
+        </is>
+      </c>
+      <c r="C49" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D49" t="n">
+        <v>1</v>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>2026-11-23</t>
+        </is>
+      </c>
+      <c r="L49" t="inlineStr">
+        <is>
+          <t>2026-11-24</t>
+        </is>
+      </c>
+      <c r="M49" t="inlineStr">
+        <is>
+          <t>Brisbane, Australia</t>
+        </is>
+      </c>
+      <c r="N49" t="inlineStr">
+        <is>
+          <t>https://easychair.org/conferences?conf=iceccs2026</t>
+        </is>
+      </c>
+      <c r="O49" t="inlineStr">
         <is>
           <t>AoE</t>
         </is>

</xml_diff>

<commit_message>
Add CAiSE 2026 - 130 total
</commit_message>
<xml_diff>
--- a/timeline_data.xlsx
+++ b/timeline_data.xlsx
@@ -786,7 +786,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O47"/>
+  <dimension ref="A1:O48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3664,6 +3664,54 @@
         </is>
       </c>
       <c r="O47" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>caise</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>CAiSE</t>
+        </is>
+      </c>
+      <c r="C48" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D48" t="n">
+        <v>1</v>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>2025-11-28</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>2026-02-01</t>
+        </is>
+      </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="L48" t="inlineStr">
+        <is>
+          <t>2026-06-12</t>
+        </is>
+      </c>
+      <c r="M48" t="inlineStr">
+        <is>
+          <t>Verona, Italy</t>
+        </is>
+      </c>
+      <c r="O48" t="inlineStr">
         <is>
           <t>AoE</t>
         </is>

</xml_diff>

<commit_message>
Add ICWS 2026 + ICSOC 2026 - 135 total
</commit_message>
<xml_diff>
--- a/timeline_data.xlsx
+++ b/timeline_data.xlsx
@@ -3728,7 +3728,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P52"/>
+  <dimension ref="A1:P54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6861,6 +6861,102 @@
         </is>
       </c>
       <c r="O52" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>icws</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>ICWS</t>
+        </is>
+      </c>
+      <c r="C53" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D53" t="n">
+        <v>1</v>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>2026-03-22</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="L53" t="inlineStr">
+        <is>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="M53" t="inlineStr">
+        <is>
+          <t>Sydney, Australia</t>
+        </is>
+      </c>
+      <c r="O53" t="inlineStr">
+        <is>
+          <t>AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>icsoc</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>ICSOC</t>
+        </is>
+      </c>
+      <c r="C54" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D54" t="n">
+        <v>1</v>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>2026-07-19</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t>2026-12-01</t>
+        </is>
+      </c>
+      <c r="L54" t="inlineStr">
+        <is>
+          <t>2026-12-04</t>
+        </is>
+      </c>
+      <c r="M54" t="inlineStr">
+        <is>
+          <t>Lodz, Poland</t>
+        </is>
+      </c>
+      <c r="O54" t="inlineStr">
         <is>
           <t>AoE</t>
         </is>

</xml_diff>